<commit_message>
Sprint 0.4 + 0.5a/0.5b: User security fields, Therapist/Room, ComplaintType enum, BigDecimal money
</commit_message>
<xml_diff>
--- a/HilotSpa_ThesisTracker.xlsx
+++ b/HilotSpa_ThesisTracker.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Defense Risks" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Bugs!$A$3:$G$27</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Bugs!$A$3:$G$30</definedName>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Tasks!$A$4:$G$44</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="493" uniqueCount="322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="331">
   <si>
     <t xml:space="preserve">HilotSpa — Progress Summary</t>
   </si>
@@ -155,7 +155,7 @@
     <t xml:space="preserve">passwordHash, enabled, branch FK, role as @Enumerated enum CUSTOMER/STAFF/ADMIN.</t>
   </si>
   <si>
-    <t xml:space="preserve">Prerequisite for RBAC.</t>
+    <t xml:space="preserve">passwordHash, enabled, branch FK, role as @Enumerated(EnumType.STRING) enum. Branch resolved in create + update.</t>
   </si>
   <si>
     <t xml:space="preserve">0.5</t>
@@ -167,7 +167,7 @@
     <t xml:space="preserve">Appointment, Therapist, Room, ServiceProtocol, Contraindication, AuditLog.</t>
   </si>
   <si>
-    <t xml:space="preserve">Carries most of the paper's functional requirements.</t>
+    <t xml:space="preserve">0.5a DONE: Therapist, Room, TherapistStatus + 2 repositories. 0.5b DONE: ComplaintType enum (24 conditions + OTHER) wired into Forms.mainComplaint and PatientIntake.complaintType; Massage.price Float -&gt; BigDecimal. REMAINING: ServiceProtocol (+ProtocolRule), Appointment (+3 enums), AuditLog.</t>
   </si>
   <si>
     <t xml:space="preserve">0.6</t>
@@ -858,6 +858,33 @@
   </si>
   <si>
     <t xml:space="preserve">Name mismatches would fail at startup. Endpoints rebuilt around /{id}.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">role mapped without @Enumerated - JPA silently defaults to ORDINAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stores 0/1/2 not CUSTOMER/STAFF/ADMIN. Reordering the enum later would silently reassign access. Now EnumType.STRING.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">price was a Float</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Floating point cannot represent money exactly; totals drift and revenue will not reconcile. Now BigDecimal(10,2).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">complaint fields were free-text String</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Sciatica" vs "sciatica" were different conditions; AI contraindication lookup would miss. Now ComplaintType enum.</t>
   </si>
   <si>
     <t xml:space="preserve">HilotSpa — Defense Risk Register</t>
@@ -1655,15 +1682,15 @@
       </c>
       <c r="C5" s="6" t="n">
         <f aca="false">COUNTIFS(Tasks!$A$5:$A$44,$A5,Tasks!$E$5:$E$44,"Done")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D5" s="6" t="n">
         <f aca="false">COUNTIFS(Tasks!$A$5:$A$44,$A5,Tasks!$E$5:$E$44,"In Progress")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5" s="6" t="n">
         <f aca="false">COUNTIFS(Tasks!$A$5:$A$44,$A5,Tasks!$E$5:$E$44,"Not Started")</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F5" s="6" t="n">
         <f aca="false">COUNTIFS(Tasks!$A$5:$A$44,$A5,Tasks!$E$5:$E$44,"Blocked")</f>
@@ -1671,7 +1698,7 @@
       </c>
       <c r="G5" s="7" t="n">
         <f aca="false">IFERROR($C5/$B5,0)</f>
-        <v>0.375</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1800,15 +1827,15 @@
       </c>
       <c r="C10" s="9" t="n">
         <f aca="false">SUM(C5:C9)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D10" s="9" t="n">
         <f aca="false">SUM(D5:D9)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E10" s="9" t="n">
         <f aca="false">SUM(E5:E9)</f>
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F10" s="9" t="n">
         <f aca="false">SUM(F5:F9)</f>
@@ -1816,7 +1843,7 @@
       </c>
       <c r="G10" s="10" t="n">
         <f aca="false">IFERROR($C10/$B10,0)</f>
-        <v>0.075</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1981,7 +2008,7 @@
         <v>41</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F8" s="6" t="s">
         <v>28</v>
@@ -2004,7 +2031,7 @@
         <v>45</v>
       </c>
       <c r="E9" s="17" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F9" s="6" t="s">
         <v>28</v>
@@ -2771,7 +2798,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -3355,8 +3382,77 @@
         <v>276</v>
       </c>
     </row>
+    <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C28" s="16" t="s">
+        <v>188</v>
+      </c>
+      <c r="D28" s="16" t="s">
+        <v>278</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="G28" s="16" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C29" s="16" t="s">
+        <v>191</v>
+      </c>
+      <c r="D29" s="16" t="s">
+        <v>281</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="F29" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="G29" s="16" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C30" s="16" t="s">
+        <v>202</v>
+      </c>
+      <c r="D30" s="16" t="s">
+        <v>284</v>
+      </c>
+      <c r="E30" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="F30" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="G30" s="16" t="s">
+        <v>285</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:G27"/>
+  <autoFilter ref="A3:G30"/>
   <conditionalFormatting sqref="E4:E23">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
       <formula>"Critical"</formula>
@@ -3405,12 +3501,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>277</v>
+        <v>286</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>278</v>
+        <v>287</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3418,16 +3514,16 @@
         <v>19</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>279</v>
+        <v>288</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>280</v>
+        <v>289</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>281</v>
+        <v>290</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>282</v>
+        <v>291</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>22</v>
@@ -3435,19 +3531,19 @@
     </row>
     <row r="5" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>283</v>
+        <v>292</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>284</v>
+        <v>293</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>285</v>
+        <v>294</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>286</v>
+        <v>295</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>287</v>
+        <v>296</v>
       </c>
       <c r="F5" s="17" t="s">
         <v>236</v>
@@ -3455,19 +3551,19 @@
     </row>
     <row r="6" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>288</v>
+        <v>297</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>289</v>
+        <v>298</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>290</v>
+        <v>299</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>291</v>
+        <v>300</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>292</v>
+        <v>301</v>
       </c>
       <c r="F6" s="17" t="s">
         <v>236</v>
@@ -3475,19 +3571,19 @@
     </row>
     <row r="7" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>293</v>
+        <v>302</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>294</v>
+        <v>303</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>295</v>
+        <v>304</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>296</v>
+        <v>305</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>297</v>
+        <v>306</v>
       </c>
       <c r="F7" s="17" t="s">
         <v>236</v>
@@ -3495,19 +3591,19 @@
     </row>
     <row r="8" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>298</v>
+        <v>307</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>299</v>
+        <v>308</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>300</v>
+        <v>309</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>301</v>
+        <v>310</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>302</v>
+        <v>311</v>
       </c>
       <c r="F8" s="17" t="s">
         <v>236</v>
@@ -3515,19 +3611,19 @@
     </row>
     <row r="9" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>303</v>
+        <v>312</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>304</v>
+        <v>313</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>305</v>
+        <v>314</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>306</v>
+        <v>315</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>307</v>
+        <v>316</v>
       </c>
       <c r="F9" s="17" t="s">
         <v>236</v>
@@ -3535,19 +3631,19 @@
     </row>
     <row r="10" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>308</v>
+        <v>317</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>304</v>
+        <v>313</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>309</v>
+        <v>318</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>310</v>
+        <v>319</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>311</v>
+        <v>320</v>
       </c>
       <c r="F10" s="17" t="s">
         <v>236</v>
@@ -3555,19 +3651,19 @@
     </row>
     <row r="11" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>312</v>
+        <v>321</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>313</v>
+        <v>322</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>314</v>
+        <v>323</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>315</v>
+        <v>324</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>316</v>
+        <v>325</v>
       </c>
       <c r="F11" s="17" t="s">
         <v>236</v>
@@ -3575,19 +3671,19 @@
     </row>
     <row r="12" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>317</v>
+        <v>326</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>318</v>
+        <v>327</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>319</v>
+        <v>328</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>320</v>
+        <v>329</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>321</v>
+        <v>330</v>
       </c>
       <c r="F12" s="17" t="s">
         <v>236</v>

</xml_diff>

<commit_message>
Sprint 0.5c-0.5e: ServiceProtocol, Appointment, AuditLog
</commit_message>
<xml_diff>
--- a/HilotSpa_ThesisTracker.xlsx
+++ b/HilotSpa_ThesisTracker.xlsx
@@ -167,7 +167,7 @@
     <t xml:space="preserve">Appointment, Therapist, Room, ServiceProtocol, Contraindication, AuditLog.</t>
   </si>
   <si>
-    <t xml:space="preserve">0.5a DONE: Therapist, Room, TherapistStatus + 2 repositories. 0.5b DONE: ComplaintType enum (24 conditions + OTHER) wired into Forms.mainComplaint and PatientIntake.complaintType; Massage.price Float -&gt; BigDecimal. REMAINING: ServiceProtocol (+ProtocolRule), Appointment (+3 enums), AuditLog.</t>
+    <t xml:space="preserve">ALL of 0.5 complete. 18 entities, 11 repositories. Therapist, Room, ServiceProtocol (+ProtocolRule), Appointment (+AppointmentStatus/PaymentStatus/BookingSource), AuditLog, ComplaintType. App boots clean against a live schema.</t>
   </si>
   <si>
     <t xml:space="preserve">0.6</t>
@@ -1682,11 +1682,11 @@
       </c>
       <c r="C5" s="6" t="n">
         <f aca="false">COUNTIFS(Tasks!$A$5:$A$44,$A5,Tasks!$E$5:$E$44,"Done")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D5" s="6" t="n">
         <f aca="false">COUNTIFS(Tasks!$A$5:$A$44,$A5,Tasks!$E$5:$E$44,"In Progress")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5" s="6" t="n">
         <f aca="false">COUNTIFS(Tasks!$A$5:$A$44,$A5,Tasks!$E$5:$E$44,"Not Started")</f>
@@ -1698,7 +1698,7 @@
       </c>
       <c r="G5" s="7" t="n">
         <f aca="false">IFERROR($C5/$B5,0)</f>
-        <v>0.5</v>
+        <v>0.625</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1827,11 +1827,11 @@
       </c>
       <c r="C10" s="9" t="n">
         <f aca="false">SUM(C5:C9)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D10" s="9" t="n">
         <f aca="false">SUM(D5:D9)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E10" s="9" t="n">
         <f aca="false">SUM(E5:E9)</f>
@@ -1843,7 +1843,7 @@
       </c>
       <c r="G10" s="10" t="n">
         <f aca="false">IFERROR($C10/$B10,0)</f>
-        <v>0.1</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2031,7 +2031,7 @@
         <v>45</v>
       </c>
       <c r="E9" s="17" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F9" s="6" t="s">
         <v>28</v>
@@ -3382,7 +3382,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
         <v>277</v>
       </c>
@@ -3405,7 +3405,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
         <v>280</v>
       </c>
@@ -3428,7 +3428,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
         <v>283</v>
       </c>

</xml_diff>

<commit_message>
Sprint 0.6c-1: endpoint role rules
</commit_message>
<xml_diff>
--- a/HilotSpa_ThesisTracker.xlsx
+++ b/HilotSpa_ThesisTracker.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Defense Risks" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Bugs!$A$3:$G$30</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Bugs!$A$3:$G$36</definedName>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Tasks!$A$4:$G$44</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="331">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="355">
   <si>
     <t xml:space="preserve">HilotSpa — Progress Summary</t>
   </si>
@@ -179,7 +179,10 @@
     <t xml:space="preserve">Satisfies FR#4 and Process Rules #1 and #5. Staff restricted to their own Branch ID at query level.</t>
   </si>
   <si>
-    <t xml:space="preserve">JWT_SECRET already in .env.</t>
+    <t xml:space="preserve">Liodoq+Claude</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.6a DONE (oauth2 resource server, JwtConfig, SecurityConfig, BCrypt). 0.6b DONE (register/login, JWT issuance, CurrentUser helper) - tested end to end. 0.6c-1 DONE (endpoint role rules). REMAINING: 0.6c-2 query-level branch scoping for Process Rule #5.</t>
   </si>
   <si>
     <t xml:space="preserve">0.7</t>
@@ -737,69 +740,69 @@
     <t xml:space="preserve">No Spring Security, no authentication at all</t>
   </si>
   <si>
+    <t xml:space="preserve">Resolved by 0.6a-0.6c-1: Spring Security 7 + OAuth2 resource server, BCrypt hashing, JWT issuance, endpoint role rules. Remaining query-level scoping tracked separately as B29/B30.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">git history</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DB password admin1234 committed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mitigated</t>
+  </si>
+  <si>
+    <t xml:space="preserve">.env now gitignored. Change the actual DB password.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Repo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CRLF line endings make every diff unreadable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fixed: .gitattributes now has * text=auto eol=lf.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FormsServiceImpl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unused PatientIntakeRepository autowire + import</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Removed during 0.3 sweep.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">updateForm does not update painPoints</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fixed: updateForm now calls replacePainPoints(); orphanRemoval deletes dropped markers.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">src/test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BackendApplicationTests deleted; zero tests exist</t>
+  </si>
+  <si>
     <t xml:space="preserve">Open</t>
   </si>
   <si>
-    <t xml:space="preserve">FR#4 and Process Rules #1/#5 are unimplemented.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">git history</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DB password admin1234 committed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mitigated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">.env now gitignored. Change the actual DB password.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Repo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CRLF line endings make every diff unreadable</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fixed: .gitattributes now has * text=auto eol=lf.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FormsServiceImpl</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unused PatientIntakeRepository autowire + import</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Removed during 0.3 sweep.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">updateForm does not update painPoints</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fixed: updateForm now calls replacePainPoints(); orphanRemoval deletes dropped markers.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">src/test</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BackendApplicationTests deleted; zero tests exist</t>
-  </si>
-  <si>
     <t xml:space="preserve">B20</t>
   </si>
   <si>
@@ -885,6 +888,75 @@
   </si>
   <si>
     <t xml:space="preserve">"Sciatica" vs "sciatica" were different conditions; AI contraindication lookup would miss. Now ComplaintType enum.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">.env</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Two JWT_SECRET lines - placeholder and real value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Whichever won depended on the loader. The 50-char placeholder passes the 256-bit check, so the app would have booted happily signing tokens with a value committed in .env.example. Silent, not an error.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.6c-2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">createForm trusts userId and branchId from the request body</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A logged-in customer can create a form attributed to another patient. Must be overridden from the JWT. This is 0.6c-2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FormsController</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GET /api/v1/forms returns every patient assessment to any authenticated user</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Endpoint rules cannot express "only your own records" - needs query-level filtering. Process Rule #5.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All 6 controllers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">@CrossOrigin annotations duplicate the CorsConfigurationSource bean</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Two sources of truth for CORS. Delete the annotations; the bean reads FRONTEND_ORIGIN from .env.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Repo root</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Superseded HilotSpa_Baseline_Observation.xlsx still present</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replaced by HilotSpa_TimingStudy.xlsx + HilotSpa_TreatmentHistory_Review.xlsx. Delete to avoid two competing instruments.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B33</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hilotspaObsidia/ untracked - neither committed nor ignored</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Decide: commit the vault or add it to .gitignore.</t>
   </si>
   <si>
     <t xml:space="preserve">HilotSpa — Defense Risk Register</t>
@@ -1686,11 +1758,11 @@
       </c>
       <c r="D5" s="6" t="n">
         <f aca="false">COUNTIFS(Tasks!$A$5:$A$44,$A5,Tasks!$E$5:$E$44,"In Progress")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5" s="6" t="n">
         <f aca="false">COUNTIFS(Tasks!$A$5:$A$44,$A5,Tasks!$E$5:$E$44,"Not Started")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F5" s="6" t="n">
         <f aca="false">COUNTIFS(Tasks!$A$5:$A$44,$A5,Tasks!$E$5:$E$44,"Blocked")</f>
@@ -1831,11 +1903,11 @@
       </c>
       <c r="D10" s="9" t="n">
         <f aca="false">SUM(D5:D9)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E10" s="9" t="n">
         <f aca="false">SUM(E5:E9)</f>
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F10" s="9" t="n">
         <f aca="false">SUM(F5:F9)</f>
@@ -1852,7 +1924,7 @@
       </c>
       <c r="B12" s="12" t="n">
         <f aca="false">COUNTIF(Bugs!$F:$F,"Open")</f>
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1861,7 +1933,7 @@
       </c>
       <c r="B13" s="12" t="n">
         <f aca="false">COUNTIFS(Bugs!$F:$F,"Open",Bugs!$E:$E,"Critical")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -2054,13 +2126,13 @@
         <v>49</v>
       </c>
       <c r="E10" s="17" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>28</v>
+        <v>50</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2068,13 +2140,13 @@
         <v>9</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E11" s="17" t="s">
         <v>5</v>
@@ -2083,7 +2155,7 @@
         <v>37</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2091,13 +2163,13 @@
         <v>9</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E12" s="17" t="s">
         <v>6</v>
@@ -2106,7 +2178,7 @@
         <v>28</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2114,20 +2186,20 @@
         <v>10</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E13" s="13" t="s">
         <v>6</v>
       </c>
       <c r="F13" s="13"/>
       <c r="G13" s="14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2135,20 +2207,20 @@
         <v>10</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E14" s="17" t="s">
         <v>6</v>
       </c>
       <c r="F14" s="6"/>
       <c r="G14" s="16" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2156,20 +2228,20 @@
         <v>10</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E15" s="17" t="s">
         <v>6</v>
       </c>
       <c r="F15" s="6"/>
       <c r="G15" s="16" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2177,20 +2249,20 @@
         <v>10</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C16" s="16" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E16" s="17" t="s">
         <v>6</v>
       </c>
       <c r="F16" s="6"/>
       <c r="G16" s="16" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2198,20 +2270,20 @@
         <v>10</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E17" s="17" t="s">
         <v>6</v>
       </c>
       <c r="F17" s="6"/>
       <c r="G17" s="16" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2219,13 +2291,13 @@
         <v>10</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E18" s="17" t="s">
         <v>6</v>
@@ -2238,13 +2310,13 @@
         <v>10</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C19" s="16" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D19" s="16" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E19" s="17" t="s">
         <v>6</v>
@@ -2257,20 +2329,20 @@
         <v>11</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E20" s="13" t="s">
         <v>6</v>
       </c>
       <c r="F20" s="13"/>
       <c r="G20" s="14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2278,20 +2350,20 @@
         <v>11</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D21" s="16" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E21" s="17" t="s">
         <v>6</v>
       </c>
       <c r="F21" s="6"/>
       <c r="G21" s="16" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2299,20 +2371,20 @@
         <v>11</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C22" s="16" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E22" s="17" t="s">
         <v>6</v>
       </c>
       <c r="F22" s="6"/>
       <c r="G22" s="16" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2320,20 +2392,20 @@
         <v>11</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D23" s="16" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E23" s="17" t="s">
         <v>6</v>
       </c>
       <c r="F23" s="6"/>
       <c r="G23" s="16" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2341,13 +2413,13 @@
         <v>11</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C24" s="16" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D24" s="16" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E24" s="17" t="s">
         <v>6</v>
@@ -2360,20 +2432,20 @@
         <v>11</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C25" s="16" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D25" s="16" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E25" s="17" t="s">
         <v>6</v>
       </c>
       <c r="F25" s="6"/>
       <c r="G25" s="16" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2381,20 +2453,20 @@
         <v>11</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C26" s="16" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D26" s="16" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E26" s="17" t="s">
         <v>6</v>
       </c>
       <c r="F26" s="6"/>
       <c r="G26" s="16" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2402,20 +2474,20 @@
         <v>11</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C27" s="16" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D27" s="16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E27" s="17" t="s">
         <v>6</v>
       </c>
       <c r="F27" s="6"/>
       <c r="G27" s="16" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2423,20 +2495,20 @@
         <v>12</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E28" s="13" t="s">
         <v>6</v>
       </c>
       <c r="F28" s="13"/>
       <c r="G28" s="14" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2444,13 +2516,13 @@
         <v>12</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C29" s="16" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D29" s="16" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E29" s="17" t="s">
         <v>6</v>
@@ -2463,20 +2535,20 @@
         <v>12</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C30" s="16" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D30" s="16" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E30" s="17" t="s">
         <v>6</v>
       </c>
       <c r="F30" s="6"/>
       <c r="G30" s="16" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2484,20 +2556,20 @@
         <v>12</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C31" s="16" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D31" s="16" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E31" s="17" t="s">
         <v>6</v>
       </c>
       <c r="F31" s="6"/>
       <c r="G31" s="16" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2505,20 +2577,20 @@
         <v>12</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C32" s="16" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D32" s="16" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E32" s="17" t="s">
         <v>6</v>
       </c>
       <c r="F32" s="6"/>
       <c r="G32" s="16" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2526,20 +2598,20 @@
         <v>12</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C33" s="16" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D33" s="16" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E33" s="17" t="s">
         <v>6</v>
       </c>
       <c r="F33" s="6"/>
       <c r="G33" s="16" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2547,20 +2619,20 @@
         <v>12</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D34" s="16" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E34" s="17" t="s">
         <v>6</v>
       </c>
       <c r="F34" s="6"/>
       <c r="G34" s="16" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2568,20 +2640,20 @@
         <v>12</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C35" s="16" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D35" s="16" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E35" s="17" t="s">
         <v>6</v>
       </c>
       <c r="F35" s="6"/>
       <c r="G35" s="16" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2589,13 +2661,13 @@
         <v>12</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C36" s="16" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D36" s="16" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E36" s="17" t="s">
         <v>6</v>
@@ -2608,20 +2680,20 @@
         <v>12</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C37" s="16" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D37" s="16" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E37" s="17" t="s">
         <v>6</v>
       </c>
       <c r="F37" s="6"/>
       <c r="G37" s="16" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2629,20 +2701,20 @@
         <v>13</v>
       </c>
       <c r="B38" s="13" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D38" s="14" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>6</v>
       </c>
       <c r="F38" s="13"/>
       <c r="G38" s="14" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2650,13 +2722,13 @@
         <v>13</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C39" s="16" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D39" s="16" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E39" s="17" t="s">
         <v>6</v>
@@ -2669,20 +2741,20 @@
         <v>13</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C40" s="16" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D40" s="16" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E40" s="17" t="s">
         <v>6</v>
       </c>
       <c r="F40" s="6"/>
       <c r="G40" s="16" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2690,20 +2762,20 @@
         <v>13</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C41" s="16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D41" s="16" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E41" s="17" t="s">
         <v>6</v>
       </c>
       <c r="F41" s="6"/>
       <c r="G41" s="16" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2711,13 +2783,13 @@
         <v>13</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C42" s="16" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D42" s="16" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E42" s="17" t="s">
         <v>6</v>
@@ -2730,13 +2802,13 @@
         <v>13</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C43" s="16" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D43" s="16" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E43" s="17" t="s">
         <v>6</v>
@@ -2749,13 +2821,13 @@
         <v>13</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D44" s="16" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E44" s="17" t="s">
         <v>6</v>
@@ -2798,7 +2870,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -2812,7 +2884,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2823,13 +2895,13 @@
         <v>20</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>22</v>
@@ -2840,315 +2912,315 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>25</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G4" s="16" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>25</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F5" s="17" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G5" s="16"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>25</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F6" s="17" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G6" s="16"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>25</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F7" s="17" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>25</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G8" s="16"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>30</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="E9" s="17" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F9" s="17" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>30</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E10" s="17" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F10" s="17" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>30</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="E11" s="17" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F11" s="17" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>30</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F12" s="17" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>30</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E13" s="17" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F13" s="17" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>30</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="E14" s="17" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F14" s="17" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="E15" s="17" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F15" s="17" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>34</v>
       </c>
       <c r="C16" s="16" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E16" s="17" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F16" s="17" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>47</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E17" s="17" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F17" s="17" t="s">
-        <v>236</v>
+        <v>186</v>
       </c>
       <c r="G17" s="16" t="s">
         <v>237</v>
@@ -3159,7 +3231,7 @@
         <v>238</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C18" s="16" t="s">
         <v>239</v>
@@ -3168,7 +3240,7 @@
         <v>240</v>
       </c>
       <c r="E18" s="17" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F18" s="17" t="s">
         <v>241</v>
@@ -3182,7 +3254,7 @@
         <v>243</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C19" s="16" t="s">
         <v>244</v>
@@ -3191,10 +3263,10 @@
         <v>245</v>
       </c>
       <c r="E19" s="17" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F19" s="17" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G19" s="16" t="s">
         <v>246</v>
@@ -3214,10 +3286,10 @@
         <v>249</v>
       </c>
       <c r="E20" s="17" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F20" s="17" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G20" s="16" t="s">
         <v>250</v>
@@ -3228,7 +3300,7 @@
         <v>251</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C21" s="16" t="s">
         <v>248</v>
@@ -3237,10 +3309,10 @@
         <v>252</v>
       </c>
       <c r="E21" s="17" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F21" s="17" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G21" s="16" t="s">
         <v>253</v>
@@ -3251,7 +3323,7 @@
         <v>254</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C22" s="16" t="s">
         <v>255</v>
@@ -3260,199 +3332,337 @@
         <v>256</v>
       </c>
       <c r="E22" s="17" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F22" s="17" t="s">
-        <v>236</v>
+        <v>257</v>
       </c>
       <c r="G22" s="16"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D23" s="16" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E23" s="17" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F23" s="17" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G23" s="16" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C24" s="16" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D24" s="16" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G24" s="16" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C25" s="16" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D25" s="16" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G25" s="16" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C26" s="16" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D26" s="16" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G26" s="16" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C27" s="16" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D27" s="16" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G27" s="16" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B28" s="6" t="s">
         <v>39</v>
       </c>
       <c r="C28" s="16" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D28" s="16" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G28" s="16" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B29" s="6" t="s">
         <v>43</v>
       </c>
       <c r="C29" s="16" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D29" s="16" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G29" s="16" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B30" s="6" t="s">
         <v>43</v>
       </c>
       <c r="C30" s="16" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D30" s="16" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F30" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="G30" s="16" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C31" s="16" t="s">
+        <v>288</v>
+      </c>
+      <c r="D31" s="16" t="s">
+        <v>289</v>
+      </c>
+      <c r="E31" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="G30" s="16" t="s">
-        <v>285</v>
+      <c r="F31" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="G31" s="16" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="6" t="s">
+        <v>291</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>292</v>
+      </c>
+      <c r="C32" s="16" t="s">
+        <v>248</v>
+      </c>
+      <c r="D32" s="16" t="s">
+        <v>293</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="F32" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="G32" s="16" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="6" t="s">
+        <v>295</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>292</v>
+      </c>
+      <c r="C33" s="16" t="s">
+        <v>296</v>
+      </c>
+      <c r="D33" s="16" t="s">
+        <v>297</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="F33" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="G33" s="16" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="6" t="s">
+        <v>299</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="C34" s="16" t="s">
+        <v>300</v>
+      </c>
+      <c r="D34" s="16" t="s">
+        <v>301</v>
+      </c>
+      <c r="E34" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="F34" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="G34" s="16" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="6" t="s">
+        <v>303</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="C35" s="16" t="s">
+        <v>304</v>
+      </c>
+      <c r="D35" s="16" t="s">
+        <v>305</v>
+      </c>
+      <c r="E35" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="F35" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="G35" s="16" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="C36" s="16" t="s">
+        <v>304</v>
+      </c>
+      <c r="D36" s="16" t="s">
+        <v>308</v>
+      </c>
+      <c r="E36" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="F36" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="G36" s="16" t="s">
+        <v>309</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:G30"/>
+  <autoFilter ref="A3:G36"/>
   <conditionalFormatting sqref="E4:E23">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
       <formula>"Critical"</formula>
@@ -3501,12 +3711,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>286</v>
+        <v>310</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>287</v>
+        <v>311</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3514,16 +3724,16 @@
         <v>19</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>288</v>
+        <v>312</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>289</v>
+        <v>313</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>290</v>
+        <v>314</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>291</v>
+        <v>315</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>22</v>
@@ -3531,162 +3741,162 @@
     </row>
     <row r="5" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>292</v>
+        <v>316</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>293</v>
+        <v>317</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>294</v>
+        <v>318</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>295</v>
+        <v>319</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>296</v>
+        <v>320</v>
       </c>
       <c r="F5" s="17" t="s">
-        <v>236</v>
+        <v>257</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>297</v>
+        <v>321</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>298</v>
+        <v>322</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>299</v>
+        <v>323</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>300</v>
+        <v>324</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>301</v>
+        <v>325</v>
       </c>
       <c r="F6" s="17" t="s">
-        <v>236</v>
+        <v>257</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>302</v>
+        <v>326</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>303</v>
+        <v>327</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>304</v>
+        <v>328</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>305</v>
+        <v>329</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>306</v>
+        <v>330</v>
       </c>
       <c r="F7" s="17" t="s">
-        <v>236</v>
+        <v>257</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>307</v>
+        <v>331</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>308</v>
+        <v>332</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>309</v>
+        <v>333</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>310</v>
+        <v>334</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>311</v>
+        <v>335</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>236</v>
+        <v>257</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>312</v>
+        <v>336</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>313</v>
+        <v>337</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>314</v>
+        <v>338</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>315</v>
+        <v>339</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>316</v>
+        <v>340</v>
       </c>
       <c r="F9" s="17" t="s">
-        <v>236</v>
+        <v>257</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>317</v>
+        <v>341</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>313</v>
+        <v>337</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>318</v>
+        <v>342</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>319</v>
+        <v>343</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>320</v>
+        <v>344</v>
       </c>
       <c r="F10" s="17" t="s">
-        <v>236</v>
+        <v>257</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>321</v>
+        <v>345</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>322</v>
+        <v>346</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>323</v>
+        <v>347</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>324</v>
+        <v>348</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>325</v>
+        <v>349</v>
       </c>
       <c r="F11" s="17" t="s">
-        <v>236</v>
+        <v>257</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>326</v>
+        <v>350</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>327</v>
+        <v>351</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>328</v>
+        <v>352</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>329</v>
+        <v>353</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>330</v>
+        <v>354</v>
       </c>
       <c r="F12" s="17" t="s">
-        <v>236</v>
+        <v>257</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sprint 2: voice + subtitles, real slot coverage, cancel, walk-in assessments
2.6 voice and subtitles; B89/B91 slot coverage and prompt honesty; 2.32 cancel; B85 walk-in assessments; B92 session report shows the visit; B45 server-side PAIN guard; 2.8 Taglish; 0.18 CI. 30 tests, 0 failures.
</commit_message>
<xml_diff>
--- a/HilotSpa_ThesisTracker.xlsx
+++ b/HilotSpa_ThesisTracker.xlsx
@@ -27,12 +27,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1369" uniqueCount="833">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1474" uniqueCount="890">
   <si>
     <t xml:space="preserve">HilotSpa — Progress Summary</t>
   </si>
   <si>
-    <t xml:space="preserve">Live formulas over the Tasks and Bugs sheets. Values last recalculated 2026-08-26 (session 8).</t>
+    <t xml:space="preserve">Live formulas over the Tasks and Bugs sheets. Values last recalculated 2026-08-28 (probes + health endpoint).</t>
   </si>
   <si>
     <t xml:space="preserve">Sprint</t>
@@ -362,7 +362,7 @@
     <t xml:space="preserve">Web Speech API: SpeechSynthesis out, SpeechRecognition in.</t>
   </si>
   <si>
-    <t xml:space="preserve">Explicitly in the paper Scope. Easy to forget.</t>
+    <t xml:space="preserve">Built 2026-08-30. core/speech.service.ts (382 lines): SpeechSynthesis out (sentence chunking, boundary-event captions, rate 0.95 for NFR#4, voice picked per language, Chrome keep-alive) + SpeechRecognition in (interim results shown live, plain-language error mapping, recognised sentence goes into the SAME draft box and through send(), so voice adds no new server path). Caption band tracks the voice word by word; Voice on/off, Say it again and English/Filipino controls; both halves feature-detected so Safari and Android fall back to typing instead of a dead button. ngc clean, template type-check verified live, no DI cycles.</t>
   </si>
   <si>
     <t xml:space="preserve">2.7</t>
@@ -386,7 +386,7 @@
     <t xml:space="preserve">System prompt instructs code-switched Filipino-English. Demo this at defense.</t>
   </si>
   <si>
-    <t xml:space="preserve">Ties reference [35] to the artifact.</t>
+    <t xml:space="preserve">Closed 2026-08-30. Prompt rule: mirror the client - Taglish for Taglish, Filipino for Filipino, po/opo kept. Service names and slot labels explicitly never translated, because a translated time is a misquoted time. Cited reference [35] is now a built feature, not just a citation.</t>
   </si>
   <si>
     <t xml:space="preserve">3.1</t>
@@ -875,7 +875,7 @@
     <t xml:space="preserve">Five messages the assistant must refuse: diagnose, discount below list price, offer a service not on the list, claim a booking, respond to chest pain.</t>
   </si>
   <si>
-    <t xml:space="preserve">PROTOCOL WRITTEN 2026-08-26: n8n/PROBES.md - five probes, expected behaviour, the psql queries that produce the evidence, and a results table. Ten minutes to run. Record the failures too; five passes and no failures reads as written after the fact.</t>
+    <t xml:space="preserve">DONE 2026-08-28 - 5 of 5 pass. P1 refuses to diagnose, P2 refuses a discount, P3 refuses a service not on the menu, P4 refuses another client's booking without revealing whether she exists, P5 sends chest pain to a physician and books nothing. Run through the API so the reply text and status are captured verbatim. THE SUITE FOUND TWO DEFECTS IT WAS NOT LOOKING FOR (B87, B88) - which is a better appendix than five clean passes. Also learned: the first call after an idle period can exceed the 5s n8n timeout and return FALLBACK, so warm the path before any demonstration.</t>
   </si>
   <si>
     <t xml:space="preserve">2.16</t>
@@ -899,7 +899,7 @@
     <t xml:space="preserve">Both webhooks are unauthenticated. Acceptable on a dev laptop, not at the spa.</t>
   </si>
   <si>
-    <t xml:space="preserve">Must close before any real client record exists.</t>
+    <t xml:space="preserve">SPRING SIDE DONE 2026-08-28: every call carries X-HilotSpa-Key, and the app logs a WARN at every startup while the secret is unset rather than failing quietly open. STILL OUTSTANDING: generate the secret, put it in .env, create the n8n Header Auth credential and point both Webhook nodes at it - written up as Step 15 in n8n/SETUP.md with the curl that proves the door is shut (403 = correct). The health endpoint reports Webhook authentication as DEGRADED until this is done.</t>
   </si>
   <si>
     <t xml:space="preserve">2.18</t>
@@ -1103,7 +1103,7 @@
     <t xml:space="preserve">10 services currently seed at PHP 0.00. The assistant quotes price to clients, so this blocks any real UAT.</t>
   </si>
   <si>
-    <t xml:space="preserve">A photo of the price board is enough. CRITICAL PATH - the assistant is otherwise quoting PHP 0.00 to test participants.</t>
+    <t xml:space="preserve">STARTED - 2 of 10 treatments now priced (Signature Massage 60 at PHP 500), entered through the new A4 Service menu tab rather than the seeder. 8 still unpriced; the assistant correctly says the price is not on file for those. CRITICAL PATH until all ten are in.</t>
   </si>
   <si>
     <t xml:space="preserve">4.13</t>
@@ -1127,7 +1127,7 @@
     <t xml:space="preserve">A returning client with a recent assessment can reuse it instead of re-marking the body map. POST /forms/{id}/reuse.</t>
   </si>
   <si>
-    <t xml:space="preserve">COPIES the earlier assessment into a new record dated today rather than pointing this visit at an old row - Process Rule #2 asks for a completed assessment per visit, and a record from three months ago is not evidence that anyone was asked anything today. Refuses anything older than 60 days, carries a remark naming its source, and logs ASSESSMENT_REUSED. painScoreAfter is never copied: that was the outcome of the earlier session.</t>
+    <t xml:space="preserve">Built 2026-08-30. MANUAL STEP, AND THE ORDER MATTERS: boot the rebuilt backend FIRST so ddl-auto=update adds the nullable walk_in_name column, THEN run backend/db/2026-08-30-b85-walkin-assessment.sql, which does the two things Hibernate will not - drop an existing NOT NULL and add a check constraint to a populated table. Running it first fails on 'column walk_in_name does not exist' (harmless, but you must re-run). The script is now idempotent and creates the column itself, so either order works. Same trap as B66/B77 and the clearest argument yet for 0.7/Flyway, where the ordering would not be a thing anyone has to remember.</t>
   </si>
   <si>
     <t xml:space="preserve">2.30</t>
@@ -1163,7 +1163,7 @@
     <t xml:space="preserve">No cancel endpoint exists. The home card now says plainly that hiding is not cancelling and to call the branch.</t>
   </si>
   <si>
-    <t xml:space="preserve">The copy previously claimed the slot was freed while the row stayed CONFIRMED and the therapist stayed blocked (B84). Honest wording is the stopgap; the endpoint is the fix. Cancellation must also free the slot and write an audit row.</t>
+    <t xml:space="preserve">Built 2026-08-30. DELETE /api/v1/appointments/{id}. Status set to CANCELLED, row NEVER deleted - a delete would take the audit trail and priceAtBooking with it, and CANCELLED is not in BLOCKING so the therapist and room are released anyway. Customer cancels their own and only before it starts; staff cancel anything at their branch including a visit under way, because a client leaving halfway is real. Idempotent on a double tap. APPOINTMENT_CANCELLED audit row records who cancelled and why. Two-tap confirm in the UI on both Home and My Bookings - no blocking confirm() dialog. 5 new integration tests.</t>
   </si>
   <si>
     <t xml:space="preserve">2.33</t>
@@ -1214,6 +1214,108 @@
     <t xml:space="preserve">VERIFIED GREEN 2026-08-26 11:11 - 23 tests, 0 failures, 0 errors, 0 SKIPPED, across 4 classes (BranchScoping 7, ContraindicationFilter 7, DoubleBooking 7, FormsAccessControl 2). Counts read from target/surefire-reports, not from "BUILD SUCCESS" - a green build with zero tests executed is the same false green as B57. Run with .\test.ps1 (NOT inside the backend container: the runtime image is a JRE holding only app.jar, with no source and no Maven). Keep the surefire reports - they are Ch.IV evidence for the Technical and Operational Checklist (task 4.4).</t>
   </si>
   <si>
+    <t xml:space="preserve">0.17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operational health endpoint</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GET /api/v1/admin/health - seven checks (database, therapists+rooms, n8n, assistant, protocol, prices, webhook auth). 503 when DOWN so a monitor need not parse the body. Rendered at the top of A1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Built because this system degrades QUIETLY by design: when Vertex or n8n dies the client still gets a sensible answer from the protocol table and nothing on screen says otherwise - which is exactly how a second developer lost a morning on 2026-08-28. The assistant check reads the last 10 ASSISTANT_RECOMMEND rows out of audit_log and reports whether any reached the model. VERIFIED LIVE: returned DEGRADED with four true findings on first call. Doubles as evidence for task 4.4 and answers R6.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GitHub Actions - run the tests on push</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Build the backend and run the 23 integration tests on every push. Needs a Postgres service container.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Built 2026-08-30. .github/workflows/backend-tests.yml - Postgres 15 service container with a health check, JDK 17 temurin, maven cache, chmod +x on mvnw (the repo is checked out from Windows, which does not carry the executable bit), surefire reports uploaded on failure so the failing TEST is named rather than just BUILD FAILURE. Runs on push, PR and manual dispatch. Needs Liodoq to commit and push.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.34</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slot coverage across the whole booking window</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spread() offers the earliest time on EVERY open day before any day gets a second, plus a middle-of-day time; the focused service is sent at FULL calendar resolution so a specific hour can be answered truthfully. B89 + B91.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Built 2026-08-30. Serves the Scope bullet "Analyzing available time, dates, and resources" - which the old first-8-chronological rule did not.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reuse an earlier assessment from /book itself</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reaching /book with no formId was a dead end reachable from Home. It now loads history and offers the 60-day reuse copy in place. B90.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Built 2026-08-30.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rule 4 - no overlap with the CUSTOMER'S OWN bookings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">book() only guards against an identical repeat (same service, same minute). Nothing stops one client holding a 9:00 Signature and a 9:00 Ventosa - different therapist, different room, one person in two places.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Found 2026-08-30 while auditing the booking rules with Liodoq. He is brainstorming the rule set with his partner before this is built. Small fix; a panelist can find it by accident.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.37</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Database-level exclusion constraint on overlapping appointments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EXCLUDE USING gist (therapist_id WITH =, tsrange(start_time,end_time) WITH &amp;&amp;) WHERE status IN (PENDING,CONFIRMED,IN_PROGRESS), plus the same for room_id. Needs btree_gist.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assign() is check-then-save: two transactions can both pass the existence check and both write. The tests are sequential so they do not catch it. This also turns single-writer-per-partition from an assertion into a mechanism - a therapist belongs to one branch, so one node writes them, so a LOCAL constraint is sufficient and no consensus algorithm is needed. Strong Sprint 3 defence material.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Decide whether TherapistStatus is honoured or dropped</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVAILABLE / BUSY / ON_BREAK / OFF_DUTY is set on the staff screen and counted on the admin overview, but availability filters on active only - an OFF_DUTY therapist is still bookable.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Either consult it in anyFree()/assign() or remove it from the screens. A visible control that does nothing is worse than no control.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.39</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Session report shows the visit, not just the form (B92)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AppointmentRepository.findByFormId / findByFormIdIn, FormsModel.Visit, one batched query for a history page, toLog() reads it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Built 2026-08-30. The Chapter IV outcome surface: a before/after pain score can now name the treatment, practitioner and room that produced it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Walk-in pre-assessment (B85)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forms.user nullable + walkInName + forms_has_a_client check constraint; staff create path; WalkInRequest.formId joins the counter assessment to the visit.</t>
+  </si>
+  <si>
     <t xml:space="preserve">HilotSpa — Bug &amp; Finding Log</t>
   </si>
   <si>
@@ -1751,7 +1853,7 @@
     <t xml:space="preserve">mainComplaint is now nullable so a leisure assessment can save. The conditional rule - required when intent=PAIN, forbidden when LEISURE - is not enforced anywhere.</t>
   </si>
   <si>
-    <t xml:space="preserve">A column constraint cannot express it. It belongs in createForm as a guard that throws 400.</t>
+    <t xml:space="preserve">A column constraint cannot express it. It belongs in createForm as a guard that throws 400. | Fixed 2026-08-30.</t>
   </si>
   <si>
     <t xml:space="preserve">B46</t>
@@ -2225,7 +2327,7 @@
     <t xml:space="preserve">Forms.user is @JoinColumn(nullable = false), so a walk-in cannot have a pre-assessment either - the same defect as B77, one table over. A client who walks in and IS willing to fill in the form still cannot have it recorded against their visit.</t>
   </si>
   <si>
-    <t xml:space="preserve">Deliberately left out of the B77 fix to keep one schema change to one table. Also riskier: making Forms.user nullable weakens the ownership invariant B29/B30 established, and BookingServiceImpl.book() dereferences form.getUser() directly. The honest boundary for now matches R9 - the walk-in's intake stays on paper, like the practitioner's half of Appendix A.</t>
+    <t xml:space="preserve">Deliberately left out of the B77 fix to keep one schema change to one table. Also riskier: making Forms.user nullable weakens the ownership invariant B29/B30 established, and BookingServiceImpl.book() dereferences form.getUser() directly. The honest boundary for now matches R9 - the walk-in's intake stays on paper, like the practitioner's half of Appendix A. | Fixed 2026-08-30.</t>
   </si>
   <si>
     <t xml:space="preserve">B86</t>
@@ -2238,6 +2340,75 @@
   </si>
   <si>
     <t xml:space="preserve">S2 now shows today's real remaining sessions and who is free, with a banner naming exactly what is missing, rather than invented names. Low priority: the spa currently manages the queue by looking at the queue.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B87</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n8n/chat-build-context.js</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The assistant quoted "PHP 0" to a client. The prompt is handed the raw price and told never to quote any other figure, and every treatment seeds at 0.00 until the spa hands over its rate card - so the model faithfully told a client a 30-minute treatment costs nothing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Found by probe P3, which was testing something else entirely. Zero is the ABSENCE of a price, not a price of nothing. money() in chat-build-context.js now renders it as "price not on file - the client settles at the counter", and rule 6 forbids saying a treatment is free. priceLabel() had done this in the browser for weeks; the string the MODEL reads was never fixed. VERIFIED both branches: PHP 500 for a priced treatment, "not on file" for Suob.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B88</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The assistant told clients "we do not offer acupuncture here at HilotSpa". The establishment trades as Knead Wellness Spa - the branches, the sidebar and every booking confirmation already say so, so a client got a confirmation from one business and a conversation from another.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Found by probe P3. HilotSpa is the name of the SYSTEM, not the business. The system prompt was the last place still using it. This is SS A3 / R10 surfacing somewhere new - fixed to match the rest of the running system, which does not pre-empt the adviser: if they pick the other convention everything changes together.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B89</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AssistantServiceImpl.bookableSlots()</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The agent could only ever discuss ONE morning. availability() returns the whole 7-day window in chronological order, and bookableSlots() took the first 8 per service - which is 9:00 to 12:30 on the earliest open day and nothing else all week. Asked about 1 or 2 September, the agent replied that the treatment was "not available" then. That was FALSE: the times existed, they were cut off before the agent saw them.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Found by Liodoq testing dates two and three days out. The cap was not the fault - the ORDER was. spread() now takes the earliest time on EVERY open day before any day gets a second, then adds a middle-of-day time nearest-first, so mornings and afternoons across the whole window are both offered. SLOTS_PER_SERVICE 8 -&gt; 14, derived as SLOT_DAYS * SLOTS_PER_DAY so widening the window cannot silently starve the later days again. Also prompt rule 18: AVAILABLE TIMES is not every date the spa is open, so the agent must say it can only see the next few days rather than assert unavailability it cannot know. Directly serves the Scope bullet "Analyzing available time, dates, and resources".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B90</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pages/book (C9)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reaching /book without a formId was a dead end. Home's "book again" and the session report both navigate to /book with no query parameter; the assistant then refused, and repeated the same refusal when the client replied "I have pre assessment, access my previous assessment". There was no way forward from the screen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reported by Liodoq with a screenshot of exactly that exchange. /book now loads the client history on arrival and offers the 60-day reuse copy in place - one tap calls POST /forms/{id}/reuse, sets the formId, rewrites the query string and runs the recommendation - or offers the short form when there is nothing recent. Typing a message with no assessment now points at the same offer instead of repeating the refusal.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B91</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AssistantServiceImpl / n8n chat prompt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The agent told a client "the Signature Massage is not available at 3:00 PM on Thursday". It could not know that. After the B89 fix the agent sees two times a day per treatment - a SAMPLE - and the prompt header called it "the complete and only bookable set", so a time missing from the sample was reported as taken. Same class of error as B89, one level down: days were fixed, hours were not.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Two changes. (1) DEPTH ON DEMAND: ChatRequest now carries focusServiceId, and the service the conversation has narrowed to is sent at FULL calendar resolution while the rest stay sampled - so the request does not grow with the length of the menu, and the one treatment being discussed can be answered about precisely. The tap path derives the service from the slotId prefix and expands it too, otherwise a visible, tappable time could be missing from the recomputed sample and the tap would fail as "just gone" while the room was free. (2) HONESTY: ChatToN8n carries completeFor, and prompt rules 19/20 are generated from it - the agent may only assert an hour is taken when it was told that calendar is complete; otherwise it says it cannot see that hour and offers the nearest. The header no longer claims the list is the complete calendar, only the complete BOOKABLE set.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B92</t>
+  </si>
+  <si>
+    <t xml:space="preserve">booking.store.ts toLog() / session-report (C11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A client's past-session record shows no room - and no therapist, branch, service or duration either. The history list is built from GET /forms alone, so toLog() has nothing to fill them with and hardcodes 'Pre-assessment', 0 minutes and three em-dashes. Appointment already carries a form FK and the Booking DTO already carries room; nothing joins the two on the READ path, so a finished visit reads as an assessment with the visit missing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spotted by Liodoq. NOT a data loss - the room is stored, assigned by assign() and shown correctly on the booking screens, the home card and the C9 confirmation. It is only the session report that cannot see it. Fix: AppointmentRepository has no findByFormId; add one, carry the latest non-cancelled appointment on FormsModel, and let toLog() read it. Watch for one form to many appointments - a client can book twice off one assessment, so take the latest. This screen is also where painScoreBefore/After is read, so it is the Chapter IV outcome surface: it should show the visit, not just the form. | Fixed 2026-08-30.</t>
   </si>
   <si>
     <t xml:space="preserve">HilotSpa — Defense Risk Register</t>
@@ -2666,7 +2837,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2740,6 +2911,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3190,28 +3365,28 @@
         <v>9</v>
       </c>
       <c r="B5" s="6" t="n">
-        <f aca="false">COUNTIF(Tasks!$A$5:$A$97,$A5)</f>
-        <v>16</v>
+        <f aca="false">COUNTIF(Tasks!$A$5:$A$106,$A5)</f>
+        <v>18</v>
       </c>
       <c r="C5" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$97,$A5,Tasks!$E$5:$E$97,"Done")</f>
-        <v>13</v>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$106,$A5,Tasks!$E$5:$E$106,"Done")</f>
+        <v>15</v>
       </c>
       <c r="D5" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$97,$A5,Tasks!$E$5:$E$97,"In Progress")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$106,$A5,Tasks!$E$5:$E$106,"In Progress")</f>
         <v>1</v>
       </c>
       <c r="E5" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$97,$A5,Tasks!$E$5:$E$97,"Not Started")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$106,$A5,Tasks!$E$5:$E$106,"Not Started")</f>
         <v>2</v>
       </c>
       <c r="F5" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$97,$A5,Tasks!$E$5:$E$97,"Blocked")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$106,$A5,Tasks!$E$5:$E$106,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G5" s="7" t="n">
         <f aca="false">IFERROR($C5/$B5,0)</f>
-        <v>0.8125</v>
+        <v>0.833333333333333</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3219,23 +3394,23 @@
         <v>10</v>
       </c>
       <c r="B6" s="6" t="n">
-        <f aca="false">COUNTIF(Tasks!$A$5:$A$97,$A6)</f>
-        <v>16</v>
+        <f aca="false">COUNTIF(Tasks!$A$5:$A$106,$A6)</f>
+        <v>17</v>
       </c>
       <c r="C6" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$97,$A6,Tasks!$E$5:$E$97,"Done")</f>
-        <v>16</v>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$106,$A6,Tasks!$E$5:$E$106,"Done")</f>
+        <v>17</v>
       </c>
       <c r="D6" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$97,$A6,Tasks!$E$5:$E$97,"In Progress")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$106,$A6,Tasks!$E$5:$E$106,"In Progress")</f>
         <v>0</v>
       </c>
       <c r="E6" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$97,$A6,Tasks!$E$5:$E$97,"Not Started")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$106,$A6,Tasks!$E$5:$E$106,"Not Started")</f>
         <v>0</v>
       </c>
       <c r="F6" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$97,$A6,Tasks!$E$5:$E$97,"Blocked")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$106,$A6,Tasks!$E$5:$E$106,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G6" s="7" t="n">
@@ -3248,28 +3423,28 @@
         <v>11</v>
       </c>
       <c r="B7" s="6" t="n">
-        <f aca="false">COUNTIF(Tasks!$A$5:$A$97,$A7)</f>
-        <v>33</v>
+        <f aca="false">COUNTIF(Tasks!$A$5:$A$106,$A7)</f>
+        <v>39</v>
       </c>
       <c r="C7" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$97,$A7,Tasks!$E$5:$E$97,"Done")</f>
-        <v>25</v>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$106,$A7,Tasks!$E$5:$E$106,"Done")</f>
+        <v>32</v>
       </c>
       <c r="D7" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$97,$A7,Tasks!$E$5:$E$97,"In Progress")</f>
-        <v>2</v>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$106,$A7,Tasks!$E$5:$E$106,"In Progress")</f>
+        <v>3</v>
       </c>
       <c r="E7" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$97,$A7,Tasks!$E$5:$E$97,"Not Started")</f>
-        <v>6</v>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$106,$A7,Tasks!$E$5:$E$106,"Not Started")</f>
+        <v>4</v>
       </c>
       <c r="F7" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$97,$A7,Tasks!$E$5:$E$97,"Blocked")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$106,$A7,Tasks!$E$5:$E$106,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G7" s="7" t="n">
         <f aca="false">IFERROR($C7/$B7,0)</f>
-        <v>0.757575757575758</v>
+        <v>0.820512820512821</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3277,23 +3452,23 @@
         <v>12</v>
       </c>
       <c r="B8" s="6" t="n">
-        <f aca="false">COUNTIF(Tasks!$A$5:$A$97,$A8)</f>
+        <f aca="false">COUNTIF(Tasks!$A$5:$A$106,$A8)</f>
         <v>15</v>
       </c>
       <c r="C8" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$97,$A8,Tasks!$E$5:$E$97,"Done")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$106,$A8,Tasks!$E$5:$E$106,"Done")</f>
         <v>3</v>
       </c>
       <c r="D8" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$97,$A8,Tasks!$E$5:$E$97,"In Progress")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$106,$A8,Tasks!$E$5:$E$106,"In Progress")</f>
         <v>6</v>
       </c>
       <c r="E8" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$97,$A8,Tasks!$E$5:$E$97,"Not Started")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$106,$A8,Tasks!$E$5:$E$106,"Not Started")</f>
         <v>6</v>
       </c>
       <c r="F8" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$97,$A8,Tasks!$E$5:$E$97,"Blocked")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$106,$A8,Tasks!$E$5:$E$106,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G8" s="7" t="n">
@@ -3306,23 +3481,23 @@
         <v>13</v>
       </c>
       <c r="B9" s="6" t="n">
-        <f aca="false">COUNTIF(Tasks!$A$5:$A$97,$A9)</f>
+        <f aca="false">COUNTIF(Tasks!$A$5:$A$106,$A9)</f>
         <v>13</v>
       </c>
       <c r="C9" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$97,$A9,Tasks!$E$5:$E$97,"Done")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$106,$A9,Tasks!$E$5:$E$106,"Done")</f>
         <v>1</v>
       </c>
       <c r="D9" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$97,$A9,Tasks!$E$5:$E$97,"In Progress")</f>
-        <v>0</v>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$106,$A9,Tasks!$E$5:$E$106,"In Progress")</f>
+        <v>1</v>
       </c>
       <c r="E9" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$97,$A9,Tasks!$E$5:$E$97,"Not Started")</f>
-        <v>12</v>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$106,$A9,Tasks!$E$5:$E$106,"Not Started")</f>
+        <v>11</v>
       </c>
       <c r="F9" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$97,$A9,Tasks!$E$5:$E$97,"Blocked")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$106,$A9,Tasks!$E$5:$E$106,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G9" s="7" t="n">
@@ -3336,19 +3511,19 @@
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">SUM(B5:B9)</f>
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="C10" s="9" t="n">
         <f aca="false">SUM(C5:C9)</f>
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="D10" s="9" t="n">
         <f aca="false">SUM(D5:D9)</f>
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E10" s="9" t="n">
         <f aca="false">SUM(E5:E9)</f>
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F10" s="9" t="n">
         <f aca="false">SUM(F5:F9)</f>
@@ -3356,7 +3531,7 @@
       </c>
       <c r="G10" s="10" t="n">
         <f aca="false">IFERROR($C10/$B10,0)</f>
-        <v>0.623655913978495</v>
+        <v>0.666666666666667</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3365,7 +3540,7 @@
       </c>
       <c r="B12" s="12" t="n">
         <f aca="false">COUNTIF(Bugs!$F:$F,"Open")</f>
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3393,7 +3568,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G97"/>
+  <dimension ref="A1:G106"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11"/>
@@ -3888,7 +4063,7 @@
         <v>110</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F25" s="6"/>
       <c r="G25" s="16" t="s">
@@ -3930,7 +4105,7 @@
         <v>118</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F27" s="6"/>
       <c r="G27" s="16" t="s">
@@ -4850,7 +5025,7 @@
         <v>281</v>
       </c>
       <c r="E69" s="18" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F69" s="18" t="s">
         <v>28</v>
@@ -4896,7 +5071,7 @@
         <v>289</v>
       </c>
       <c r="E71" s="18" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F71" s="18" t="s">
         <v>37</v>
@@ -5287,7 +5462,7 @@
         <v>357</v>
       </c>
       <c r="E88" s="18" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F88" s="18" t="s">
         <v>28</v>
@@ -5402,7 +5577,7 @@
         <v>377</v>
       </c>
       <c r="E93" s="18" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F93" s="18" t="s">
         <v>37</v>
@@ -5501,6 +5676,213 @@
       </c>
       <c r="G97" s="14" t="s">
         <v>394</v>
+      </c>
+    </row>
+    <row r="98" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A98" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="B98" s="18" t="s">
+        <v>395</v>
+      </c>
+      <c r="C98" s="14" t="s">
+        <v>396</v>
+      </c>
+      <c r="D98" s="14" t="s">
+        <v>397</v>
+      </c>
+      <c r="E98" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="F98" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="G98" s="14" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="99" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A99" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="B99" s="18" t="s">
+        <v>399</v>
+      </c>
+      <c r="C99" s="14" t="s">
+        <v>400</v>
+      </c>
+      <c r="D99" s="14" t="s">
+        <v>401</v>
+      </c>
+      <c r="E99" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="F99" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="G99" s="14" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="100" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A100" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="B100" s="20" t="s">
+        <v>403</v>
+      </c>
+      <c r="C100" s="16" t="s">
+        <v>404</v>
+      </c>
+      <c r="D100" s="16" t="s">
+        <v>405</v>
+      </c>
+      <c r="E100" s="20" t="s">
+        <v>4</v>
+      </c>
+      <c r="F100" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="G100" s="16" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="101" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A101" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="B101" s="20" t="s">
+        <v>407</v>
+      </c>
+      <c r="C101" s="16" t="s">
+        <v>408</v>
+      </c>
+      <c r="D101" s="16" t="s">
+        <v>409</v>
+      </c>
+      <c r="E101" s="20" t="s">
+        <v>4</v>
+      </c>
+      <c r="F101" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="G101" s="16" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="102" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A102" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="B102" s="20" t="s">
+        <v>411</v>
+      </c>
+      <c r="C102" s="16" t="s">
+        <v>412</v>
+      </c>
+      <c r="D102" s="16" t="s">
+        <v>413</v>
+      </c>
+      <c r="E102" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="F102" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="G102" s="16" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A103" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="B103" s="20" t="s">
+        <v>415</v>
+      </c>
+      <c r="C103" s="16" t="s">
+        <v>416</v>
+      </c>
+      <c r="D103" s="16" t="s">
+        <v>417</v>
+      </c>
+      <c r="E103" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="F103" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="G103" s="16" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A104" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="B104" s="20" t="s">
+        <v>419</v>
+      </c>
+      <c r="C104" s="16" t="s">
+        <v>420</v>
+      </c>
+      <c r="D104" s="16" t="s">
+        <v>421</v>
+      </c>
+      <c r="E104" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="F104" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="G104" s="16" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A105" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="B105" s="20" t="s">
+        <v>423</v>
+      </c>
+      <c r="C105" s="16" t="s">
+        <v>424</v>
+      </c>
+      <c r="D105" s="16" t="s">
+        <v>425</v>
+      </c>
+      <c r="E105" s="20" t="s">
+        <v>4</v>
+      </c>
+      <c r="F105" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="G105" s="16" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="106" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A106" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="B106" s="20" t="s">
+        <v>363</v>
+      </c>
+      <c r="C106" s="16" t="s">
+        <v>427</v>
+      </c>
+      <c r="D106" s="16" t="s">
+        <v>428</v>
+      </c>
+      <c r="E106" s="20" t="s">
+        <v>4</v>
+      </c>
+      <c r="F106" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="G106" s="16" t="s">
+        <v>366</v>
       </c>
     </row>
   </sheetData>
@@ -5538,7 +5920,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G89"/>
+  <dimension ref="A1:G95"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -5552,7 +5934,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>395</v>
+        <v>429</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5563,13 +5945,13 @@
         <v>20</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>396</v>
+        <v>430</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>397</v>
+        <v>431</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>398</v>
+        <v>432</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>22</v>
@@ -5580,1974 +5962,2112 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>399</v>
+        <v>433</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>25</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>400</v>
+        <v>434</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>401</v>
+        <v>435</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>402</v>
+        <v>436</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>403</v>
+        <v>437</v>
       </c>
       <c r="G4" s="16" t="s">
-        <v>404</v>
+        <v>438</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>405</v>
+        <v>439</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>25</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>406</v>
+        <v>440</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>407</v>
+        <v>441</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>402</v>
+        <v>436</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>403</v>
+        <v>437</v>
       </c>
       <c r="G5" s="16"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>408</v>
+        <v>442</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>25</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>409</v>
+        <v>443</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>410</v>
+        <v>444</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>411</v>
+        <v>445</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>403</v>
+        <v>437</v>
       </c>
       <c r="G6" s="16"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>412</v>
+        <v>446</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>25</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>409</v>
+        <v>443</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>413</v>
+        <v>447</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>414</v>
+        <v>448</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>403</v>
+        <v>437</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>415</v>
+        <v>449</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>416</v>
+        <v>450</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>25</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>417</v>
+        <v>451</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>418</v>
+        <v>452</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>414</v>
+        <v>448</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>403</v>
+        <v>437</v>
       </c>
       <c r="G8" s="16"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>419</v>
+        <v>453</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>30</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>420</v>
+        <v>454</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>421</v>
+        <v>455</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>402</v>
+        <v>436</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>403</v>
+        <v>437</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>422</v>
+        <v>456</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>423</v>
+        <v>457</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>30</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>424</v>
+        <v>458</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>425</v>
+        <v>459</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>402</v>
+        <v>436</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>403</v>
+        <v>437</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>426</v>
+        <v>460</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>427</v>
+        <v>461</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>30</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>400</v>
+        <v>434</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>428</v>
+        <v>462</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>402</v>
+        <v>436</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>403</v>
+        <v>437</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>429</v>
+        <v>463</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>430</v>
+        <v>464</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>30</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>431</v>
+        <v>465</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>432</v>
+        <v>466</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>414</v>
+        <v>448</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>403</v>
+        <v>437</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>433</v>
+        <v>467</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>434</v>
+        <v>468</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>30</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>435</v>
+        <v>469</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>436</v>
+        <v>470</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>414</v>
+        <v>448</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>403</v>
+        <v>437</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>437</v>
+        <v>471</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>438</v>
+        <v>472</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>30</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>439</v>
+        <v>473</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>440</v>
+        <v>474</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>414</v>
+        <v>448</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>403</v>
+        <v>437</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>441</v>
+        <v>475</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>442</v>
+        <v>476</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>443</v>
+        <v>477</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>444</v>
+        <v>478</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>445</v>
+        <v>479</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>414</v>
+        <v>448</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>403</v>
+        <v>437</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>446</v>
+        <v>480</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>447</v>
+        <v>481</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>34</v>
       </c>
       <c r="C16" s="16" t="s">
-        <v>448</v>
+        <v>482</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>449</v>
+        <v>483</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>402</v>
+        <v>436</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>403</v>
+        <v>437</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>450</v>
+        <v>484</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>451</v>
+        <v>485</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>47</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>452</v>
+        <v>486</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>453</v>
+        <v>487</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>402</v>
+        <v>436</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>403</v>
+        <v>437</v>
       </c>
       <c r="G17" s="16" t="s">
-        <v>454</v>
+        <v>488</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>455</v>
+        <v>489</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>52</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>456</v>
+        <v>490</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>457</v>
+        <v>491</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>411</v>
+        <v>445</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>458</v>
+        <v>492</v>
       </c>
       <c r="G18" s="16" t="s">
-        <v>459</v>
+        <v>493</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>460</v>
+        <v>494</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>443</v>
+        <v>477</v>
       </c>
       <c r="C19" s="16" t="s">
-        <v>461</v>
+        <v>495</v>
       </c>
       <c r="D19" s="16" t="s">
-        <v>462</v>
+        <v>496</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>411</v>
+        <v>445</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>403</v>
+        <v>437</v>
       </c>
       <c r="G19" s="16" t="s">
-        <v>463</v>
+        <v>497</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>464</v>
+        <v>498</v>
       </c>
       <c r="B20" s="6" t="s">
         <v>30</v>
       </c>
       <c r="C20" s="16" t="s">
-        <v>465</v>
+        <v>499</v>
       </c>
       <c r="D20" s="16" t="s">
-        <v>466</v>
+        <v>500</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>411</v>
+        <v>445</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>403</v>
+        <v>437</v>
       </c>
       <c r="G20" s="16" t="s">
-        <v>467</v>
+        <v>501</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>468</v>
+        <v>502</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>443</v>
+        <v>477</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>465</v>
+        <v>499</v>
       </c>
       <c r="D21" s="16" t="s">
-        <v>469</v>
+        <v>503</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>414</v>
+        <v>448</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>403</v>
+        <v>437</v>
       </c>
       <c r="G21" s="16" t="s">
-        <v>470</v>
+        <v>504</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>471</v>
+        <v>505</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>443</v>
+        <v>477</v>
       </c>
       <c r="C22" s="16" t="s">
-        <v>472</v>
+        <v>506</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>473</v>
+        <v>507</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>414</v>
+        <v>448</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>403</v>
+        <v>437</v>
       </c>
       <c r="G22" s="16" t="s">
-        <v>474</v>
+        <v>508</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>475</v>
+        <v>509</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>443</v>
+        <v>477</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>476</v>
+        <v>510</v>
       </c>
       <c r="D23" s="16" t="s">
-        <v>477</v>
+        <v>511</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>411</v>
+        <v>445</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>403</v>
+        <v>437</v>
       </c>
       <c r="G23" s="16" t="s">
-        <v>478</v>
+        <v>512</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>479</v>
+        <v>513</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>443</v>
+        <v>477</v>
       </c>
       <c r="C24" s="16" t="s">
-        <v>480</v>
+        <v>514</v>
       </c>
       <c r="D24" s="16" t="s">
-        <v>481</v>
+        <v>515</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>402</v>
+        <v>436</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>403</v>
+        <v>437</v>
       </c>
       <c r="G24" s="16" t="s">
-        <v>482</v>
+        <v>516</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>483</v>
+        <v>517</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>443</v>
+        <v>477</v>
       </c>
       <c r="C25" s="16" t="s">
-        <v>484</v>
+        <v>518</v>
       </c>
       <c r="D25" s="16" t="s">
-        <v>485</v>
+        <v>519</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>414</v>
+        <v>448</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>403</v>
+        <v>437</v>
       </c>
       <c r="G25" s="16" t="s">
-        <v>486</v>
+        <v>520</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>487</v>
+        <v>521</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>443</v>
+        <v>477</v>
       </c>
       <c r="C26" s="16" t="s">
-        <v>488</v>
+        <v>522</v>
       </c>
       <c r="D26" s="16" t="s">
-        <v>489</v>
+        <v>523</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>411</v>
+        <v>445</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>403</v>
+        <v>437</v>
       </c>
       <c r="G26" s="16" t="s">
-        <v>490</v>
+        <v>524</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>491</v>
+        <v>525</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>443</v>
+        <v>477</v>
       </c>
       <c r="C27" s="16" t="s">
-        <v>492</v>
+        <v>526</v>
       </c>
       <c r="D27" s="16" t="s">
-        <v>493</v>
+        <v>527</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>402</v>
+        <v>436</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>403</v>
+        <v>437</v>
       </c>
       <c r="G27" s="16" t="s">
-        <v>494</v>
+        <v>528</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>495</v>
+        <v>529</v>
       </c>
       <c r="B28" s="6" t="s">
         <v>39</v>
       </c>
       <c r="C28" s="16" t="s">
-        <v>406</v>
+        <v>440</v>
       </c>
       <c r="D28" s="16" t="s">
-        <v>496</v>
+        <v>530</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>402</v>
+        <v>436</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>403</v>
+        <v>437</v>
       </c>
       <c r="G28" s="16" t="s">
-        <v>497</v>
+        <v>531</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>498</v>
+        <v>532</v>
       </c>
       <c r="B29" s="6" t="s">
         <v>43</v>
       </c>
       <c r="C29" s="16" t="s">
-        <v>409</v>
+        <v>443</v>
       </c>
       <c r="D29" s="16" t="s">
-        <v>499</v>
+        <v>533</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>414</v>
+        <v>448</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>403</v>
+        <v>437</v>
       </c>
       <c r="G29" s="16" t="s">
-        <v>500</v>
+        <v>534</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>501</v>
+        <v>535</v>
       </c>
       <c r="B30" s="6" t="s">
         <v>43</v>
       </c>
       <c r="C30" s="16" t="s">
-        <v>420</v>
+        <v>454</v>
       </c>
       <c r="D30" s="16" t="s">
-        <v>502</v>
+        <v>536</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>414</v>
+        <v>448</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>403</v>
+        <v>437</v>
       </c>
       <c r="G30" s="16" t="s">
-        <v>503</v>
+        <v>537</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>504</v>
+        <v>538</v>
       </c>
       <c r="B31" s="6" t="s">
         <v>47</v>
       </c>
       <c r="C31" s="16" t="s">
-        <v>505</v>
+        <v>539</v>
       </c>
       <c r="D31" s="16" t="s">
-        <v>506</v>
+        <v>540</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>402</v>
+        <v>436</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>403</v>
+        <v>437</v>
       </c>
       <c r="G31" s="16" t="s">
-        <v>507</v>
+        <v>541</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>508</v>
+        <v>542</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>509</v>
+        <v>543</v>
       </c>
       <c r="C32" s="16" t="s">
-        <v>465</v>
+        <v>499</v>
       </c>
       <c r="D32" s="16" t="s">
-        <v>510</v>
+        <v>544</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>402</v>
+        <v>436</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>403</v>
+        <v>437</v>
       </c>
       <c r="G32" s="16" t="s">
-        <v>511</v>
+        <v>545</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="s">
-        <v>512</v>
+        <v>546</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>509</v>
+        <v>543</v>
       </c>
       <c r="C33" s="16" t="s">
-        <v>513</v>
+        <v>547</v>
       </c>
       <c r="D33" s="16" t="s">
-        <v>514</v>
+        <v>548</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>402</v>
+        <v>436</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>403</v>
+        <v>437</v>
       </c>
       <c r="G33" s="16" t="s">
-        <v>515</v>
+        <v>549</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="s">
-        <v>516</v>
+        <v>550</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>443</v>
+        <v>477</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>517</v>
+        <v>551</v>
       </c>
       <c r="D34" s="16" t="s">
-        <v>518</v>
+        <v>552</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>411</v>
+        <v>445</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>519</v>
+        <v>553</v>
       </c>
       <c r="G34" s="16" t="s">
-        <v>520</v>
+        <v>554</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="6" t="s">
-        <v>521</v>
+        <v>555</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>443</v>
+        <v>477</v>
       </c>
       <c r="C35" s="16" t="s">
-        <v>522</v>
+        <v>556</v>
       </c>
       <c r="D35" s="16" t="s">
-        <v>523</v>
+        <v>557</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>411</v>
+        <v>445</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>519</v>
+        <v>553</v>
       </c>
       <c r="G35" s="16" t="s">
-        <v>524</v>
+        <v>558</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="s">
-        <v>525</v>
+        <v>559</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>443</v>
+        <v>477</v>
       </c>
       <c r="C36" s="16" t="s">
-        <v>522</v>
+        <v>556</v>
       </c>
       <c r="D36" s="16" t="s">
-        <v>526</v>
+        <v>560</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>411</v>
+        <v>445</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>403</v>
+        <v>437</v>
       </c>
       <c r="G36" s="16" t="s">
-        <v>527</v>
+        <v>561</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="19" t="s">
-        <v>528</v>
-      </c>
-      <c r="B37" s="19" t="s">
+      <c r="A37" s="20" t="s">
+        <v>562</v>
+      </c>
+      <c r="B37" s="20" t="s">
         <v>56</v>
       </c>
-      <c r="C37" s="19" t="s">
-        <v>529</v>
+      <c r="C37" s="20" t="s">
+        <v>563</v>
       </c>
       <c r="D37" s="16" t="s">
-        <v>530</v>
-      </c>
-      <c r="E37" s="19" t="s">
-        <v>414</v>
-      </c>
-      <c r="F37" s="19" t="s">
-        <v>403</v>
+        <v>564</v>
+      </c>
+      <c r="E37" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="F37" s="20" t="s">
+        <v>437</v>
       </c>
       <c r="G37" s="16" t="s">
-        <v>531</v>
+        <v>565</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="19" t="s">
-        <v>532</v>
-      </c>
-      <c r="B38" s="19" t="s">
-        <v>533</v>
-      </c>
-      <c r="C38" s="19" t="s">
-        <v>534</v>
+      <c r="A38" s="20" t="s">
+        <v>566</v>
+      </c>
+      <c r="B38" s="20" t="s">
+        <v>567</v>
+      </c>
+      <c r="C38" s="20" t="s">
+        <v>568</v>
       </c>
       <c r="D38" s="16" t="s">
-        <v>535</v>
-      </c>
-      <c r="E38" s="19" t="s">
-        <v>411</v>
-      </c>
-      <c r="F38" s="19" t="s">
-        <v>519</v>
+        <v>569</v>
+      </c>
+      <c r="E38" s="20" t="s">
+        <v>445</v>
+      </c>
+      <c r="F38" s="20" t="s">
+        <v>553</v>
       </c>
       <c r="G38" s="16" t="s">
-        <v>536</v>
+        <v>570</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="19" t="s">
-        <v>537</v>
-      </c>
-      <c r="B39" s="19" t="s">
+      <c r="A39" s="20" t="s">
+        <v>571</v>
+      </c>
+      <c r="B39" s="20" t="s">
         <v>52</v>
       </c>
-      <c r="C39" s="19" t="s">
-        <v>417</v>
+      <c r="C39" s="20" t="s">
+        <v>451</v>
       </c>
       <c r="D39" s="16" t="s">
-        <v>538</v>
-      </c>
-      <c r="E39" s="19" t="s">
-        <v>402</v>
-      </c>
-      <c r="F39" s="19" t="s">
-        <v>403</v>
+        <v>572</v>
+      </c>
+      <c r="E39" s="20" t="s">
+        <v>436</v>
+      </c>
+      <c r="F39" s="20" t="s">
+        <v>437</v>
       </c>
       <c r="G39" s="16" t="s">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="20" t="s">
+        <v>574</v>
+      </c>
+      <c r="B40" s="20" t="s">
+        <v>505</v>
+      </c>
+      <c r="C40" s="20" t="s">
+        <v>575</v>
+      </c>
+      <c r="D40" s="16" t="s">
+        <v>576</v>
+      </c>
+      <c r="E40" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="F40" s="20" t="s">
+        <v>553</v>
+      </c>
+      <c r="G40" s="16" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="20" t="s">
+        <v>578</v>
+      </c>
+      <c r="B41" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="C41" s="20" t="s">
+        <v>579</v>
+      </c>
+      <c r="D41" s="16" t="s">
+        <v>580</v>
+      </c>
+      <c r="E41" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="F41" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G41" s="16" t="s">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="20" t="s">
+        <v>582</v>
+      </c>
+      <c r="B42" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="C42" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="D42" s="16" t="s">
+        <v>584</v>
+      </c>
+      <c r="E42" s="20" t="s">
+        <v>445</v>
+      </c>
+      <c r="F42" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G42" s="16" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="20" t="s">
+        <v>586</v>
+      </c>
+      <c r="B43" s="20" t="s">
+        <v>84</v>
+      </c>
+      <c r="C43" s="20" t="s">
+        <v>587</v>
+      </c>
+      <c r="D43" s="16" t="s">
+        <v>588</v>
+      </c>
+      <c r="E43" s="20" t="s">
+        <v>445</v>
+      </c>
+      <c r="F43" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G43" s="16" t="s">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="20" t="s">
+        <v>590</v>
+      </c>
+      <c r="B44" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="C44" s="20" t="s">
+        <v>591</v>
+      </c>
+      <c r="D44" s="16" t="s">
+        <v>592</v>
+      </c>
+      <c r="E44" s="20" t="s">
+        <v>445</v>
+      </c>
+      <c r="F44" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G44" s="16" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="20" t="s">
+        <v>594</v>
+      </c>
+      <c r="B45" s="20" t="s">
+        <v>183</v>
+      </c>
+      <c r="C45" s="20" t="s">
+        <v>595</v>
+      </c>
+      <c r="D45" s="16" t="s">
+        <v>596</v>
+      </c>
+      <c r="E45" s="20" t="s">
+        <v>436</v>
+      </c>
+      <c r="F45" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G45" s="16" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="20" t="s">
+        <v>598</v>
+      </c>
+      <c r="B46" s="20" t="s">
+        <v>80</v>
+      </c>
+      <c r="C46" s="20" t="s">
+        <v>599</v>
+      </c>
+      <c r="D46" s="16" t="s">
+        <v>600</v>
+      </c>
+      <c r="E46" s="20" t="s">
+        <v>436</v>
+      </c>
+      <c r="F46" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G46" s="16" t="s">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="20" t="s">
+        <v>602</v>
+      </c>
+      <c r="B47" s="20" t="s">
+        <v>183</v>
+      </c>
+      <c r="C47" s="20" t="s">
+        <v>603</v>
+      </c>
+      <c r="D47" s="16" t="s">
+        <v>604</v>
+      </c>
+      <c r="E47" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="F47" s="20" t="s">
+        <v>553</v>
+      </c>
+      <c r="G47" s="16" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="20" t="s">
+        <v>606</v>
+      </c>
+      <c r="B48" s="20" t="s">
+        <v>183</v>
+      </c>
+      <c r="C48" s="20" t="s">
+        <v>499</v>
+      </c>
+      <c r="D48" s="16" t="s">
+        <v>607</v>
+      </c>
+      <c r="E48" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="F48" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G48" s="16" t="s">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="20" t="s">
+        <v>609</v>
+      </c>
+      <c r="B49" s="20" t="s">
+        <v>207</v>
+      </c>
+      <c r="C49" s="20" t="s">
+        <v>610</v>
+      </c>
+      <c r="D49" s="16" t="s">
+        <v>611</v>
+      </c>
+      <c r="E49" s="20" t="s">
+        <v>445</v>
+      </c>
+      <c r="F49" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G49" s="16" t="s">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="20" t="s">
+        <v>613</v>
+      </c>
+      <c r="B50" s="20" t="s">
+        <v>231</v>
+      </c>
+      <c r="C50" s="20" t="s">
+        <v>614</v>
+      </c>
+      <c r="D50" s="16" t="s">
+        <v>615</v>
+      </c>
+      <c r="E50" s="20" t="s">
+        <v>436</v>
+      </c>
+      <c r="F50" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G50" s="16" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="20" t="s">
+        <v>617</v>
+      </c>
+      <c r="B51" s="20" t="s">
+        <v>231</v>
+      </c>
+      <c r="C51" s="20" t="s">
+        <v>618</v>
+      </c>
+      <c r="D51" s="16" t="s">
+        <v>619</v>
+      </c>
+      <c r="E51" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="F51" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G51" s="16" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="20" t="s">
+        <v>621</v>
+      </c>
+      <c r="B52" s="20" t="s">
+        <v>231</v>
+      </c>
+      <c r="C52" s="20" t="s">
+        <v>587</v>
+      </c>
+      <c r="D52" s="16" t="s">
+        <v>622</v>
+      </c>
+      <c r="E52" s="20" t="s">
+        <v>445</v>
+      </c>
+      <c r="F52" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G52" s="16" t="s">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="20" t="s">
+        <v>624</v>
+      </c>
+      <c r="B53" s="20" t="s">
+        <v>231</v>
+      </c>
+      <c r="C53" s="20" t="s">
+        <v>625</v>
+      </c>
+      <c r="D53" s="16" t="s">
+        <v>626</v>
+      </c>
+      <c r="E53" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="F53" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G53" s="16" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="20" t="s">
+        <v>628</v>
+      </c>
+      <c r="B54" s="20" t="s">
+        <v>231</v>
+      </c>
+      <c r="C54" s="20" t="s">
+        <v>629</v>
+      </c>
+      <c r="D54" s="16" t="s">
+        <v>630</v>
+      </c>
+      <c r="E54" s="20" t="s">
+        <v>436</v>
+      </c>
+      <c r="F54" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G54" s="16" t="s">
+        <v>631</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="20" t="s">
+        <v>632</v>
+      </c>
+      <c r="B55" s="20" t="s">
+        <v>231</v>
+      </c>
+      <c r="C55" s="20" t="s">
+        <v>633</v>
+      </c>
+      <c r="D55" s="16" t="s">
+        <v>634</v>
+      </c>
+      <c r="E55" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="F55" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G55" s="16" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="20" t="s">
+        <v>636</v>
+      </c>
+      <c r="B56" s="20" t="s">
+        <v>231</v>
+      </c>
+      <c r="C56" s="20" t="s">
+        <v>625</v>
+      </c>
+      <c r="D56" s="16" t="s">
+        <v>637</v>
+      </c>
+      <c r="E56" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="F56" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G56" s="16" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="20" t="s">
+        <v>639</v>
+      </c>
+      <c r="B57" s="20" t="s">
+        <v>231</v>
+      </c>
+      <c r="C57" s="20" t="s">
+        <v>640</v>
+      </c>
+      <c r="D57" s="16" t="s">
+        <v>641</v>
+      </c>
+      <c r="E57" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="F57" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G57" s="16" t="s">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="20" t="s">
+        <v>643</v>
+      </c>
+      <c r="B58" s="20" t="s">
+        <v>231</v>
+      </c>
+      <c r="C58" s="20" t="s">
+        <v>644</v>
+      </c>
+      <c r="D58" s="16" t="s">
+        <v>645</v>
+      </c>
+      <c r="E58" s="20" t="s">
+        <v>436</v>
+      </c>
+      <c r="F58" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G58" s="16" t="s">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="20" t="s">
+        <v>647</v>
+      </c>
+      <c r="B59" s="20" t="s">
+        <v>231</v>
+      </c>
+      <c r="C59" s="20" t="s">
+        <v>648</v>
+      </c>
+      <c r="D59" s="16" t="s">
+        <v>649</v>
+      </c>
+      <c r="E59" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="F59" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G59" s="16" t="s">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="20" t="s">
+        <v>651</v>
+      </c>
+      <c r="B60" s="20" t="s">
+        <v>231</v>
+      </c>
+      <c r="C60" s="20" t="s">
+        <v>652</v>
+      </c>
+      <c r="D60" s="16" t="s">
+        <v>653</v>
+      </c>
+      <c r="E60" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="F60" s="20" t="s">
+        <v>492</v>
+      </c>
+      <c r="G60" s="16" t="s">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="20" t="s">
+        <v>655</v>
+      </c>
+      <c r="B61" s="20" t="s">
+        <v>231</v>
+      </c>
+      <c r="C61" s="20" t="s">
+        <v>656</v>
+      </c>
+      <c r="D61" s="16" t="s">
+        <v>657</v>
+      </c>
+      <c r="E61" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="F61" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G61" s="16" t="s">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="20" t="s">
+        <v>659</v>
+      </c>
+      <c r="B62" s="20" t="s">
+        <v>255</v>
+      </c>
+      <c r="C62" s="20" t="s">
+        <v>660</v>
+      </c>
+      <c r="D62" s="16" t="s">
+        <v>661</v>
+      </c>
+      <c r="E62" s="20" t="s">
+        <v>436</v>
+      </c>
+      <c r="F62" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G62" s="16" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="20" t="s">
+        <v>663</v>
+      </c>
+      <c r="B63" s="20" t="s">
+        <v>267</v>
+      </c>
+      <c r="C63" s="20" t="s">
+        <v>664</v>
+      </c>
+      <c r="D63" s="16" t="s">
+        <v>665</v>
+      </c>
+      <c r="E63" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="F63" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G63" s="16" t="s">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="20" t="s">
+        <v>667</v>
+      </c>
+      <c r="B64" s="20" t="s">
+        <v>275</v>
+      </c>
+      <c r="C64" s="20" t="s">
+        <v>668</v>
+      </c>
+      <c r="D64" s="16" t="s">
+        <v>669</v>
+      </c>
+      <c r="E64" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="F64" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G64" s="16" t="s">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="20" t="s">
+        <v>671</v>
+      </c>
+      <c r="B65" s="20" t="s">
+        <v>263</v>
+      </c>
+      <c r="C65" s="20" t="s">
         <v>539</v>
       </c>
-    </row>
-    <row r="40" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="19" t="s">
-        <v>540</v>
-      </c>
-      <c r="B40" s="19" t="s">
-        <v>471</v>
-      </c>
-      <c r="C40" s="19" t="s">
-        <v>541</v>
-      </c>
-      <c r="D40" s="16" t="s">
-        <v>542</v>
-      </c>
-      <c r="E40" s="19" t="s">
-        <v>414</v>
-      </c>
-      <c r="F40" s="19" t="s">
-        <v>519</v>
-      </c>
-      <c r="G40" s="16" t="s">
-        <v>543</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="19" t="s">
-        <v>544</v>
-      </c>
-      <c r="B41" s="19" t="s">
-        <v>76</v>
-      </c>
-      <c r="C41" s="19" t="s">
-        <v>545</v>
-      </c>
-      <c r="D41" s="16" t="s">
-        <v>546</v>
-      </c>
-      <c r="E41" s="19" t="s">
-        <v>414</v>
-      </c>
-      <c r="F41" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G41" s="16" t="s">
-        <v>547</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="19" t="s">
-        <v>548</v>
-      </c>
-      <c r="B42" s="19" t="s">
-        <v>76</v>
-      </c>
-      <c r="C42" s="19" t="s">
-        <v>549</v>
-      </c>
-      <c r="D42" s="16" t="s">
-        <v>550</v>
-      </c>
-      <c r="E42" s="19" t="s">
-        <v>411</v>
-      </c>
-      <c r="F42" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G42" s="16" t="s">
-        <v>551</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="19" t="s">
-        <v>552</v>
-      </c>
-      <c r="B43" s="19" t="s">
-        <v>84</v>
-      </c>
-      <c r="C43" s="19" t="s">
+      <c r="D65" s="16" t="s">
+        <v>672</v>
+      </c>
+      <c r="E65" s="20" t="s">
+        <v>445</v>
+      </c>
+      <c r="F65" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G65" s="16" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="20" t="s">
+        <v>674</v>
+      </c>
+      <c r="B66" s="20" t="s">
+        <v>275</v>
+      </c>
+      <c r="C66" s="20" t="s">
+        <v>675</v>
+      </c>
+      <c r="D66" s="16" t="s">
+        <v>676</v>
+      </c>
+      <c r="E66" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="F66" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G66" s="16" t="s">
+        <v>677</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="20" t="s">
+        <v>678</v>
+      </c>
+      <c r="B67" s="20" t="s">
+        <v>271</v>
+      </c>
+      <c r="C67" s="20" t="s">
+        <v>679</v>
+      </c>
+      <c r="D67" s="16" t="s">
+        <v>680</v>
+      </c>
+      <c r="E67" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="F67" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G67" s="16" t="s">
+        <v>681</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="20" t="s">
+        <v>682</v>
+      </c>
+      <c r="B68" s="20" t="s">
+        <v>307</v>
+      </c>
+      <c r="C68" s="20" t="s">
+        <v>683</v>
+      </c>
+      <c r="D68" s="16" t="s">
+        <v>684</v>
+      </c>
+      <c r="E68" s="20" t="s">
+        <v>436</v>
+      </c>
+      <c r="F68" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G68" s="16" t="s">
+        <v>685</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="20" t="s">
+        <v>686</v>
+      </c>
+      <c r="B69" s="20" t="s">
+        <v>307</v>
+      </c>
+      <c r="C69" s="20" t="s">
+        <v>687</v>
+      </c>
+      <c r="D69" s="16" t="s">
+        <v>688</v>
+      </c>
+      <c r="E69" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="F69" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G69" s="16" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A70" s="20" t="s">
+        <v>690</v>
+      </c>
+      <c r="B70" s="20" t="s">
+        <v>307</v>
+      </c>
+      <c r="C70" s="20" t="s">
+        <v>691</v>
+      </c>
+      <c r="D70" s="16" t="s">
+        <v>692</v>
+      </c>
+      <c r="E70" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="F70" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G70" s="16" t="s">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A71" s="20" t="s">
+        <v>694</v>
+      </c>
+      <c r="B71" s="20" t="s">
+        <v>263</v>
+      </c>
+      <c r="C71" s="20" t="s">
+        <v>695</v>
+      </c>
+      <c r="D71" s="16" t="s">
+        <v>696</v>
+      </c>
+      <c r="E71" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="F71" s="20" t="s">
+        <v>492</v>
+      </c>
+      <c r="G71" s="16" t="s">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A72" s="20" t="s">
+        <v>698</v>
+      </c>
+      <c r="B72" s="20" t="s">
+        <v>699</v>
+      </c>
+      <c r="C72" s="20" t="s">
+        <v>700</v>
+      </c>
+      <c r="D72" s="16" t="s">
+        <v>701</v>
+      </c>
+      <c r="E72" s="20" t="s">
+        <v>436</v>
+      </c>
+      <c r="F72" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G72" s="16" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A73" s="20" t="s">
+        <v>703</v>
+      </c>
+      <c r="B73" s="20" t="s">
+        <v>699</v>
+      </c>
+      <c r="C73" s="20" t="s">
+        <v>704</v>
+      </c>
+      <c r="D73" s="16" t="s">
+        <v>705</v>
+      </c>
+      <c r="E73" s="20" t="s">
+        <v>436</v>
+      </c>
+      <c r="F73" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G73" s="16" t="s">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A74" s="20" t="s">
+        <v>707</v>
+      </c>
+      <c r="B74" s="20" t="s">
+        <v>699</v>
+      </c>
+      <c r="C74" s="20" t="s">
+        <v>644</v>
+      </c>
+      <c r="D74" s="16" t="s">
+        <v>708</v>
+      </c>
+      <c r="E74" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="F74" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G74" s="16" t="s">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A75" s="20" t="s">
+        <v>710</v>
+      </c>
+      <c r="B75" s="20" t="s">
+        <v>351</v>
+      </c>
+      <c r="C75" s="20" t="s">
+        <v>711</v>
+      </c>
+      <c r="D75" s="16" t="s">
+        <v>712</v>
+      </c>
+      <c r="E75" s="20" t="s">
+        <v>436</v>
+      </c>
+      <c r="F75" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G75" s="16" t="s">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A76" s="20" t="s">
+        <v>714</v>
+      </c>
+      <c r="B76" s="20" t="s">
+        <v>351</v>
+      </c>
+      <c r="C76" s="20" t="s">
+        <v>715</v>
+      </c>
+      <c r="D76" s="16" t="s">
+        <v>716</v>
+      </c>
+      <c r="E76" s="20" t="s">
+        <v>436</v>
+      </c>
+      <c r="F76" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G76" s="16" t="s">
+        <v>717</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A77" s="20" t="s">
+        <v>718</v>
+      </c>
+      <c r="B77" s="20" t="s">
+        <v>351</v>
+      </c>
+      <c r="C77" s="20" t="s">
+        <v>719</v>
+      </c>
+      <c r="D77" s="16" t="s">
+        <v>720</v>
+      </c>
+      <c r="E77" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="F77" s="20" t="s">
         <v>553</v>
       </c>
-      <c r="D43" s="16" t="s">
-        <v>554</v>
-      </c>
-      <c r="E43" s="19" t="s">
-        <v>411</v>
-      </c>
-      <c r="F43" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G43" s="16" t="s">
-        <v>555</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="19" t="s">
-        <v>556</v>
-      </c>
-      <c r="B44" s="19" t="s">
-        <v>76</v>
-      </c>
-      <c r="C44" s="19" t="s">
-        <v>557</v>
-      </c>
-      <c r="D44" s="16" t="s">
-        <v>558</v>
-      </c>
-      <c r="E44" s="19" t="s">
-        <v>411</v>
-      </c>
-      <c r="F44" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G44" s="16" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="19" t="s">
-        <v>560</v>
-      </c>
-      <c r="B45" s="19" t="s">
-        <v>183</v>
-      </c>
-      <c r="C45" s="19" t="s">
-        <v>561</v>
-      </c>
-      <c r="D45" s="16" t="s">
-        <v>562</v>
-      </c>
-      <c r="E45" s="19" t="s">
-        <v>402</v>
-      </c>
-      <c r="F45" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G45" s="16" t="s">
-        <v>563</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="19" t="s">
-        <v>564</v>
-      </c>
-      <c r="B46" s="19" t="s">
-        <v>80</v>
-      </c>
-      <c r="C46" s="19" t="s">
-        <v>565</v>
-      </c>
-      <c r="D46" s="16" t="s">
-        <v>566</v>
-      </c>
-      <c r="E46" s="19" t="s">
-        <v>402</v>
-      </c>
-      <c r="F46" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G46" s="16" t="s">
-        <v>567</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="19" t="s">
-        <v>568</v>
-      </c>
-      <c r="B47" s="19" t="s">
-        <v>183</v>
-      </c>
-      <c r="C47" s="19" t="s">
-        <v>569</v>
-      </c>
-      <c r="D47" s="16" t="s">
-        <v>570</v>
-      </c>
-      <c r="E47" s="19" t="s">
-        <v>414</v>
-      </c>
-      <c r="F47" s="19" t="s">
-        <v>519</v>
-      </c>
-      <c r="G47" s="16" t="s">
-        <v>571</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="19" t="s">
-        <v>572</v>
-      </c>
-      <c r="B48" s="19" t="s">
-        <v>183</v>
-      </c>
-      <c r="C48" s="19" t="s">
-        <v>465</v>
-      </c>
-      <c r="D48" s="16" t="s">
-        <v>573</v>
-      </c>
-      <c r="E48" s="19" t="s">
-        <v>414</v>
-      </c>
-      <c r="F48" s="19" t="s">
-        <v>519</v>
-      </c>
-      <c r="G48" s="16" t="s">
-        <v>574</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="19" t="s">
-        <v>575</v>
-      </c>
-      <c r="B49" s="19" t="s">
-        <v>207</v>
-      </c>
-      <c r="C49" s="19" t="s">
-        <v>576</v>
-      </c>
-      <c r="D49" s="16" t="s">
-        <v>577</v>
-      </c>
-      <c r="E49" s="19" t="s">
-        <v>411</v>
-      </c>
-      <c r="F49" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G49" s="16" t="s">
-        <v>578</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="19" t="s">
-        <v>579</v>
-      </c>
-      <c r="B50" s="19" t="s">
-        <v>231</v>
-      </c>
-      <c r="C50" s="19" t="s">
-        <v>580</v>
-      </c>
-      <c r="D50" s="16" t="s">
-        <v>581</v>
-      </c>
-      <c r="E50" s="19" t="s">
-        <v>402</v>
-      </c>
-      <c r="F50" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G50" s="16" t="s">
-        <v>582</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="19" t="s">
-        <v>583</v>
-      </c>
-      <c r="B51" s="19" t="s">
-        <v>231</v>
-      </c>
-      <c r="C51" s="19" t="s">
-        <v>584</v>
-      </c>
-      <c r="D51" s="16" t="s">
-        <v>585</v>
-      </c>
-      <c r="E51" s="19" t="s">
-        <v>414</v>
-      </c>
-      <c r="F51" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G51" s="16" t="s">
-        <v>586</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="19" t="s">
-        <v>587</v>
-      </c>
-      <c r="B52" s="19" t="s">
-        <v>231</v>
-      </c>
-      <c r="C52" s="19" t="s">
+      <c r="G77" s="16" t="s">
+        <v>721</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A78" s="20" t="s">
+        <v>722</v>
+      </c>
+      <c r="B78" s="20" t="s">
+        <v>723</v>
+      </c>
+      <c r="C78" s="20" t="s">
+        <v>724</v>
+      </c>
+      <c r="D78" s="16" t="s">
+        <v>725</v>
+      </c>
+      <c r="E78" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="F78" s="20" t="s">
         <v>553</v>
       </c>
-      <c r="D52" s="16" t="s">
-        <v>588</v>
-      </c>
-      <c r="E52" s="19" t="s">
-        <v>411</v>
-      </c>
-      <c r="F52" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G52" s="16" t="s">
-        <v>589</v>
-      </c>
-    </row>
-    <row r="53" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="19" t="s">
-        <v>590</v>
-      </c>
-      <c r="B53" s="19" t="s">
-        <v>231</v>
-      </c>
-      <c r="C53" s="19" t="s">
-        <v>591</v>
-      </c>
-      <c r="D53" s="16" t="s">
-        <v>592</v>
-      </c>
-      <c r="E53" s="19" t="s">
-        <v>414</v>
-      </c>
-      <c r="F53" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G53" s="16" t="s">
-        <v>593</v>
-      </c>
-    </row>
-    <row r="54" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="19" t="s">
-        <v>594</v>
-      </c>
-      <c r="B54" s="19" t="s">
-        <v>231</v>
-      </c>
-      <c r="C54" s="19" t="s">
-        <v>595</v>
-      </c>
-      <c r="D54" s="16" t="s">
-        <v>596</v>
-      </c>
-      <c r="E54" s="19" t="s">
-        <v>402</v>
-      </c>
-      <c r="F54" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G54" s="16" t="s">
-        <v>597</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="19" t="s">
-        <v>598</v>
-      </c>
-      <c r="B55" s="19" t="s">
-        <v>231</v>
-      </c>
-      <c r="C55" s="19" t="s">
-        <v>599</v>
-      </c>
-      <c r="D55" s="16" t="s">
-        <v>600</v>
-      </c>
-      <c r="E55" s="19" t="s">
-        <v>414</v>
-      </c>
-      <c r="F55" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G55" s="16" t="s">
-        <v>601</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="19" t="s">
-        <v>602</v>
-      </c>
-      <c r="B56" s="19" t="s">
-        <v>231</v>
-      </c>
-      <c r="C56" s="19" t="s">
-        <v>591</v>
-      </c>
-      <c r="D56" s="16" t="s">
-        <v>603</v>
-      </c>
-      <c r="E56" s="19" t="s">
-        <v>414</v>
-      </c>
-      <c r="F56" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G56" s="16" t="s">
-        <v>604</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="19" t="s">
-        <v>605</v>
-      </c>
-      <c r="B57" s="19" t="s">
-        <v>231</v>
-      </c>
-      <c r="C57" s="19" t="s">
-        <v>606</v>
-      </c>
-      <c r="D57" s="16" t="s">
-        <v>607</v>
-      </c>
-      <c r="E57" s="19" t="s">
-        <v>414</v>
-      </c>
-      <c r="F57" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G57" s="16" t="s">
-        <v>608</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="19" t="s">
-        <v>609</v>
-      </c>
-      <c r="B58" s="19" t="s">
-        <v>231</v>
-      </c>
-      <c r="C58" s="19" t="s">
-        <v>610</v>
-      </c>
-      <c r="D58" s="16" t="s">
-        <v>611</v>
-      </c>
-      <c r="E58" s="19" t="s">
-        <v>402</v>
-      </c>
-      <c r="F58" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G58" s="16" t="s">
-        <v>612</v>
-      </c>
-    </row>
-    <row r="59" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="19" t="s">
-        <v>613</v>
-      </c>
-      <c r="B59" s="19" t="s">
-        <v>231</v>
-      </c>
-      <c r="C59" s="19" t="s">
-        <v>614</v>
-      </c>
-      <c r="D59" s="16" t="s">
-        <v>615</v>
-      </c>
-      <c r="E59" s="19" t="s">
-        <v>414</v>
-      </c>
-      <c r="F59" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G59" s="16" t="s">
-        <v>616</v>
-      </c>
-    </row>
-    <row r="60" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="19" t="s">
-        <v>617</v>
-      </c>
-      <c r="B60" s="19" t="s">
-        <v>231</v>
-      </c>
-      <c r="C60" s="19" t="s">
-        <v>618</v>
-      </c>
-      <c r="D60" s="16" t="s">
-        <v>619</v>
-      </c>
-      <c r="E60" s="19" t="s">
-        <v>414</v>
-      </c>
-      <c r="F60" s="19" t="s">
-        <v>458</v>
-      </c>
-      <c r="G60" s="16" t="s">
-        <v>620</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="19" t="s">
-        <v>621</v>
-      </c>
-      <c r="B61" s="19" t="s">
-        <v>231</v>
-      </c>
-      <c r="C61" s="19" t="s">
-        <v>622</v>
-      </c>
-      <c r="D61" s="16" t="s">
-        <v>623</v>
-      </c>
-      <c r="E61" s="19" t="s">
-        <v>414</v>
-      </c>
-      <c r="F61" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G61" s="16" t="s">
-        <v>624</v>
-      </c>
-    </row>
-    <row r="62" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="19" t="s">
-        <v>625</v>
-      </c>
-      <c r="B62" s="19" t="s">
-        <v>255</v>
-      </c>
-      <c r="C62" s="19" t="s">
-        <v>626</v>
-      </c>
-      <c r="D62" s="16" t="s">
-        <v>627</v>
-      </c>
-      <c r="E62" s="19" t="s">
-        <v>402</v>
-      </c>
-      <c r="F62" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G62" s="16" t="s">
-        <v>628</v>
-      </c>
-    </row>
-    <row r="63" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="19" t="s">
-        <v>629</v>
-      </c>
-      <c r="B63" s="19" t="s">
-        <v>267</v>
-      </c>
-      <c r="C63" s="19" t="s">
-        <v>630</v>
-      </c>
-      <c r="D63" s="16" t="s">
-        <v>631</v>
-      </c>
-      <c r="E63" s="19" t="s">
-        <v>414</v>
-      </c>
-      <c r="F63" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G63" s="16" t="s">
-        <v>632</v>
-      </c>
-    </row>
-    <row r="64" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="19" t="s">
-        <v>633</v>
-      </c>
-      <c r="B64" s="19" t="s">
-        <v>275</v>
-      </c>
-      <c r="C64" s="19" t="s">
-        <v>634</v>
-      </c>
-      <c r="D64" s="16" t="s">
-        <v>635</v>
-      </c>
-      <c r="E64" s="19" t="s">
-        <v>414</v>
-      </c>
-      <c r="F64" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G64" s="16" t="s">
-        <v>636</v>
-      </c>
-    </row>
-    <row r="65" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="B65" s="19" t="s">
-        <v>263</v>
-      </c>
-      <c r="C65" s="19" t="s">
-        <v>505</v>
-      </c>
-      <c r="D65" s="16" t="s">
-        <v>638</v>
-      </c>
-      <c r="E65" s="19" t="s">
-        <v>411</v>
-      </c>
-      <c r="F65" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G65" s="16" t="s">
-        <v>639</v>
-      </c>
-    </row>
-    <row r="66" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="19" t="s">
-        <v>640</v>
-      </c>
-      <c r="B66" s="19" t="s">
-        <v>275</v>
-      </c>
-      <c r="C66" s="19" t="s">
-        <v>641</v>
-      </c>
-      <c r="D66" s="16" t="s">
-        <v>642</v>
-      </c>
-      <c r="E66" s="19" t="s">
-        <v>414</v>
-      </c>
-      <c r="F66" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G66" s="16" t="s">
-        <v>643</v>
-      </c>
-    </row>
-    <row r="67" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="19" t="s">
-        <v>644</v>
-      </c>
-      <c r="B67" s="19" t="s">
-        <v>271</v>
-      </c>
-      <c r="C67" s="19" t="s">
-        <v>645</v>
-      </c>
-      <c r="D67" s="16" t="s">
-        <v>646</v>
-      </c>
-      <c r="E67" s="19" t="s">
-        <v>414</v>
-      </c>
-      <c r="F67" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G67" s="16" t="s">
-        <v>647</v>
-      </c>
-    </row>
-    <row r="68" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="19" t="s">
-        <v>648</v>
-      </c>
-      <c r="B68" s="19" t="s">
-        <v>307</v>
-      </c>
-      <c r="C68" s="19" t="s">
-        <v>649</v>
-      </c>
-      <c r="D68" s="16" t="s">
-        <v>650</v>
-      </c>
-      <c r="E68" s="19" t="s">
-        <v>402</v>
-      </c>
-      <c r="F68" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G68" s="16" t="s">
-        <v>651</v>
-      </c>
-    </row>
-    <row r="69" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="19" t="s">
-        <v>652</v>
-      </c>
-      <c r="B69" s="19" t="s">
-        <v>307</v>
-      </c>
-      <c r="C69" s="19" t="s">
-        <v>653</v>
-      </c>
-      <c r="D69" s="16" t="s">
-        <v>654</v>
-      </c>
-      <c r="E69" s="19" t="s">
-        <v>414</v>
-      </c>
-      <c r="F69" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G69" s="16" t="s">
-        <v>655</v>
-      </c>
-    </row>
-    <row r="70" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="19" t="s">
-        <v>656</v>
-      </c>
-      <c r="B70" s="19" t="s">
-        <v>307</v>
-      </c>
-      <c r="C70" s="19" t="s">
-        <v>657</v>
-      </c>
-      <c r="D70" s="16" t="s">
-        <v>658</v>
-      </c>
-      <c r="E70" s="19" t="s">
-        <v>414</v>
-      </c>
-      <c r="F70" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G70" s="16" t="s">
-        <v>659</v>
-      </c>
-    </row>
-    <row r="71" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A71" s="19" t="s">
-        <v>660</v>
-      </c>
-      <c r="B71" s="19" t="s">
-        <v>263</v>
-      </c>
-      <c r="C71" s="19" t="s">
-        <v>661</v>
-      </c>
-      <c r="D71" s="16" t="s">
-        <v>662</v>
-      </c>
-      <c r="E71" s="19" t="s">
-        <v>414</v>
-      </c>
-      <c r="F71" s="19" t="s">
-        <v>458</v>
-      </c>
-      <c r="G71" s="16" t="s">
-        <v>663</v>
-      </c>
-    </row>
-    <row r="72" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A72" s="19" t="s">
-        <v>664</v>
-      </c>
-      <c r="B72" s="19" t="s">
-        <v>665</v>
-      </c>
-      <c r="C72" s="19" t="s">
-        <v>666</v>
-      </c>
-      <c r="D72" s="16" t="s">
-        <v>667</v>
-      </c>
-      <c r="E72" s="19" t="s">
-        <v>402</v>
-      </c>
-      <c r="F72" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G72" s="16" t="s">
-        <v>668</v>
-      </c>
-    </row>
-    <row r="73" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="19" t="s">
-        <v>669</v>
-      </c>
-      <c r="B73" s="19" t="s">
-        <v>665</v>
-      </c>
-      <c r="C73" s="19" t="s">
-        <v>670</v>
-      </c>
-      <c r="D73" s="16" t="s">
-        <v>671</v>
-      </c>
-      <c r="E73" s="19" t="s">
-        <v>402</v>
-      </c>
-      <c r="F73" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G73" s="16" t="s">
-        <v>672</v>
-      </c>
-    </row>
-    <row r="74" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A74" s="19" t="s">
-        <v>673</v>
-      </c>
-      <c r="B74" s="19" t="s">
-        <v>665</v>
-      </c>
-      <c r="C74" s="19" t="s">
-        <v>610</v>
-      </c>
-      <c r="D74" s="16" t="s">
-        <v>674</v>
-      </c>
-      <c r="E74" s="19" t="s">
-        <v>414</v>
-      </c>
-      <c r="F74" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G74" s="16" t="s">
-        <v>675</v>
-      </c>
-    </row>
-    <row r="75" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A75" s="19" t="s">
-        <v>676</v>
-      </c>
-      <c r="B75" s="19" t="s">
+      <c r="G78" s="16" t="s">
+        <v>726</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A79" s="20" t="s">
+        <v>727</v>
+      </c>
+      <c r="B79" s="20" t="s">
+        <v>723</v>
+      </c>
+      <c r="C79" s="20" t="s">
+        <v>728</v>
+      </c>
+      <c r="D79" s="16" t="s">
+        <v>729</v>
+      </c>
+      <c r="E79" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="F79" s="20" t="s">
+        <v>553</v>
+      </c>
+      <c r="G79" s="16" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A80" s="20" t="s">
+        <v>731</v>
+      </c>
+      <c r="B80" s="20" t="s">
+        <v>379</v>
+      </c>
+      <c r="C80" s="20" t="s">
+        <v>732</v>
+      </c>
+      <c r="D80" s="16" t="s">
+        <v>733</v>
+      </c>
+      <c r="E80" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="F80" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G80" s="16" t="s">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A81" s="20" t="s">
+        <v>735</v>
+      </c>
+      <c r="B81" s="20" t="s">
+        <v>371</v>
+      </c>
+      <c r="C81" s="20" t="s">
+        <v>736</v>
+      </c>
+      <c r="D81" s="16" t="s">
+        <v>737</v>
+      </c>
+      <c r="E81" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="F81" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G81" s="16" t="s">
+        <v>738</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A82" s="20" t="s">
+        <v>739</v>
+      </c>
+      <c r="B82" s="20" t="s">
+        <v>367</v>
+      </c>
+      <c r="C82" s="20" t="s">
+        <v>740</v>
+      </c>
+      <c r="D82" s="16" t="s">
+        <v>741</v>
+      </c>
+      <c r="E82" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="F82" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G82" s="16" t="s">
+        <v>742</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A83" s="20" t="s">
+        <v>743</v>
+      </c>
+      <c r="B83" s="20" t="s">
+        <v>367</v>
+      </c>
+      <c r="C83" s="20" t="s">
+        <v>744</v>
+      </c>
+      <c r="D83" s="16" t="s">
+        <v>745</v>
+      </c>
+      <c r="E83" s="20" t="s">
+        <v>445</v>
+      </c>
+      <c r="F83" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G83" s="16" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A84" s="20" t="s">
+        <v>747</v>
+      </c>
+      <c r="B84" s="20" t="s">
         <v>351</v>
       </c>
-      <c r="C75" s="19" t="s">
-        <v>677</v>
-      </c>
-      <c r="D75" s="16" t="s">
-        <v>678</v>
-      </c>
-      <c r="E75" s="19" t="s">
-        <v>402</v>
-      </c>
-      <c r="F75" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G75" s="16" t="s">
-        <v>679</v>
-      </c>
-    </row>
-    <row r="76" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A76" s="19" t="s">
-        <v>680</v>
-      </c>
-      <c r="B76" s="19" t="s">
-        <v>351</v>
-      </c>
-      <c r="C76" s="19" t="s">
-        <v>681</v>
-      </c>
-      <c r="D76" s="16" t="s">
-        <v>682</v>
-      </c>
-      <c r="E76" s="19" t="s">
-        <v>402</v>
-      </c>
-      <c r="F76" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G76" s="16" t="s">
-        <v>683</v>
-      </c>
-    </row>
-    <row r="77" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A77" s="19" t="s">
-        <v>684</v>
-      </c>
-      <c r="B77" s="19" t="s">
-        <v>351</v>
-      </c>
-      <c r="C77" s="19" t="s">
-        <v>685</v>
-      </c>
-      <c r="D77" s="16" t="s">
-        <v>686</v>
-      </c>
-      <c r="E77" s="19" t="s">
-        <v>414</v>
-      </c>
-      <c r="F77" s="19" t="s">
-        <v>519</v>
-      </c>
-      <c r="G77" s="16" t="s">
-        <v>687</v>
-      </c>
-    </row>
-    <row r="78" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A78" s="19" t="s">
-        <v>688</v>
-      </c>
-      <c r="B78" s="19" t="s">
-        <v>689</v>
-      </c>
-      <c r="C78" s="19" t="s">
-        <v>690</v>
-      </c>
-      <c r="D78" s="16" t="s">
-        <v>691</v>
-      </c>
-      <c r="E78" s="19" t="s">
-        <v>414</v>
-      </c>
-      <c r="F78" s="19" t="s">
-        <v>519</v>
-      </c>
-      <c r="G78" s="16" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="79" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A79" s="19" t="s">
-        <v>693</v>
-      </c>
-      <c r="B79" s="19" t="s">
-        <v>689</v>
-      </c>
-      <c r="C79" s="19" t="s">
-        <v>694</v>
-      </c>
-      <c r="D79" s="16" t="s">
-        <v>695</v>
-      </c>
-      <c r="E79" s="19" t="s">
-        <v>414</v>
-      </c>
-      <c r="F79" s="19" t="s">
-        <v>519</v>
-      </c>
-      <c r="G79" s="16" t="s">
-        <v>696</v>
-      </c>
-    </row>
-    <row r="80" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A80" s="19" t="s">
-        <v>697</v>
-      </c>
-      <c r="B80" s="19" t="s">
+      <c r="C84" s="20" t="s">
+        <v>748</v>
+      </c>
+      <c r="D84" s="16" t="s">
+        <v>749</v>
+      </c>
+      <c r="E84" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="F84" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G84" s="16" t="s">
+        <v>750</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A85" s="20" t="s">
+        <v>751</v>
+      </c>
+      <c r="B85" s="20" t="s">
+        <v>323</v>
+      </c>
+      <c r="C85" s="20" t="s">
+        <v>752</v>
+      </c>
+      <c r="D85" s="16" t="s">
+        <v>753</v>
+      </c>
+      <c r="E85" s="20" t="s">
+        <v>436</v>
+      </c>
+      <c r="F85" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G85" s="16" t="s">
+        <v>754</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A86" s="20" t="s">
+        <v>755</v>
+      </c>
+      <c r="B86" s="20" t="s">
+        <v>323</v>
+      </c>
+      <c r="C86" s="20" t="s">
+        <v>756</v>
+      </c>
+      <c r="D86" s="16" t="s">
+        <v>757</v>
+      </c>
+      <c r="E86" s="20" t="s">
+        <v>445</v>
+      </c>
+      <c r="F86" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G86" s="16" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A87" s="20" t="s">
+        <v>759</v>
+      </c>
+      <c r="B87" s="20" t="s">
+        <v>375</v>
+      </c>
+      <c r="C87" s="20" t="s">
+        <v>760</v>
+      </c>
+      <c r="D87" s="16" t="s">
+        <v>761</v>
+      </c>
+      <c r="E87" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="F87" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G87" s="16" t="s">
+        <v>762</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A88" s="20" t="s">
+        <v>763</v>
+      </c>
+      <c r="B88" s="20" t="s">
         <v>379</v>
       </c>
-      <c r="C80" s="19" t="s">
-        <v>698</v>
-      </c>
-      <c r="D80" s="16" t="s">
-        <v>699</v>
-      </c>
-      <c r="E80" s="19" t="s">
-        <v>414</v>
-      </c>
-      <c r="F80" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G80" s="16" t="s">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="81" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A81" s="19" t="s">
-        <v>701</v>
-      </c>
-      <c r="B81" s="19" t="s">
+      <c r="C88" s="20" t="s">
+        <v>764</v>
+      </c>
+      <c r="D88" s="16" t="s">
+        <v>765</v>
+      </c>
+      <c r="E88" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="F88" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G88" s="16" t="s">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A89" s="20" t="s">
+        <v>767</v>
+      </c>
+      <c r="B89" s="20" t="s">
+        <v>331</v>
+      </c>
+      <c r="C89" s="20" t="s">
+        <v>768</v>
+      </c>
+      <c r="D89" s="16" t="s">
+        <v>769</v>
+      </c>
+      <c r="E89" s="20" t="s">
+        <v>445</v>
+      </c>
+      <c r="F89" s="20" t="s">
+        <v>553</v>
+      </c>
+      <c r="G89" s="16" t="s">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A90" s="20" t="s">
+        <v>771</v>
+      </c>
+      <c r="B90" s="20" t="s">
+        <v>279</v>
+      </c>
+      <c r="C90" s="20" t="s">
+        <v>772</v>
+      </c>
+      <c r="D90" s="16" t="s">
+        <v>773</v>
+      </c>
+      <c r="E90" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="F90" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G90" s="16" t="s">
+        <v>774</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A91" s="20" t="s">
+        <v>775</v>
+      </c>
+      <c r="B91" s="20" t="s">
+        <v>279</v>
+      </c>
+      <c r="C91" s="20" t="s">
+        <v>772</v>
+      </c>
+      <c r="D91" s="16" t="s">
+        <v>776</v>
+      </c>
+      <c r="E91" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="F91" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G91" s="16" t="s">
+        <v>777</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A92" s="20" t="s">
+        <v>778</v>
+      </c>
+      <c r="B92" s="20" t="s">
+        <v>291</v>
+      </c>
+      <c r="C92" s="20" t="s">
+        <v>779</v>
+      </c>
+      <c r="D92" s="16" t="s">
+        <v>780</v>
+      </c>
+      <c r="E92" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="F92" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G92" s="16" t="s">
+        <v>781</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A93" s="20" t="s">
+        <v>782</v>
+      </c>
+      <c r="B93" s="20" t="s">
+        <v>299</v>
+      </c>
+      <c r="C93" s="20" t="s">
+        <v>783</v>
+      </c>
+      <c r="D93" s="16" t="s">
+        <v>784</v>
+      </c>
+      <c r="E93" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="F93" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G93" s="16" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="157.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A94" s="20" t="s">
+        <v>786</v>
+      </c>
+      <c r="B94" s="20" t="s">
+        <v>291</v>
+      </c>
+      <c r="C94" s="20" t="s">
+        <v>787</v>
+      </c>
+      <c r="D94" s="16" t="s">
+        <v>788</v>
+      </c>
+      <c r="E94" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="F94" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G94" s="16" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A95" s="20" t="s">
+        <v>790</v>
+      </c>
+      <c r="B95" s="20" t="s">
         <v>371</v>
       </c>
-      <c r="C81" s="19" t="s">
-        <v>702</v>
-      </c>
-      <c r="D81" s="16" t="s">
-        <v>703</v>
-      </c>
-      <c r="E81" s="19" t="s">
-        <v>414</v>
-      </c>
-      <c r="F81" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G81" s="16" t="s">
-        <v>704</v>
-      </c>
-    </row>
-    <row r="82" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A82" s="19" t="s">
-        <v>705</v>
-      </c>
-      <c r="B82" s="19" t="s">
-        <v>367</v>
-      </c>
-      <c r="C82" s="19" t="s">
-        <v>706</v>
-      </c>
-      <c r="D82" s="16" t="s">
-        <v>707</v>
-      </c>
-      <c r="E82" s="19" t="s">
-        <v>414</v>
-      </c>
-      <c r="F82" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G82" s="16" t="s">
-        <v>708</v>
-      </c>
-    </row>
-    <row r="83" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A83" s="19" t="s">
-        <v>709</v>
-      </c>
-      <c r="B83" s="19" t="s">
-        <v>367</v>
-      </c>
-      <c r="C83" s="19" t="s">
-        <v>710</v>
-      </c>
-      <c r="D83" s="16" t="s">
-        <v>711</v>
-      </c>
-      <c r="E83" s="19" t="s">
-        <v>411</v>
-      </c>
-      <c r="F83" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G83" s="16" t="s">
-        <v>712</v>
-      </c>
-    </row>
-    <row r="84" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A84" s="19" t="s">
-        <v>713</v>
-      </c>
-      <c r="B84" s="19" t="s">
-        <v>351</v>
-      </c>
-      <c r="C84" s="19" t="s">
-        <v>714</v>
-      </c>
-      <c r="D84" s="16" t="s">
-        <v>715</v>
-      </c>
-      <c r="E84" s="19" t="s">
-        <v>414</v>
-      </c>
-      <c r="F84" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G84" s="16" t="s">
-        <v>716</v>
-      </c>
-    </row>
-    <row r="85" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A85" s="19" t="s">
-        <v>717</v>
-      </c>
-      <c r="B85" s="19" t="s">
-        <v>323</v>
-      </c>
-      <c r="C85" s="19" t="s">
-        <v>718</v>
-      </c>
-      <c r="D85" s="16" t="s">
-        <v>719</v>
-      </c>
-      <c r="E85" s="19" t="s">
-        <v>402</v>
-      </c>
-      <c r="F85" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G85" s="16" t="s">
-        <v>720</v>
-      </c>
-    </row>
-    <row r="86" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A86" s="19" t="s">
-        <v>721</v>
-      </c>
-      <c r="B86" s="19" t="s">
-        <v>323</v>
-      </c>
-      <c r="C86" s="19" t="s">
-        <v>722</v>
-      </c>
-      <c r="D86" s="16" t="s">
-        <v>723</v>
-      </c>
-      <c r="E86" s="19" t="s">
-        <v>411</v>
-      </c>
-      <c r="F86" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G86" s="16" t="s">
-        <v>724</v>
-      </c>
-    </row>
-    <row r="87" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A87" s="19" t="s">
-        <v>725</v>
-      </c>
-      <c r="B87" s="19" t="s">
-        <v>375</v>
-      </c>
-      <c r="C87" s="19" t="s">
-        <v>726</v>
-      </c>
-      <c r="D87" s="16" t="s">
-        <v>727</v>
-      </c>
-      <c r="E87" s="19" t="s">
-        <v>414</v>
-      </c>
-      <c r="F87" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="G87" s="16" t="s">
-        <v>728</v>
-      </c>
-    </row>
-    <row r="88" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A88" s="19" t="s">
-        <v>729</v>
-      </c>
-      <c r="B88" s="19" t="s">
-        <v>379</v>
-      </c>
-      <c r="C88" s="19" t="s">
-        <v>730</v>
-      </c>
-      <c r="D88" s="16" t="s">
-        <v>731</v>
-      </c>
-      <c r="E88" s="19" t="s">
-        <v>414</v>
-      </c>
-      <c r="F88" s="19" t="s">
-        <v>519</v>
-      </c>
-      <c r="G88" s="16" t="s">
-        <v>732</v>
-      </c>
-    </row>
-    <row r="89" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A89" s="19" t="s">
-        <v>733</v>
-      </c>
-      <c r="B89" s="19" t="s">
-        <v>331</v>
-      </c>
-      <c r="C89" s="19" t="s">
-        <v>734</v>
-      </c>
-      <c r="D89" s="16" t="s">
-        <v>735</v>
-      </c>
-      <c r="E89" s="19" t="s">
-        <v>411</v>
-      </c>
-      <c r="F89" s="19" t="s">
-        <v>519</v>
-      </c>
-      <c r="G89" s="16" t="s">
-        <v>736</v>
+      <c r="C95" s="20" t="s">
+        <v>791</v>
+      </c>
+      <c r="D95" s="16" t="s">
+        <v>792</v>
+      </c>
+      <c r="E95" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="F95" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="G95" s="16" t="s">
+        <v>793</v>
       </c>
     </row>
   </sheetData>
@@ -7600,12 +8120,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>737</v>
+        <v>794</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>738</v>
+        <v>795</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7613,16 +8133,16 @@
         <v>19</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>739</v>
+        <v>796</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>740</v>
+        <v>797</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>741</v>
+        <v>798</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>742</v>
+        <v>799</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>22</v>
@@ -7630,382 +8150,382 @@
     </row>
     <row r="5" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>743</v>
+        <v>800</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>744</v>
+        <v>801</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>745</v>
+        <v>802</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>746</v>
+        <v>803</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>747</v>
+        <v>804</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>519</v>
+        <v>553</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>748</v>
+        <v>805</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>749</v>
+        <v>806</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>750</v>
+        <v>807</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>751</v>
+        <v>808</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>752</v>
+        <v>809</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>753</v>
+        <v>810</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>754</v>
+        <v>811</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>755</v>
+        <v>812</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>756</v>
+        <v>813</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>757</v>
+        <v>814</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>758</v>
+        <v>815</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>458</v>
+        <v>492</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>759</v>
+        <v>816</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>760</v>
+        <v>817</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>761</v>
+        <v>818</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>762</v>
+        <v>819</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>763</v>
+        <v>820</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>458</v>
+        <v>492</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>764</v>
+        <v>821</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>765</v>
+        <v>822</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>766</v>
+        <v>823</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>767</v>
+        <v>824</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>768</v>
+        <v>825</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>519</v>
+        <v>553</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>769</v>
+        <v>826</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>765</v>
+        <v>822</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>770</v>
+        <v>827</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>771</v>
+        <v>828</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>772</v>
+        <v>829</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>519</v>
+        <v>553</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>773</v>
+        <v>830</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>774</v>
+        <v>831</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>775</v>
+        <v>832</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>776</v>
+        <v>833</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>777</v>
+        <v>834</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>753</v>
+        <v>810</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>778</v>
+        <v>835</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>779</v>
+        <v>836</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>780</v>
+        <v>837</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>781</v>
+        <v>838</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>782</v>
+        <v>839</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>519</v>
+        <v>553</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="19" t="s">
-        <v>783</v>
-      </c>
-      <c r="B13" s="19" t="s">
-        <v>774</v>
+      <c r="A13" s="20" t="s">
+        <v>840</v>
+      </c>
+      <c r="B13" s="20" t="s">
+        <v>831</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>784</v>
+        <v>841</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>785</v>
-      </c>
-      <c r="E13" s="19" t="s">
-        <v>786</v>
-      </c>
-      <c r="F13" s="19" t="s">
-        <v>519</v>
+        <v>842</v>
+      </c>
+      <c r="E13" s="20" t="s">
+        <v>843</v>
+      </c>
+      <c r="F13" s="20" t="s">
+        <v>553</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="19" t="s">
-        <v>787</v>
-      </c>
-      <c r="B14" s="19" t="s">
-        <v>779</v>
+      <c r="A14" s="20" t="s">
+        <v>844</v>
+      </c>
+      <c r="B14" s="20" t="s">
+        <v>836</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>788</v>
+        <v>845</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>789</v>
-      </c>
-      <c r="E14" s="19" t="s">
-        <v>790</v>
-      </c>
-      <c r="F14" s="19" t="s">
-        <v>519</v>
+        <v>846</v>
+      </c>
+      <c r="E14" s="20" t="s">
+        <v>847</v>
+      </c>
+      <c r="F14" s="20" t="s">
+        <v>553</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="19" t="s">
-        <v>791</v>
-      </c>
-      <c r="B15" s="19" t="s">
-        <v>792</v>
+      <c r="A15" s="20" t="s">
+        <v>848</v>
+      </c>
+      <c r="B15" s="20" t="s">
+        <v>849</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>793</v>
+        <v>850</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>794</v>
-      </c>
-      <c r="E15" s="19" t="s">
-        <v>795</v>
-      </c>
-      <c r="F15" s="19" t="s">
-        <v>519</v>
+        <v>851</v>
+      </c>
+      <c r="E15" s="20" t="s">
+        <v>852</v>
+      </c>
+      <c r="F15" s="20" t="s">
+        <v>553</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="19" t="s">
-        <v>796</v>
-      </c>
-      <c r="B16" s="19" t="s">
-        <v>744</v>
+      <c r="A16" s="20" t="s">
+        <v>853</v>
+      </c>
+      <c r="B16" s="20" t="s">
+        <v>801</v>
       </c>
       <c r="C16" s="16" t="s">
-        <v>797</v>
+        <v>854</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>798</v>
-      </c>
-      <c r="E16" s="19" t="s">
-        <v>799</v>
-      </c>
-      <c r="F16" s="19" t="s">
-        <v>519</v>
+        <v>855</v>
+      </c>
+      <c r="E16" s="20" t="s">
+        <v>856</v>
+      </c>
+      <c r="F16" s="20" t="s">
+        <v>553</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="19" t="s">
-        <v>800</v>
-      </c>
-      <c r="B17" s="19" t="s">
-        <v>765</v>
+      <c r="A17" s="20" t="s">
+        <v>857</v>
+      </c>
+      <c r="B17" s="20" t="s">
+        <v>822</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>801</v>
+        <v>858</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>802</v>
-      </c>
-      <c r="E17" s="19" t="s">
-        <v>803</v>
-      </c>
-      <c r="F17" s="19" t="s">
-        <v>519</v>
+        <v>859</v>
+      </c>
+      <c r="E17" s="20" t="s">
+        <v>860</v>
+      </c>
+      <c r="F17" s="20" t="s">
+        <v>553</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="19" t="s">
-        <v>804</v>
-      </c>
-      <c r="B18" s="19" t="s">
-        <v>774</v>
+      <c r="A18" s="20" t="s">
+        <v>861</v>
+      </c>
+      <c r="B18" s="20" t="s">
+        <v>831</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>805</v>
+        <v>862</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>806</v>
-      </c>
-      <c r="E18" s="19" t="s">
-        <v>807</v>
-      </c>
-      <c r="F18" s="19" t="s">
-        <v>519</v>
+        <v>863</v>
+      </c>
+      <c r="E18" s="20" t="s">
+        <v>864</v>
+      </c>
+      <c r="F18" s="20" t="s">
+        <v>553</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="19" t="s">
-        <v>808</v>
-      </c>
-      <c r="B19" s="19" t="s">
-        <v>809</v>
+      <c r="A19" s="20" t="s">
+        <v>865</v>
+      </c>
+      <c r="B19" s="20" t="s">
+        <v>866</v>
       </c>
       <c r="C19" s="16" t="s">
+        <v>867</v>
+      </c>
+      <c r="D19" s="16" t="s">
+        <v>868</v>
+      </c>
+      <c r="E19" s="20" t="s">
+        <v>869</v>
+      </c>
+      <c r="F19" s="20" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="20" t="s">
+        <v>870</v>
+      </c>
+      <c r="B20" s="20" t="s">
+        <v>871</v>
+      </c>
+      <c r="C20" s="16" t="s">
+        <v>872</v>
+      </c>
+      <c r="D20" s="16" t="s">
+        <v>873</v>
+      </c>
+      <c r="E20" s="20" t="s">
+        <v>874</v>
+      </c>
+      <c r="F20" s="20" t="s">
         <v>810</v>
       </c>
-      <c r="D19" s="16" t="s">
-        <v>811</v>
-      </c>
-      <c r="E19" s="19" t="s">
-        <v>812</v>
-      </c>
-      <c r="F19" s="19" t="s">
-        <v>519</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="19" t="s">
-        <v>813</v>
-      </c>
-      <c r="B20" s="19" t="s">
-        <v>814</v>
-      </c>
-      <c r="C20" s="16" t="s">
-        <v>815</v>
-      </c>
-      <c r="D20" s="16" t="s">
-        <v>816</v>
-      </c>
-      <c r="E20" s="19" t="s">
-        <v>817</v>
-      </c>
-      <c r="F20" s="19" t="s">
-        <v>753</v>
-      </c>
     </row>
     <row r="21" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="19" t="s">
-        <v>818</v>
-      </c>
-      <c r="B21" s="19" t="s">
-        <v>819</v>
+      <c r="A21" s="20" t="s">
+        <v>875</v>
+      </c>
+      <c r="B21" s="20" t="s">
+        <v>876</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>820</v>
+        <v>877</v>
       </c>
       <c r="D21" s="16" t="s">
-        <v>821</v>
-      </c>
-      <c r="E21" s="19" t="s">
-        <v>822</v>
-      </c>
-      <c r="F21" s="19" t="s">
-        <v>458</v>
+        <v>878</v>
+      </c>
+      <c r="E21" s="20" t="s">
+        <v>879</v>
+      </c>
+      <c r="F21" s="20" t="s">
+        <v>492</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="19" t="s">
-        <v>823</v>
-      </c>
-      <c r="B22" s="19" t="s">
-        <v>824</v>
+      <c r="A22" s="20" t="s">
+        <v>880</v>
+      </c>
+      <c r="B22" s="20" t="s">
+        <v>881</v>
       </c>
       <c r="C22" s="16" t="s">
-        <v>825</v>
+        <v>882</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>826</v>
-      </c>
-      <c r="E22" s="19" t="s">
-        <v>827</v>
-      </c>
-      <c r="F22" s="19" t="s">
-        <v>519</v>
+        <v>883</v>
+      </c>
+      <c r="E22" s="20" t="s">
+        <v>884</v>
+      </c>
+      <c r="F22" s="20" t="s">
+        <v>553</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="19" t="s">
-        <v>828</v>
-      </c>
-      <c r="B23" s="19" t="s">
-        <v>829</v>
+      <c r="A23" s="20" t="s">
+        <v>885</v>
+      </c>
+      <c r="B23" s="20" t="s">
+        <v>886</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>830</v>
+        <v>887</v>
       </c>
       <c r="D23" s="16" t="s">
-        <v>831</v>
-      </c>
-      <c r="E23" s="19" t="s">
-        <v>832</v>
-      </c>
-      <c r="F23" s="19" t="s">
-        <v>519</v>
+        <v>888</v>
+      </c>
+      <c r="E23" s="20" t="s">
+        <v>889</v>
+      </c>
+      <c r="F23" s="20" t="s">
+        <v>553</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Flyway owns the schema; rule 4 and database-level double-booking constraints
0.7 - Flyway with a pg_dump baseline at V1 and ddl-auto=validate. Hibernate now verifies the schema instead of mutating it, and passed against the live database first try. Env-driven via FLYWAY_ENABLED / DDL_AUTO so the rollback is two lines in .env.

Boot 4 note: flyway-core alone does nothing. Auto-configuration is modular now, so FlywayAutoConfiguration ships with spring-boot-starter-flyway. Without it every spring.flyway.* property is inert and the app starts perfectly without migrating.

2.36 - rule 4, a client cannot be in two rooms at once. The 409 now carries its own reason on both the REST and chat paths.

2.37 - V2 adds EXCLUDE USING gist constraints per therapist and per room, partial on blocking statuses. assign() cannot be atomic against a concurrent transaction; this is where the guarantee actually lives.

33 tests, 0 failures.
</commit_message>
<xml_diff>
--- a/HilotSpa_ThesisTracker.xlsx
+++ b/HilotSpa_ThesisTracker.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1495" uniqueCount="902">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1502" uniqueCount="906">
   <si>
     <t xml:space="preserve">HilotSpa — Progress Summary</t>
   </si>
@@ -194,7 +194,7 @@
     <t xml:space="preserve">Flyway so every node shares an identical schema. Redis into pom.xml + compose.yaml.</t>
   </si>
   <si>
-    <t xml:space="preserve">Secrets/.env done. Flyway NOT started, Redis deferred to Sprint 2. ddl-auto=update is still what builds the schema.</t>
+    <t xml:space="preserve">Closed 2026-08-30. Flyway owns the schema; Hibernate switched to ddl-auto=validate and PASSED against the live database on the first try, which also proves the V1 baseline dump is accurate. V1 is a pg_dump of the schema as ddl-auto left it (three lines stripped: \restrict / \unrestrict psql meta-commands that pg_dump 15.18 emits and JDBC cannot parse, and the search_path reset that would have broken Flyway's own INSERT into flyway_schema_history). Both settings are env-driven - FLYWAY_ENABLED / DDL_AUTO - so the rollback is deleting two lines from .env, no rebuild. THE TRAP: on Spring Boot 4, flyway-core alone is NOT enough. Boot 4 split auto-configuration into one module per technology, so FlywayAutoConfiguration ships with spring-boot-starter-flyway. With only flyway-core the library is present, the auto-configuration is not, and every spring.flyway.* property is an inert string - no error, no warning, no log line, the app starts perfectly and never migrates. Cost about 40 minutes of chasing a stale Docker image that was not stale.</t>
   </si>
   <si>
     <t xml:space="preserve">0.8</t>
@@ -1271,7 +1271,7 @@
     <t xml:space="preserve">book() only guards against an identical repeat (same service, same minute). Nothing stops one client holding a 9:00 Signature and a 9:00 Ventosa - different therapist, different room, one person in two places.</t>
   </si>
   <si>
-    <t xml:space="preserve">Found 2026-08-30 while auditing the booking rules with Liodoq. He is brainstorming the rule set with his partner before this is built. Small fix; a panelist can find it by accident.</t>
+    <t xml:space="preserve">Built 2026-08-30. Rule 4 - a client cannot be in two rooms at once. The spa's three stated rules are all about the SPA's resources; none of them looks at the client, and the idempotency guard only caught an identical repeat, so one person could hold a 9:00 Signature and a 9:00 Ventosa with every rule satisfied. The 409 carries its own reason now instead of being flattened into 'that time was just taken', on both the REST and the chat paths - the slot going to someone else and the client being busy need different things done about them. 2 tests: one asserts the MESSAGE, because Bulan has a spare pair at that minute so a bare 409 could equally mean exhaustion; the other proves the rule blocks the CLIENT, not the slot.</t>
   </si>
   <si>
     <t xml:space="preserve">2.37</t>
@@ -1283,7 +1283,7 @@
     <t xml:space="preserve">EXCLUDE USING gist (therapist_id WITH =, tsrange(start_time,end_time) WITH &amp;&amp;) WHERE status IN (PENDING,CONFIRMED,IN_PROGRESS), plus the same for room_id. Needs btree_gist.</t>
   </si>
   <si>
-    <t xml:space="preserve">assign() is check-then-save: two transactions can both pass the existence check and both write. The tests are sequential so they do not catch it. This also turns single-writer-per-partition from an assertion into a mechanism - a therapist belongs to one branch, so one node writes them, so a LOCAL constraint is sufficient and no consensus algorithm is needed. Strong Sprint 3 defence material.</t>
+    <t xml:space="preserve">Built 2026-08-30 as Flyway migration V2. EXCLUDE USING gist on (therapist_id, tsrange(start_time,end_time)) and the same for room_id, partial on PENDING/CONFIRMED/IN_PROGRESS so cancelled rows release the hour, half-open ranges matching the application's own rule. assign() cannot be atomic against a concurrent transaction under READ COMMITTED - two requests milliseconds apart can both pass the check and both insert, and every test we have runs sequentially so none could catch it. writeOrConflict() uses saveAndFlush and translates the database's veto into a 409 rather than a 500, because JPA is free to defer the INSERT to commit where the catch block is out of scope. This also turns single-writer-per-partition from a claim in the paper into a constraint a panelist can read: a therapist belongs to one branch, so one node writes them, so a LOCAL constraint is sufficient and no consensus is required.</t>
   </si>
   <si>
     <t xml:space="preserve">2.38</t>
@@ -1350,6 +1350,18 @@
   </si>
   <si>
     <t xml:space="preserve">Built 2026-08-30. No manual SQL needed - ddl-auto=update creates a new table and adds a nullable column happily. The assistant used to be told only noted_on_record:true because a claim parsed out of prose is a guess, and guessing about pregnancy is not something this system should do; it now receives the flags the client actually ticked. pressurePreference was hardcoded null in the prompt and is now real. Flags deliberately do NOT filter the service list - that stays with the practitioner-signed ServiceProtocol table until she authors a rule (4.13). Review screen and session report read the enum back in the client wording. 1 new round-trip test.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flyway migration discipline documented</t>
+  </si>
+  <si>
+    <t xml:space="preserve">db/migration/README.md - never edit an applied migration, one concern per file, every entity change ships its migration in the same commit, migrations must be safe on a populated database.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Written 2026-08-30 alongside 0.7. The rules exist because ddl-auto=validate now fails the boot when an entity and the migrations disagree - which is the point, but only helps if the next person knows why.</t>
   </si>
   <si>
     <t xml:space="preserve">HilotSpa — Bug &amp; Finding Log</t>
@@ -3401,28 +3413,28 @@
         <v>9</v>
       </c>
       <c r="B5" s="6" t="n">
-        <f aca="false">COUNTIF(Tasks!$A$5:$A$109,$A5)</f>
-        <v>18</v>
+        <f aca="false">COUNTIF(Tasks!$A$5:$A$110,$A5)</f>
+        <v>19</v>
       </c>
       <c r="C5" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$109,$A5,Tasks!$E$5:$E$109,"Done")</f>
-        <v>15</v>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A5,Tasks!$E$5:$E$110,"Done")</f>
+        <v>17</v>
       </c>
       <c r="D5" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$109,$A5,Tasks!$E$5:$E$109,"In Progress")</f>
-        <v>1</v>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A5,Tasks!$E$5:$E$110,"In Progress")</f>
+        <v>0</v>
       </c>
       <c r="E5" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$109,$A5,Tasks!$E$5:$E$109,"Not Started")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A5,Tasks!$E$5:$E$110,"Not Started")</f>
         <v>2</v>
       </c>
       <c r="F5" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$109,$A5,Tasks!$E$5:$E$109,"Blocked")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A5,Tasks!$E$5:$E$110,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G5" s="7" t="n">
         <f aca="false">IFERROR($C5/$B5,0)</f>
-        <v>0.833333333333333</v>
+        <v>0.894736842105263</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3430,23 +3442,23 @@
         <v>10</v>
       </c>
       <c r="B6" s="6" t="n">
-        <f aca="false">COUNTIF(Tasks!$A$5:$A$109,$A6)</f>
+        <f aca="false">COUNTIF(Tasks!$A$5:$A$110,$A6)</f>
         <v>20</v>
       </c>
       <c r="C6" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$109,$A6,Tasks!$E$5:$E$109,"Done")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A6,Tasks!$E$5:$E$110,"Done")</f>
         <v>20</v>
       </c>
       <c r="D6" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$109,$A6,Tasks!$E$5:$E$109,"In Progress")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A6,Tasks!$E$5:$E$110,"In Progress")</f>
         <v>0</v>
       </c>
       <c r="E6" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$109,$A6,Tasks!$E$5:$E$109,"Not Started")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A6,Tasks!$E$5:$E$110,"Not Started")</f>
         <v>0</v>
       </c>
       <c r="F6" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$109,$A6,Tasks!$E$5:$E$109,"Blocked")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A6,Tasks!$E$5:$E$110,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G6" s="7" t="n">
@@ -3459,28 +3471,28 @@
         <v>11</v>
       </c>
       <c r="B7" s="6" t="n">
-        <f aca="false">COUNTIF(Tasks!$A$5:$A$109,$A7)</f>
+        <f aca="false">COUNTIF(Tasks!$A$5:$A$110,$A7)</f>
         <v>39</v>
       </c>
       <c r="C7" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$109,$A7,Tasks!$E$5:$E$109,"Done")</f>
-        <v>32</v>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A7,Tasks!$E$5:$E$110,"Done")</f>
+        <v>34</v>
       </c>
       <c r="D7" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$109,$A7,Tasks!$E$5:$E$109,"In Progress")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A7,Tasks!$E$5:$E$110,"In Progress")</f>
         <v>3</v>
       </c>
       <c r="E7" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$109,$A7,Tasks!$E$5:$E$109,"Not Started")</f>
-        <v>4</v>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A7,Tasks!$E$5:$E$110,"Not Started")</f>
+        <v>2</v>
       </c>
       <c r="F7" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$109,$A7,Tasks!$E$5:$E$109,"Blocked")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A7,Tasks!$E$5:$E$110,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G7" s="7" t="n">
         <f aca="false">IFERROR($C7/$B7,0)</f>
-        <v>0.820512820512821</v>
+        <v>0.871794871794872</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3488,23 +3500,23 @@
         <v>12</v>
       </c>
       <c r="B8" s="6" t="n">
-        <f aca="false">COUNTIF(Tasks!$A$5:$A$109,$A8)</f>
+        <f aca="false">COUNTIF(Tasks!$A$5:$A$110,$A8)</f>
         <v>15</v>
       </c>
       <c r="C8" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$109,$A8,Tasks!$E$5:$E$109,"Done")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A8,Tasks!$E$5:$E$110,"Done")</f>
         <v>4</v>
       </c>
       <c r="D8" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$109,$A8,Tasks!$E$5:$E$109,"In Progress")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A8,Tasks!$E$5:$E$110,"In Progress")</f>
         <v>5</v>
       </c>
       <c r="E8" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$109,$A8,Tasks!$E$5:$E$109,"Not Started")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A8,Tasks!$E$5:$E$110,"Not Started")</f>
         <v>6</v>
       </c>
       <c r="F8" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$109,$A8,Tasks!$E$5:$E$109,"Blocked")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A8,Tasks!$E$5:$E$110,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G8" s="7" t="n">
@@ -3517,23 +3529,23 @@
         <v>13</v>
       </c>
       <c r="B9" s="6" t="n">
-        <f aca="false">COUNTIF(Tasks!$A$5:$A$109,$A9)</f>
+        <f aca="false">COUNTIF(Tasks!$A$5:$A$110,$A9)</f>
         <v>13</v>
       </c>
       <c r="C9" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$109,$A9,Tasks!$E$5:$E$109,"Done")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A9,Tasks!$E$5:$E$110,"Done")</f>
         <v>1</v>
       </c>
       <c r="D9" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$109,$A9,Tasks!$E$5:$E$109,"In Progress")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A9,Tasks!$E$5:$E$110,"In Progress")</f>
         <v>1</v>
       </c>
       <c r="E9" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$109,$A9,Tasks!$E$5:$E$109,"Not Started")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A9,Tasks!$E$5:$E$110,"Not Started")</f>
         <v>11</v>
       </c>
       <c r="F9" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$109,$A9,Tasks!$E$5:$E$109,"Blocked")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A9,Tasks!$E$5:$E$110,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G9" s="7" t="n">
@@ -3547,19 +3559,19 @@
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">SUM(B5:B9)</f>
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C10" s="9" t="n">
         <f aca="false">SUM(C5:C9)</f>
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D10" s="9" t="n">
         <f aca="false">SUM(D5:D9)</f>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E10" s="9" t="n">
         <f aca="false">SUM(E5:E9)</f>
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F10" s="9" t="n">
         <f aca="false">SUM(F5:F9)</f>
@@ -3567,7 +3579,7 @@
       </c>
       <c r="G10" s="10" t="n">
         <f aca="false">IFERROR($C10/$B10,0)</f>
-        <v>0.685714285714286</v>
+        <v>0.716981132075472</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3604,7 +3616,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G109"/>
+  <dimension ref="A1:G110"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11"/>
@@ -3801,7 +3813,7 @@
         <v>54</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F11" s="6" t="s">
         <v>37</v>
@@ -5820,7 +5832,7 @@
         <v>413</v>
       </c>
       <c r="E102" s="20" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F102" s="20" t="s">
         <v>28</v>
@@ -5843,7 +5855,7 @@
         <v>417</v>
       </c>
       <c r="E103" s="20" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F103" s="20" t="s">
         <v>28</v>
@@ -5921,7 +5933,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="107" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="107" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A107" s="19" t="s">
         <v>10</v>
       </c>
@@ -5944,7 +5956,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="108" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="108" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A108" s="19" t="s">
         <v>10</v>
       </c>
@@ -5967,7 +5979,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="109" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="109" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A109" s="19" t="s">
         <v>10</v>
       </c>
@@ -5988,6 +6000,29 @@
       </c>
       <c r="G109" s="16" t="s">
         <v>440</v>
+      </c>
+    </row>
+    <row r="110" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="B110" s="20" t="s">
+        <v>441</v>
+      </c>
+      <c r="C110" s="16" t="s">
+        <v>442</v>
+      </c>
+      <c r="D110" s="16" t="s">
+        <v>443</v>
+      </c>
+      <c r="E110" s="20" t="s">
+        <v>4</v>
+      </c>
+      <c r="F110" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="G110" s="16" t="s">
+        <v>444</v>
       </c>
     </row>
   </sheetData>
@@ -6039,7 +6074,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>441</v>
+        <v>445</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6050,13 +6085,13 @@
         <v>20</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>442</v>
+        <v>446</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>443</v>
+        <v>447</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>444</v>
+        <v>448</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>22</v>
@@ -6067,2112 +6102,2112 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>445</v>
+        <v>449</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>25</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G4" s="16" t="s">
-        <v>450</v>
+        <v>454</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>451</v>
+        <v>455</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>25</v>
       </c>
       <c r="C5" s="16" t="s">
+        <v>456</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>457</v>
+      </c>
+      <c r="E5" s="6" t="s">
         <v>452</v>
       </c>
-      <c r="D5" s="16" t="s">
+      <c r="F5" s="6" t="s">
         <v>453</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>448</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>449</v>
       </c>
       <c r="G5" s="16"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>454</v>
+        <v>458</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>25</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>456</v>
+        <v>460</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G6" s="16"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>458</v>
+        <v>462</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>25</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>461</v>
+        <v>465</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>25</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>463</v>
+        <v>467</v>
       </c>
       <c r="D8" s="16" t="s">
+        <v>468</v>
+      </c>
+      <c r="E8" s="6" t="s">
         <v>464</v>
       </c>
-      <c r="E8" s="6" t="s">
-        <v>460</v>
-      </c>
       <c r="F8" s="6" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G8" s="16"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>465</v>
+        <v>469</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>30</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>466</v>
+        <v>470</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>467</v>
+        <v>471</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>468</v>
+        <v>472</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>469</v>
+        <v>473</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>30</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>470</v>
+        <v>474</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>471</v>
+        <v>475</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>472</v>
+        <v>476</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>30</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>474</v>
+        <v>478</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>476</v>
+        <v>480</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>30</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>477</v>
+        <v>481</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>478</v>
+        <v>482</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>479</v>
+        <v>483</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>480</v>
+        <v>484</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>30</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>481</v>
+        <v>485</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>482</v>
+        <v>486</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>483</v>
+        <v>487</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>484</v>
+        <v>488</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>30</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>485</v>
+        <v>489</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>486</v>
+        <v>490</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>487</v>
+        <v>491</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>488</v>
+        <v>492</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>489</v>
+        <v>493</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>490</v>
+        <v>494</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>491</v>
+        <v>495</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>492</v>
+        <v>496</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>493</v>
+        <v>497</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>34</v>
       </c>
       <c r="C16" s="16" t="s">
-        <v>494</v>
+        <v>498</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>495</v>
+        <v>499</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>496</v>
+        <v>500</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>497</v>
+        <v>501</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>47</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>498</v>
+        <v>502</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>499</v>
+        <v>503</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G17" s="16" t="s">
-        <v>500</v>
+        <v>504</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>501</v>
+        <v>505</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>52</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>502</v>
+        <v>506</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>503</v>
+        <v>507</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>504</v>
+        <v>508</v>
       </c>
       <c r="G18" s="16" t="s">
-        <v>505</v>
+        <v>509</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>506</v>
+        <v>510</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>489</v>
+        <v>493</v>
       </c>
       <c r="C19" s="16" t="s">
-        <v>507</v>
+        <v>511</v>
       </c>
       <c r="D19" s="16" t="s">
-        <v>508</v>
+        <v>512</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G19" s="16" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B20" s="6" t="s">
         <v>30</v>
       </c>
       <c r="C20" s="16" t="s">
-        <v>511</v>
+        <v>515</v>
       </c>
       <c r="D20" s="16" t="s">
-        <v>512</v>
+        <v>516</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G20" s="16" t="s">
-        <v>513</v>
+        <v>517</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>514</v>
+        <v>518</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>489</v>
+        <v>493</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>511</v>
+        <v>515</v>
       </c>
       <c r="D21" s="16" t="s">
-        <v>515</v>
+        <v>519</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G21" s="16" t="s">
-        <v>516</v>
+        <v>520</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>517</v>
+        <v>521</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>489</v>
+        <v>493</v>
       </c>
       <c r="C22" s="16" t="s">
-        <v>518</v>
+        <v>522</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>519</v>
+        <v>523</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G22" s="16" t="s">
-        <v>520</v>
+        <v>524</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>521</v>
+        <v>525</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>489</v>
+        <v>493</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>522</v>
+        <v>526</v>
       </c>
       <c r="D23" s="16" t="s">
-        <v>523</v>
+        <v>527</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G23" s="16" t="s">
-        <v>524</v>
+        <v>528</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>525</v>
+        <v>529</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>489</v>
+        <v>493</v>
       </c>
       <c r="C24" s="16" t="s">
-        <v>526</v>
+        <v>530</v>
       </c>
       <c r="D24" s="16" t="s">
-        <v>527</v>
+        <v>531</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G24" s="16" t="s">
-        <v>528</v>
+        <v>532</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>529</v>
+        <v>533</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>489</v>
+        <v>493</v>
       </c>
       <c r="C25" s="16" t="s">
-        <v>530</v>
+        <v>534</v>
       </c>
       <c r="D25" s="16" t="s">
-        <v>531</v>
+        <v>535</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G25" s="16" t="s">
-        <v>532</v>
+        <v>536</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>533</v>
+        <v>537</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>489</v>
+        <v>493</v>
       </c>
       <c r="C26" s="16" t="s">
-        <v>534</v>
+        <v>538</v>
       </c>
       <c r="D26" s="16" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G26" s="16" t="s">
-        <v>536</v>
+        <v>540</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>537</v>
+        <v>541</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>489</v>
+        <v>493</v>
       </c>
       <c r="C27" s="16" t="s">
-        <v>538</v>
+        <v>542</v>
       </c>
       <c r="D27" s="16" t="s">
-        <v>539</v>
+        <v>543</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G27" s="16" t="s">
-        <v>540</v>
+        <v>544</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>541</v>
+        <v>545</v>
       </c>
       <c r="B28" s="6" t="s">
         <v>39</v>
       </c>
       <c r="C28" s="16" t="s">
+        <v>456</v>
+      </c>
+      <c r="D28" s="16" t="s">
+        <v>546</v>
+      </c>
+      <c r="E28" s="6" t="s">
         <v>452</v>
       </c>
-      <c r="D28" s="16" t="s">
-        <v>542</v>
-      </c>
-      <c r="E28" s="6" t="s">
-        <v>448</v>
-      </c>
       <c r="F28" s="6" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G28" s="16" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>544</v>
+        <v>548</v>
       </c>
       <c r="B29" s="6" t="s">
         <v>43</v>
       </c>
       <c r="C29" s="16" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
       <c r="D29" s="16" t="s">
-        <v>545</v>
+        <v>549</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G29" s="16" t="s">
-        <v>546</v>
+        <v>550</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>547</v>
+        <v>551</v>
       </c>
       <c r="B30" s="6" t="s">
         <v>43</v>
       </c>
       <c r="C30" s="16" t="s">
-        <v>466</v>
+        <v>470</v>
       </c>
       <c r="D30" s="16" t="s">
-        <v>548</v>
+        <v>552</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G30" s="16" t="s">
-        <v>549</v>
+        <v>553</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>550</v>
+        <v>554</v>
       </c>
       <c r="B31" s="6" t="s">
         <v>47</v>
       </c>
       <c r="C31" s="16" t="s">
-        <v>551</v>
+        <v>555</v>
       </c>
       <c r="D31" s="16" t="s">
-        <v>552</v>
+        <v>556</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G31" s="16" t="s">
-        <v>553</v>
+        <v>557</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>555</v>
+        <v>559</v>
       </c>
       <c r="C32" s="16" t="s">
-        <v>511</v>
+        <v>515</v>
       </c>
       <c r="D32" s="16" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G32" s="16" t="s">
-        <v>557</v>
+        <v>561</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="s">
-        <v>558</v>
+        <v>562</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>555</v>
+        <v>559</v>
       </c>
       <c r="C33" s="16" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
       <c r="D33" s="16" t="s">
-        <v>560</v>
+        <v>564</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G33" s="16" t="s">
-        <v>561</v>
+        <v>565</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="s">
-        <v>562</v>
+        <v>566</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>489</v>
+        <v>493</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>563</v>
+        <v>567</v>
       </c>
       <c r="D34" s="16" t="s">
-        <v>564</v>
+        <v>568</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
       <c r="G34" s="16" t="s">
-        <v>566</v>
+        <v>570</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="6" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>489</v>
+        <v>493</v>
       </c>
       <c r="C35" s="16" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="D35" s="16" t="s">
+        <v>573</v>
+      </c>
+      <c r="E35" s="6" t="s">
+        <v>461</v>
+      </c>
+      <c r="F35" s="6" t="s">
         <v>569</v>
       </c>
-      <c r="E35" s="6" t="s">
-        <v>457</v>
-      </c>
-      <c r="F35" s="6" t="s">
-        <v>565</v>
-      </c>
       <c r="G35" s="16" t="s">
-        <v>570</v>
+        <v>574</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>489</v>
+        <v>493</v>
       </c>
       <c r="C36" s="16" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="D36" s="16" t="s">
-        <v>572</v>
+        <v>576</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G36" s="16" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="20" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="B37" s="20" t="s">
         <v>56</v>
       </c>
       <c r="C37" s="20" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="D37" s="16" t="s">
-        <v>576</v>
+        <v>580</v>
       </c>
       <c r="E37" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F37" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G37" s="16" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="20" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="B38" s="20" t="s">
-        <v>579</v>
+        <v>583</v>
       </c>
       <c r="C38" s="20" t="s">
-        <v>580</v>
+        <v>584</v>
       </c>
       <c r="D38" s="16" t="s">
-        <v>581</v>
+        <v>585</v>
       </c>
       <c r="E38" s="20" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="F38" s="20" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
       <c r="G38" s="16" t="s">
-        <v>582</v>
+        <v>586</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="20" t="s">
-        <v>583</v>
+        <v>587</v>
       </c>
       <c r="B39" s="20" t="s">
         <v>52</v>
       </c>
       <c r="C39" s="20" t="s">
-        <v>463</v>
+        <v>467</v>
       </c>
       <c r="D39" s="16" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="E39" s="20" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="F39" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G39" s="16" t="s">
-        <v>585</v>
+        <v>589</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="20" t="s">
-        <v>586</v>
+        <v>590</v>
       </c>
       <c r="B40" s="20" t="s">
-        <v>517</v>
+        <v>521</v>
       </c>
       <c r="C40" s="20" t="s">
-        <v>587</v>
+        <v>591</v>
       </c>
       <c r="D40" s="16" t="s">
-        <v>588</v>
+        <v>592</v>
       </c>
       <c r="E40" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F40" s="20" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
       <c r="G40" s="16" t="s">
-        <v>589</v>
+        <v>593</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="20" t="s">
-        <v>590</v>
+        <v>594</v>
       </c>
       <c r="B41" s="20" t="s">
         <v>76</v>
       </c>
       <c r="C41" s="20" t="s">
-        <v>591</v>
+        <v>595</v>
       </c>
       <c r="D41" s="16" t="s">
-        <v>592</v>
+        <v>596</v>
       </c>
       <c r="E41" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F41" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G41" s="16" t="s">
-        <v>593</v>
+        <v>597</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="20" t="s">
-        <v>594</v>
+        <v>598</v>
       </c>
       <c r="B42" s="20" t="s">
         <v>76</v>
       </c>
       <c r="C42" s="20" t="s">
-        <v>595</v>
+        <v>599</v>
       </c>
       <c r="D42" s="16" t="s">
-        <v>596</v>
+        <v>600</v>
       </c>
       <c r="E42" s="20" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="F42" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G42" s="16" t="s">
-        <v>597</v>
+        <v>601</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="20" t="s">
-        <v>598</v>
+        <v>602</v>
       </c>
       <c r="B43" s="20" t="s">
         <v>84</v>
       </c>
       <c r="C43" s="20" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="D43" s="16" t="s">
-        <v>600</v>
+        <v>604</v>
       </c>
       <c r="E43" s="20" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="F43" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G43" s="16" t="s">
-        <v>601</v>
+        <v>605</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="20" t="s">
-        <v>602</v>
+        <v>606</v>
       </c>
       <c r="B44" s="20" t="s">
         <v>76</v>
       </c>
       <c r="C44" s="20" t="s">
-        <v>603</v>
+        <v>607</v>
       </c>
       <c r="D44" s="16" t="s">
-        <v>604</v>
+        <v>608</v>
       </c>
       <c r="E44" s="20" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="F44" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G44" s="16" t="s">
-        <v>605</v>
+        <v>609</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="20" t="s">
-        <v>606</v>
+        <v>610</v>
       </c>
       <c r="B45" s="20" t="s">
         <v>183</v>
       </c>
       <c r="C45" s="20" t="s">
-        <v>607</v>
+        <v>611</v>
       </c>
       <c r="D45" s="16" t="s">
-        <v>608</v>
+        <v>612</v>
       </c>
       <c r="E45" s="20" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="F45" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G45" s="16" t="s">
-        <v>609</v>
+        <v>613</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="20" t="s">
-        <v>610</v>
+        <v>614</v>
       </c>
       <c r="B46" s="20" t="s">
         <v>80</v>
       </c>
       <c r="C46" s="20" t="s">
-        <v>611</v>
+        <v>615</v>
       </c>
       <c r="D46" s="16" t="s">
-        <v>612</v>
+        <v>616</v>
       </c>
       <c r="E46" s="20" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="F46" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G46" s="16" t="s">
-        <v>613</v>
+        <v>617</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="20" t="s">
-        <v>614</v>
+        <v>618</v>
       </c>
       <c r="B47" s="20" t="s">
         <v>183</v>
       </c>
       <c r="C47" s="20" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
       <c r="D47" s="16" t="s">
-        <v>616</v>
+        <v>620</v>
       </c>
       <c r="E47" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F47" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G47" s="16" t="s">
-        <v>617</v>
+        <v>621</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="20" t="s">
-        <v>618</v>
+        <v>622</v>
       </c>
       <c r="B48" s="20" t="s">
         <v>183</v>
       </c>
       <c r="C48" s="20" t="s">
-        <v>511</v>
+        <v>515</v>
       </c>
       <c r="D48" s="16" t="s">
-        <v>619</v>
+        <v>623</v>
       </c>
       <c r="E48" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F48" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G48" s="16" t="s">
-        <v>620</v>
+        <v>624</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="20" t="s">
-        <v>621</v>
+        <v>625</v>
       </c>
       <c r="B49" s="20" t="s">
         <v>207</v>
       </c>
       <c r="C49" s="20" t="s">
-        <v>622</v>
+        <v>626</v>
       </c>
       <c r="D49" s="16" t="s">
-        <v>623</v>
+        <v>627</v>
       </c>
       <c r="E49" s="20" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="F49" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G49" s="16" t="s">
-        <v>624</v>
+        <v>628</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="20" t="s">
-        <v>625</v>
+        <v>629</v>
       </c>
       <c r="B50" s="20" t="s">
         <v>231</v>
       </c>
       <c r="C50" s="20" t="s">
-        <v>626</v>
+        <v>630</v>
       </c>
       <c r="D50" s="16" t="s">
-        <v>627</v>
+        <v>631</v>
       </c>
       <c r="E50" s="20" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="F50" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G50" s="16" t="s">
-        <v>628</v>
+        <v>632</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="20" t="s">
-        <v>629</v>
+        <v>633</v>
       </c>
       <c r="B51" s="20" t="s">
         <v>231</v>
       </c>
       <c r="C51" s="20" t="s">
-        <v>630</v>
+        <v>634</v>
       </c>
       <c r="D51" s="16" t="s">
-        <v>631</v>
+        <v>635</v>
       </c>
       <c r="E51" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F51" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G51" s="16" t="s">
-        <v>632</v>
+        <v>636</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="20" t="s">
-        <v>633</v>
+        <v>637</v>
       </c>
       <c r="B52" s="20" t="s">
         <v>231</v>
       </c>
       <c r="C52" s="20" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="D52" s="16" t="s">
-        <v>634</v>
+        <v>638</v>
       </c>
       <c r="E52" s="20" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="F52" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G52" s="16" t="s">
-        <v>635</v>
+        <v>639</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="20" t="s">
-        <v>636</v>
+        <v>640</v>
       </c>
       <c r="B53" s="20" t="s">
         <v>231</v>
       </c>
       <c r="C53" s="20" t="s">
-        <v>637</v>
+        <v>641</v>
       </c>
       <c r="D53" s="16" t="s">
-        <v>638</v>
+        <v>642</v>
       </c>
       <c r="E53" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F53" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G53" s="16" t="s">
-        <v>639</v>
+        <v>643</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="20" t="s">
-        <v>640</v>
+        <v>644</v>
       </c>
       <c r="B54" s="20" t="s">
         <v>231</v>
       </c>
       <c r="C54" s="20" t="s">
-        <v>641</v>
+        <v>645</v>
       </c>
       <c r="D54" s="16" t="s">
-        <v>642</v>
+        <v>646</v>
       </c>
       <c r="E54" s="20" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="F54" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G54" s="16" t="s">
-        <v>643</v>
+        <v>647</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="20" t="s">
-        <v>644</v>
+        <v>648</v>
       </c>
       <c r="B55" s="20" t="s">
         <v>231</v>
       </c>
       <c r="C55" s="20" t="s">
-        <v>645</v>
+        <v>649</v>
       </c>
       <c r="D55" s="16" t="s">
-        <v>646</v>
+        <v>650</v>
       </c>
       <c r="E55" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F55" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G55" s="16" t="s">
-        <v>647</v>
+        <v>651</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="20" t="s">
-        <v>648</v>
+        <v>652</v>
       </c>
       <c r="B56" s="20" t="s">
         <v>231</v>
       </c>
       <c r="C56" s="20" t="s">
-        <v>637</v>
+        <v>641</v>
       </c>
       <c r="D56" s="16" t="s">
-        <v>649</v>
+        <v>653</v>
       </c>
       <c r="E56" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F56" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G56" s="16" t="s">
-        <v>650</v>
+        <v>654</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="20" t="s">
-        <v>651</v>
+        <v>655</v>
       </c>
       <c r="B57" s="20" t="s">
         <v>231</v>
       </c>
       <c r="C57" s="20" t="s">
-        <v>652</v>
+        <v>656</v>
       </c>
       <c r="D57" s="16" t="s">
-        <v>653</v>
+        <v>657</v>
       </c>
       <c r="E57" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F57" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G57" s="16" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="20" t="s">
-        <v>655</v>
+        <v>659</v>
       </c>
       <c r="B58" s="20" t="s">
         <v>231</v>
       </c>
       <c r="C58" s="20" t="s">
-        <v>656</v>
+        <v>660</v>
       </c>
       <c r="D58" s="16" t="s">
-        <v>657</v>
+        <v>661</v>
       </c>
       <c r="E58" s="20" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="F58" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G58" s="16" t="s">
-        <v>658</v>
+        <v>662</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="20" t="s">
-        <v>659</v>
+        <v>663</v>
       </c>
       <c r="B59" s="20" t="s">
         <v>231</v>
       </c>
       <c r="C59" s="20" t="s">
-        <v>660</v>
+        <v>664</v>
       </c>
       <c r="D59" s="16" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="E59" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F59" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G59" s="16" t="s">
-        <v>662</v>
+        <v>666</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="20" t="s">
-        <v>663</v>
+        <v>667</v>
       </c>
       <c r="B60" s="20" t="s">
         <v>231</v>
       </c>
       <c r="C60" s="20" t="s">
-        <v>664</v>
+        <v>668</v>
       </c>
       <c r="D60" s="16" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="E60" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F60" s="20" t="s">
-        <v>504</v>
+        <v>508</v>
       </c>
       <c r="G60" s="16" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="20" t="s">
-        <v>667</v>
+        <v>671</v>
       </c>
       <c r="B61" s="20" t="s">
         <v>231</v>
       </c>
       <c r="C61" s="20" t="s">
-        <v>668</v>
+        <v>672</v>
       </c>
       <c r="D61" s="16" t="s">
-        <v>669</v>
+        <v>673</v>
       </c>
       <c r="E61" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F61" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G61" s="16" t="s">
-        <v>670</v>
+        <v>674</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="20" t="s">
-        <v>671</v>
+        <v>675</v>
       </c>
       <c r="B62" s="20" t="s">
         <v>255</v>
       </c>
       <c r="C62" s="20" t="s">
-        <v>672</v>
+        <v>676</v>
       </c>
       <c r="D62" s="16" t="s">
-        <v>673</v>
+        <v>677</v>
       </c>
       <c r="E62" s="20" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="F62" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G62" s="16" t="s">
-        <v>674</v>
+        <v>678</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="20" t="s">
-        <v>675</v>
+        <v>679</v>
       </c>
       <c r="B63" s="20" t="s">
         <v>267</v>
       </c>
       <c r="C63" s="20" t="s">
-        <v>676</v>
+        <v>680</v>
       </c>
       <c r="D63" s="16" t="s">
-        <v>677</v>
+        <v>681</v>
       </c>
       <c r="E63" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F63" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G63" s="16" t="s">
-        <v>678</v>
+        <v>682</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="20" t="s">
-        <v>679</v>
+        <v>683</v>
       </c>
       <c r="B64" s="20" t="s">
         <v>275</v>
       </c>
       <c r="C64" s="20" t="s">
-        <v>680</v>
+        <v>684</v>
       </c>
       <c r="D64" s="16" t="s">
-        <v>681</v>
+        <v>685</v>
       </c>
       <c r="E64" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F64" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G64" s="16" t="s">
-        <v>682</v>
+        <v>686</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="20" t="s">
-        <v>683</v>
+        <v>687</v>
       </c>
       <c r="B65" s="20" t="s">
         <v>263</v>
       </c>
       <c r="C65" s="20" t="s">
-        <v>551</v>
+        <v>555</v>
       </c>
       <c r="D65" s="16" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
       <c r="E65" s="20" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="F65" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G65" s="16" t="s">
-        <v>685</v>
+        <v>689</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="20" t="s">
-        <v>686</v>
+        <v>690</v>
       </c>
       <c r="B66" s="20" t="s">
         <v>275</v>
       </c>
       <c r="C66" s="20" t="s">
-        <v>687</v>
+        <v>691</v>
       </c>
       <c r="D66" s="16" t="s">
-        <v>688</v>
+        <v>692</v>
       </c>
       <c r="E66" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F66" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G66" s="16" t="s">
-        <v>689</v>
+        <v>693</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="20" t="s">
-        <v>690</v>
+        <v>694</v>
       </c>
       <c r="B67" s="20" t="s">
         <v>271</v>
       </c>
       <c r="C67" s="20" t="s">
-        <v>691</v>
+        <v>695</v>
       </c>
       <c r="D67" s="16" t="s">
-        <v>692</v>
+        <v>696</v>
       </c>
       <c r="E67" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F67" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G67" s="16" t="s">
-        <v>693</v>
+        <v>697</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="20" t="s">
-        <v>694</v>
+        <v>698</v>
       </c>
       <c r="B68" s="20" t="s">
         <v>307</v>
       </c>
       <c r="C68" s="20" t="s">
-        <v>695</v>
+        <v>699</v>
       </c>
       <c r="D68" s="16" t="s">
-        <v>696</v>
+        <v>700</v>
       </c>
       <c r="E68" s="20" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="F68" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G68" s="16" t="s">
-        <v>697</v>
+        <v>701</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="20" t="s">
-        <v>698</v>
+        <v>702</v>
       </c>
       <c r="B69" s="20" t="s">
         <v>307</v>
       </c>
       <c r="C69" s="20" t="s">
-        <v>699</v>
+        <v>703</v>
       </c>
       <c r="D69" s="16" t="s">
-        <v>700</v>
+        <v>704</v>
       </c>
       <c r="E69" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F69" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G69" s="16" t="s">
-        <v>701</v>
+        <v>705</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="20" t="s">
-        <v>702</v>
+        <v>706</v>
       </c>
       <c r="B70" s="20" t="s">
         <v>307</v>
       </c>
       <c r="C70" s="20" t="s">
-        <v>703</v>
+        <v>707</v>
       </c>
       <c r="D70" s="16" t="s">
-        <v>704</v>
+        <v>708</v>
       </c>
       <c r="E70" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F70" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G70" s="16" t="s">
-        <v>705</v>
+        <v>709</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="20" t="s">
-        <v>706</v>
+        <v>710</v>
       </c>
       <c r="B71" s="20" t="s">
         <v>263</v>
       </c>
       <c r="C71" s="20" t="s">
-        <v>707</v>
+        <v>711</v>
       </c>
       <c r="D71" s="16" t="s">
-        <v>708</v>
+        <v>712</v>
       </c>
       <c r="E71" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F71" s="20" t="s">
-        <v>504</v>
+        <v>508</v>
       </c>
       <c r="G71" s="16" t="s">
-        <v>709</v>
+        <v>713</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="20" t="s">
-        <v>710</v>
+        <v>714</v>
       </c>
       <c r="B72" s="20" t="s">
-        <v>711</v>
+        <v>715</v>
       </c>
       <c r="C72" s="20" t="s">
-        <v>712</v>
+        <v>716</v>
       </c>
       <c r="D72" s="16" t="s">
-        <v>713</v>
+        <v>717</v>
       </c>
       <c r="E72" s="20" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="F72" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G72" s="16" t="s">
-        <v>714</v>
+        <v>718</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="20" t="s">
+        <v>719</v>
+      </c>
+      <c r="B73" s="20" t="s">
         <v>715</v>
       </c>
-      <c r="B73" s="20" t="s">
-        <v>711</v>
-      </c>
       <c r="C73" s="20" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="D73" s="16" t="s">
-        <v>717</v>
+        <v>721</v>
       </c>
       <c r="E73" s="20" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="F73" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G73" s="16" t="s">
-        <v>718</v>
+        <v>722</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="20" t="s">
-        <v>719</v>
+        <v>723</v>
       </c>
       <c r="B74" s="20" t="s">
-        <v>711</v>
+        <v>715</v>
       </c>
       <c r="C74" s="20" t="s">
-        <v>656</v>
+        <v>660</v>
       </c>
       <c r="D74" s="16" t="s">
-        <v>720</v>
+        <v>724</v>
       </c>
       <c r="E74" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F74" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G74" s="16" t="s">
-        <v>721</v>
+        <v>725</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="20" t="s">
-        <v>722</v>
+        <v>726</v>
       </c>
       <c r="B75" s="20" t="s">
         <v>351</v>
       </c>
       <c r="C75" s="20" t="s">
-        <v>723</v>
+        <v>727</v>
       </c>
       <c r="D75" s="16" t="s">
-        <v>724</v>
+        <v>728</v>
       </c>
       <c r="E75" s="20" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="F75" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G75" s="16" t="s">
-        <v>725</v>
+        <v>729</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="20" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="B76" s="20" t="s">
         <v>351</v>
       </c>
       <c r="C76" s="20" t="s">
-        <v>727</v>
+        <v>731</v>
       </c>
       <c r="D76" s="16" t="s">
-        <v>728</v>
+        <v>732</v>
       </c>
       <c r="E76" s="20" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="F76" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G76" s="16" t="s">
-        <v>729</v>
+        <v>733</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="20" t="s">
-        <v>730</v>
+        <v>734</v>
       </c>
       <c r="B77" s="20" t="s">
         <v>351</v>
       </c>
       <c r="C77" s="20" t="s">
-        <v>731</v>
+        <v>735</v>
       </c>
       <c r="D77" s="16" t="s">
-        <v>732</v>
+        <v>736</v>
       </c>
       <c r="E77" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F77" s="20" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
       <c r="G77" s="16" t="s">
-        <v>733</v>
+        <v>737</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="20" t="s">
-        <v>734</v>
+        <v>738</v>
       </c>
       <c r="B78" s="20" t="s">
-        <v>735</v>
+        <v>739</v>
       </c>
       <c r="C78" s="20" t="s">
-        <v>736</v>
+        <v>740</v>
       </c>
       <c r="D78" s="16" t="s">
-        <v>737</v>
+        <v>741</v>
       </c>
       <c r="E78" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F78" s="20" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
       <c r="G78" s="16" t="s">
-        <v>738</v>
+        <v>742</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="20" t="s">
+        <v>743</v>
+      </c>
+      <c r="B79" s="20" t="s">
         <v>739</v>
       </c>
-      <c r="B79" s="20" t="s">
-        <v>735</v>
-      </c>
       <c r="C79" s="20" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="D79" s="16" t="s">
-        <v>741</v>
+        <v>745</v>
       </c>
       <c r="E79" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F79" s="20" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
       <c r="G79" s="16" t="s">
-        <v>742</v>
+        <v>746</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="20" t="s">
-        <v>743</v>
+        <v>747</v>
       </c>
       <c r="B80" s="20" t="s">
         <v>379</v>
       </c>
       <c r="C80" s="20" t="s">
-        <v>744</v>
+        <v>748</v>
       </c>
       <c r="D80" s="16" t="s">
-        <v>745</v>
+        <v>749</v>
       </c>
       <c r="E80" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F80" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G80" s="16" t="s">
-        <v>746</v>
+        <v>750</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="20" t="s">
-        <v>747</v>
+        <v>751</v>
       </c>
       <c r="B81" s="20" t="s">
         <v>371</v>
       </c>
       <c r="C81" s="20" t="s">
-        <v>748</v>
+        <v>752</v>
       </c>
       <c r="D81" s="16" t="s">
-        <v>749</v>
+        <v>753</v>
       </c>
       <c r="E81" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F81" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G81" s="16" t="s">
-        <v>750</v>
+        <v>754</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="20" t="s">
-        <v>751</v>
+        <v>755</v>
       </c>
       <c r="B82" s="20" t="s">
         <v>367</v>
       </c>
       <c r="C82" s="20" t="s">
-        <v>752</v>
+        <v>756</v>
       </c>
       <c r="D82" s="16" t="s">
-        <v>753</v>
+        <v>757</v>
       </c>
       <c r="E82" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F82" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G82" s="16" t="s">
-        <v>754</v>
+        <v>758</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="20" t="s">
-        <v>755</v>
+        <v>759</v>
       </c>
       <c r="B83" s="20" t="s">
         <v>367</v>
       </c>
       <c r="C83" s="20" t="s">
-        <v>756</v>
+        <v>760</v>
       </c>
       <c r="D83" s="16" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="E83" s="20" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="F83" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G83" s="16" t="s">
-        <v>758</v>
+        <v>762</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="20" t="s">
-        <v>759</v>
+        <v>763</v>
       </c>
       <c r="B84" s="20" t="s">
         <v>351</v>
       </c>
       <c r="C84" s="20" t="s">
-        <v>760</v>
+        <v>764</v>
       </c>
       <c r="D84" s="16" t="s">
-        <v>761</v>
+        <v>765</v>
       </c>
       <c r="E84" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F84" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G84" s="16" t="s">
-        <v>762</v>
+        <v>766</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="20" t="s">
-        <v>763</v>
+        <v>767</v>
       </c>
       <c r="B85" s="20" t="s">
         <v>323</v>
       </c>
       <c r="C85" s="20" t="s">
-        <v>764</v>
+        <v>768</v>
       </c>
       <c r="D85" s="16" t="s">
-        <v>765</v>
+        <v>769</v>
       </c>
       <c r="E85" s="20" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="F85" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G85" s="16" t="s">
-        <v>766</v>
+        <v>770</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="20" t="s">
-        <v>767</v>
+        <v>771</v>
       </c>
       <c r="B86" s="20" t="s">
         <v>323</v>
       </c>
       <c r="C86" s="20" t="s">
-        <v>768</v>
+        <v>772</v>
       </c>
       <c r="D86" s="16" t="s">
-        <v>769</v>
+        <v>773</v>
       </c>
       <c r="E86" s="20" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="F86" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G86" s="16" t="s">
-        <v>770</v>
+        <v>774</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="20" t="s">
-        <v>771</v>
+        <v>775</v>
       </c>
       <c r="B87" s="20" t="s">
         <v>375</v>
       </c>
       <c r="C87" s="20" t="s">
-        <v>772</v>
+        <v>776</v>
       </c>
       <c r="D87" s="16" t="s">
-        <v>773</v>
+        <v>777</v>
       </c>
       <c r="E87" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F87" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G87" s="16" t="s">
-        <v>774</v>
+        <v>778</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="20" t="s">
-        <v>775</v>
+        <v>779</v>
       </c>
       <c r="B88" s="20" t="s">
         <v>379</v>
       </c>
       <c r="C88" s="20" t="s">
-        <v>776</v>
+        <v>780</v>
       </c>
       <c r="D88" s="16" t="s">
-        <v>777</v>
+        <v>781</v>
       </c>
       <c r="E88" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F88" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G88" s="16" t="s">
-        <v>778</v>
+        <v>782</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="20" t="s">
-        <v>779</v>
+        <v>783</v>
       </c>
       <c r="B89" s="20" t="s">
         <v>331</v>
       </c>
       <c r="C89" s="20" t="s">
-        <v>780</v>
+        <v>784</v>
       </c>
       <c r="D89" s="16" t="s">
-        <v>781</v>
+        <v>785</v>
       </c>
       <c r="E89" s="20" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="F89" s="20" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
       <c r="G89" s="16" t="s">
-        <v>782</v>
+        <v>786</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="20" t="s">
-        <v>783</v>
+        <v>787</v>
       </c>
       <c r="B90" s="20" t="s">
         <v>279</v>
       </c>
       <c r="C90" s="20" t="s">
-        <v>784</v>
+        <v>788</v>
       </c>
       <c r="D90" s="16" t="s">
-        <v>785</v>
+        <v>789</v>
       </c>
       <c r="E90" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F90" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G90" s="16" t="s">
-        <v>786</v>
+        <v>790</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="20" t="s">
-        <v>787</v>
+        <v>791</v>
       </c>
       <c r="B91" s="20" t="s">
         <v>279</v>
       </c>
       <c r="C91" s="20" t="s">
-        <v>784</v>
+        <v>788</v>
       </c>
       <c r="D91" s="16" t="s">
-        <v>788</v>
+        <v>792</v>
       </c>
       <c r="E91" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F91" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G91" s="16" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="20" t="s">
-        <v>790</v>
+        <v>794</v>
       </c>
       <c r="B92" s="20" t="s">
         <v>291</v>
       </c>
       <c r="C92" s="20" t="s">
-        <v>791</v>
+        <v>795</v>
       </c>
       <c r="D92" s="16" t="s">
-        <v>792</v>
+        <v>796</v>
       </c>
       <c r="E92" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F92" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G92" s="16" t="s">
-        <v>793</v>
+        <v>797</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="20" t="s">
-        <v>794</v>
+        <v>798</v>
       </c>
       <c r="B93" s="20" t="s">
         <v>299</v>
       </c>
       <c r="C93" s="20" t="s">
-        <v>795</v>
+        <v>799</v>
       </c>
       <c r="D93" s="16" t="s">
-        <v>796</v>
+        <v>800</v>
       </c>
       <c r="E93" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F93" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G93" s="16" t="s">
-        <v>797</v>
+        <v>801</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="157.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="20" t="s">
-        <v>798</v>
+        <v>802</v>
       </c>
       <c r="B94" s="20" t="s">
         <v>291</v>
       </c>
       <c r="C94" s="20" t="s">
-        <v>799</v>
+        <v>803</v>
       </c>
       <c r="D94" s="16" t="s">
-        <v>800</v>
+        <v>804</v>
       </c>
       <c r="E94" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F94" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G94" s="16" t="s">
-        <v>801</v>
+        <v>805</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A95" s="20" t="s">
-        <v>802</v>
+        <v>806</v>
       </c>
       <c r="B95" s="20" t="s">
         <v>371</v>
       </c>
       <c r="C95" s="20" t="s">
-        <v>803</v>
+        <v>807</v>
       </c>
       <c r="D95" s="16" t="s">
-        <v>804</v>
+        <v>808</v>
       </c>
       <c r="E95" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="F95" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G95" s="16" t="s">
-        <v>805</v>
+        <v>809</v>
       </c>
     </row>
   </sheetData>
@@ -8225,12 +8260,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>806</v>
+        <v>810</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>807</v>
+        <v>811</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8238,16 +8273,16 @@
         <v>19</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>808</v>
+        <v>812</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>809</v>
+        <v>813</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>810</v>
+        <v>814</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>811</v>
+        <v>815</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>22</v>
@@ -8255,382 +8290,382 @@
     </row>
     <row r="5" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>812</v>
+        <v>816</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>813</v>
+        <v>817</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>814</v>
+        <v>818</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>815</v>
+        <v>819</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>816</v>
+        <v>820</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>817</v>
+        <v>821</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>818</v>
+        <v>822</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>819</v>
+        <v>823</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>820</v>
+        <v>824</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>821</v>
+        <v>825</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>822</v>
+        <v>826</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>823</v>
+        <v>827</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>824</v>
+        <v>828</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>825</v>
+        <v>829</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>826</v>
+        <v>830</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>827</v>
+        <v>831</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>504</v>
+        <v>508</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>828</v>
+        <v>832</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>829</v>
+        <v>833</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>830</v>
+        <v>834</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>831</v>
+        <v>835</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>832</v>
+        <v>836</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>504</v>
+        <v>508</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>833</v>
+        <v>837</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>834</v>
+        <v>838</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>835</v>
+        <v>839</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>836</v>
+        <v>840</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>837</v>
+        <v>841</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
+        <v>842</v>
+      </c>
+      <c r="B10" s="16" t="s">
         <v>838</v>
       </c>
-      <c r="B10" s="16" t="s">
-        <v>834</v>
-      </c>
       <c r="C10" s="16" t="s">
-        <v>839</v>
+        <v>843</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>840</v>
+        <v>844</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>841</v>
+        <v>845</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>842</v>
+        <v>846</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>843</v>
+        <v>847</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>844</v>
+        <v>848</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>845</v>
+        <v>849</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>846</v>
+        <v>850</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>822</v>
+        <v>826</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>847</v>
+        <v>851</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>848</v>
+        <v>852</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>849</v>
+        <v>853</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>850</v>
+        <v>854</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>851</v>
+        <v>855</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="s">
-        <v>852</v>
+        <v>856</v>
       </c>
       <c r="B13" s="20" t="s">
-        <v>843</v>
+        <v>847</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>853</v>
+        <v>857</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>854</v>
+        <v>858</v>
       </c>
       <c r="E13" s="20" t="s">
-        <v>855</v>
+        <v>859</v>
       </c>
       <c r="F13" s="20" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
-        <v>856</v>
+        <v>860</v>
       </c>
       <c r="B14" s="20" t="s">
-        <v>848</v>
+        <v>852</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>857</v>
+        <v>861</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>858</v>
+        <v>862</v>
       </c>
       <c r="E14" s="20" t="s">
-        <v>859</v>
+        <v>863</v>
       </c>
       <c r="F14" s="20" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="20" t="s">
-        <v>860</v>
+        <v>864</v>
       </c>
       <c r="B15" s="20" t="s">
-        <v>861</v>
+        <v>865</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>862</v>
+        <v>866</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>863</v>
+        <v>867</v>
       </c>
       <c r="E15" s="20" t="s">
-        <v>864</v>
+        <v>868</v>
       </c>
       <c r="F15" s="20" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="20" t="s">
-        <v>865</v>
+        <v>869</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>813</v>
+        <v>817</v>
       </c>
       <c r="C16" s="16" t="s">
-        <v>866</v>
+        <v>870</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>867</v>
+        <v>871</v>
       </c>
       <c r="E16" s="20" t="s">
-        <v>868</v>
+        <v>872</v>
       </c>
       <c r="F16" s="20" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="20" t="s">
-        <v>869</v>
+        <v>873</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>834</v>
+        <v>838</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>870</v>
+        <v>874</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="E17" s="20" t="s">
-        <v>872</v>
+        <v>876</v>
       </c>
       <c r="F17" s="20" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="20" t="s">
-        <v>873</v>
+        <v>877</v>
       </c>
       <c r="B18" s="20" t="s">
-        <v>843</v>
+        <v>847</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>874</v>
+        <v>878</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>875</v>
+        <v>879</v>
       </c>
       <c r="E18" s="20" t="s">
-        <v>876</v>
+        <v>880</v>
       </c>
       <c r="F18" s="20" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="20" t="s">
-        <v>877</v>
+        <v>881</v>
       </c>
       <c r="B19" s="20" t="s">
-        <v>878</v>
+        <v>882</v>
       </c>
       <c r="C19" s="16" t="s">
-        <v>879</v>
+        <v>883</v>
       </c>
       <c r="D19" s="16" t="s">
-        <v>880</v>
+        <v>884</v>
       </c>
       <c r="E19" s="20" t="s">
-        <v>881</v>
+        <v>885</v>
       </c>
       <c r="F19" s="20" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="20" t="s">
-        <v>882</v>
+        <v>886</v>
       </c>
       <c r="B20" s="20" t="s">
-        <v>883</v>
+        <v>887</v>
       </c>
       <c r="C20" s="16" t="s">
-        <v>884</v>
+        <v>888</v>
       </c>
       <c r="D20" s="16" t="s">
-        <v>885</v>
+        <v>889</v>
       </c>
       <c r="E20" s="20" t="s">
-        <v>886</v>
+        <v>890</v>
       </c>
       <c r="F20" s="20" t="s">
-        <v>822</v>
+        <v>826</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="20" t="s">
-        <v>887</v>
+        <v>891</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>888</v>
+        <v>892</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>889</v>
+        <v>893</v>
       </c>
       <c r="D21" s="16" t="s">
-        <v>890</v>
+        <v>894</v>
       </c>
       <c r="E21" s="20" t="s">
-        <v>891</v>
+        <v>895</v>
       </c>
       <c r="F21" s="20" t="s">
-        <v>504</v>
+        <v>508</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="20" t="s">
-        <v>892</v>
+        <v>896</v>
       </c>
       <c r="B22" s="20" t="s">
-        <v>893</v>
+        <v>897</v>
       </c>
       <c r="C22" s="16" t="s">
-        <v>894</v>
+        <v>898</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>895</v>
+        <v>899</v>
       </c>
       <c r="E22" s="20" t="s">
-        <v>896</v>
+        <v>900</v>
       </c>
       <c r="F22" s="20" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="20" t="s">
-        <v>897</v>
+        <v>901</v>
       </c>
       <c r="B23" s="20" t="s">
-        <v>898</v>
+        <v>902</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>899</v>
+        <v>903</v>
       </c>
       <c r="D23" s="16" t="s">
-        <v>900</v>
+        <v>904</v>
       </c>
       <c r="E23" s="20" t="s">
-        <v>901</v>
+        <v>905</v>
       </c>
       <c r="F23" s="20" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove temp backup file; tracker update
</commit_message>
<xml_diff>
--- a/HilotSpa_ThesisTracker.xlsx
+++ b/HilotSpa_ThesisTracker.xlsx
@@ -431,7 +431,7 @@
     <t xml:space="preserve">A node may only write resources it owns. Makes split-brain structurally impossible.</t>
   </si>
   <si>
-    <t xml:space="preserve">See Defense Risks R1. THE core architectural argument.</t>
+    <t xml:space="preserve">Half of it is now enforced, and it is the half that can be. 2026-08-30: a therapist and a room each belong to exactly one branch (schema), and Flyway migration V2 adds EXCLUDE constraints so the database itself refuses an overlapping write. Within a node, single-writer is a mechanism rather than a convention. What remains is the cross-node half - a node refusing to write a resource it does not own - which needs the node registry (3.2) to exist first.</t>
   </si>
   <si>
     <t xml:space="preserve">3.5</t>
@@ -3509,11 +3509,11 @@
       </c>
       <c r="D8" s="6" t="n">
         <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A8,Tasks!$E$5:$E$110,"In Progress")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E8" s="6" t="n">
         <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A8,Tasks!$E$5:$E$110,"Not Started")</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F8" s="6" t="n">
         <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A8,Tasks!$E$5:$E$110,"Blocked")</f>
@@ -3567,11 +3567,11 @@
       </c>
       <c r="D10" s="9" t="n">
         <f aca="false">SUM(D5:D9)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E10" s="9" t="n">
         <f aca="false">SUM(E5:E9)</f>
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F10" s="9" t="n">
         <f aca="false">SUM(F5:F9)</f>
@@ -4235,7 +4235,7 @@
         <v>133</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F31" s="6"/>
       <c r="G31" s="16" t="s">
@@ -6002,7 +6002,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="110" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="110" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="19" t="s">
         <v>9</v>
       </c>

</xml_diff>

<commit_message>
Public landing page, service photos, therapist status and preference
2.41/2.42 - public landing, browsable menu, /contact. GET /api/v1/public/** is the only unauthenticated read: the spa's details and its live menu, with a separate DTO because the logged-in catalogue carries contraindication verdicts that must never be computed for a stranger.

2.40 - service photos keyed by a filename the admin sets, never the service id, which is regenerated on every reseed.

2.38 - TherapistStatus is honoured, and only for today. The staff screen already promised this; the sentence was false until now.

2.43/2.44 - a client may ask for a woman or a man. Enforced in availability AND at assignment, because a preference the screen respects and the write path ignores is worse than none. Meet-the-team shows first names and sex only.

Migrations V3 and V4. 37 tests, 0 failures.
</commit_message>
<xml_diff>
--- a/HilotSpa_ThesisTracker.xlsx
+++ b/HilotSpa_ThesisTracker.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1502" uniqueCount="906">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1586" uniqueCount="954">
   <si>
     <t xml:space="preserve">HilotSpa — Progress Summary</t>
   </si>
@@ -194,7 +194,7 @@
     <t xml:space="preserve">Flyway so every node shares an identical schema. Redis into pom.xml + compose.yaml.</t>
   </si>
   <si>
-    <t xml:space="preserve">Closed 2026-08-30. Flyway owns the schema; Hibernate switched to ddl-auto=validate and PASSED against the live database on the first try, which also proves the V1 baseline dump is accurate. V1 is a pg_dump of the schema as ddl-auto left it (three lines stripped: \restrict / \unrestrict psql meta-commands that pg_dump 15.18 emits and JDBC cannot parse, and the search_path reset that would have broken Flyway's own INSERT into flyway_schema_history). Both settings are env-driven - FLYWAY_ENABLED / DDL_AUTO - so the rollback is deleting two lines from .env, no rebuild. THE TRAP: on Spring Boot 4, flyway-core alone is NOT enough. Boot 4 split auto-configuration into one module per technology, so FlywayAutoConfiguration ships with spring-boot-starter-flyway. With only flyway-core the library is present, the auto-configuration is not, and every spring.flyway.* property is an inert string - no error, no warning, no log line, the app starts perfectly and never migrates. Cost about 40 minutes of chasing a stale Docker image that was not stale.</t>
+    <t xml:space="preserve">Closed 2026-08-30. Flyway owns the schema; Hibernate switched to ddl-auto=validate and PASSED against the live database on the first try, which also proves the V1 baseline dump is accurate. V1 is a pg_dump of the schema as ddl-auto left it (three lines stripped: \restrict / \unrestrict psql meta-commands that pg_dump 15.18 emits and JDBC cannot parse, and the search_path reset that would have broken Flyway's own INSERT into flyway_schema_history). Both settings are env-driven - FLYWAY_ENABLED / DDL_AUTO - so the rollback is deleting two lines from .env, no rebuild. THE TRAP: on Spring Boot 4, flyway-core alone is NOT enough. Boot 4 split auto-configuration into one module per technology, so FlywayAutoConfiguration ships with spring-boot-starter-flyway. With only flyway-core the library is present, the auto-configuration is not, and every spring.flyway.* property is an inert string - no error, no warning, no log line, the app starts perfectly and never migrates. Cost about 40 minutes of chasing a stale Docker image that was not stale. | PROVEN IN ANGER 2026-08-31, the very first entity change after the switch: Massage.imageName was added without a migration and all 33 tests errored with 'Schema validation: missing column [image_name] in table [massage]' - a refusal to start, naming the exact table and column. Under the old ddl-auto=update Hibernate would have silently added it on one machine and left every other node missing it, which is B66/B77/B85 exactly. Fixed by V3__service_photo.sql. Good defence answer: the schema is versioned and the system refuses to run against a database it does not recognise - and we have a real incident to describe, not a claim.</t>
   </si>
   <si>
     <t xml:space="preserve">0.8</t>
@@ -1295,7 +1295,7 @@
     <t xml:space="preserve">AVAILABLE / BUSY / ON_BREAK / OFF_DUTY is set on the staff screen and counted on the admin overview, but availability filters on active only - an OFF_DUTY therapist is still bookable.</t>
   </si>
   <si>
-    <t xml:space="preserve">Either consult it in anyFree()/assign() or remove it from the screens. A visible control that does nothing is worse than no control.</t>
+    <t xml:space="preserve">Decided and built 2026-08-31: HONOURED, and only for TODAY. active=false means the therapist has left the spa and is gone from every day; status is a right-now flag with no end time, so it removes them from today's remaining slots and nothing else - marking someone ON_BREAK must not empty next Tuesday, or staff learn never to touch the control. Applied in availability AND again in assign(), so a walk-in cannot be handed to somebody the front desk marked off duty thirty seconds earlier. The staff Resources screen already PROMISED this ('a therapist set off duty disappears from availability at once') - the sentence was simply false until now. 2 tests, written through the walk-in path because availability only offers future times and a test against today's calendar would pass at 10am and fail at 10pm.</t>
   </si>
   <si>
     <t xml:space="preserve">2.39</t>
@@ -1362,6 +1362,150 @@
   </si>
   <si>
     <t xml:space="preserve">Written 2026-08-30 alongside 0.7. The rules exist because ddl-auto=validate now fails the boot when an entity and the migrations disagree - which is the point, but only helps if the next person knows why.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pre-deployment security checklist</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SPRING_PROFILES_ACTIVE off dev (DevDataSeeder is @Profile("dev") - leaving it on puts admin@hilotspa.test / hilotspa123 live); regenerate JWT_SECRET (went through a chat transcript); change the DB password (admin1234 is in git history); finish 2.17 and never expose 5678.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BLOCKS any public URL. About an hour together. The profile one is the dangerous one - it is a live administrator account on a system holding client health records.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Single origin - serve the Angular build from Spring Boot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ng build -&gt; src/main/resources/static/, and make API_BASE relative (/api/v1) instead of the hardcoded http://localhost:8080. One domain, one certificate, no CORS, no mixed content.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~30 min and it is the prerequisite for every hosting route. Also removes a whole class of defence-day failure: one thing to start instead of two.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reverse proxy + TLS (compose.prod.yaml)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caddy in front of the backend for automatic Let's Encrypt. Ports 80/443 only; 8080, 5432 and 5678 stay on the compose network.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Needed for a real URL by either route.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Decide the hosting route and stand it up</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Route A: Cloudflare Tunnel, node stays local - matches the paper's "localized storage at each branch". Route B: AWS EC2 t3.small (NOT micro - Postgres + JVM + n8n will OOM in 1GB), 30GB gp3, 2GB swap, ap-southeast-1, Elastic IP, SG open on 22/80/443 only, CloudWatch billing alarm.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The panel has asked for a real URL. NOTE: AWS changed the free tier - accounts after 15 Jul 2025 get $100 credits for 12 months, not 750 free hours, and a Free Plan account auto-closes when they run out.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Log the hosting deviation in paper-deltas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">If the node runs on a rented host it is no longer "localized at each branch". One paragraph: for evaluation, one node ran hosted so the panel and testers could reach it; the node software is identical either way.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Only needed for route B. Route A keeps the claim literally true, which is the strongest argument for it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Service photos keyed by a stable slug, not the service UUID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">services.html and service-detail.html point at /services/{serviceId}.jpg. Service ids are regenerated on every reseed, so real photos would break and the filenames are unreadable. Add a slug/imageUrl on Massage, editable in the A6 config screen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Built 2026-08-31. Massage.imageName holds a FILENAME set from the A6 service menu (with a live preview in the drawer), never the service id - ids are regenerated on every reseed, so real photographs would have broken and the files would have had unreadable names. Carried on both the public and the authenticated catalogue DTOs. Missing photo = tinted block, never a broken image. Seeder sets sensible defaults and public/services/README.md is the naming list for Liodoq's partner.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.41</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Public landing page and browsable menu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Landing at / (hero, live menu from the same Massage table, how-a-visit-works, find-us), public /contact, and /services + /services/:id + /about no longer behind authGuard.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Built 2026-08-31. Everything used to sit behind a guard and / redirected to login, so the first thing anyone met - client, adviser, panelist opening the URL - was a password box. Browsing is public now; BOOKING is not, and Process Rule #2 is untouched. The menu comes from the same table the assistant works from, so the public page cannot drift from what the spa actually sells.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Public read endpoint - GET /api/v1/public/**</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PublicController: the spa's own details (config-driven, so SS A3 is one line to change) and its live menu. Withdrawn treatments filtered out. GET-only permitAll; a POST falls through to authenticated().</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The ONLY unauthenticated read in the system, and a separate DTO on purpose: the logged-in catalogue carries contraindication verdicts, which are a judgement about a named client and must never be computed for a stranger. No protocol rules, no availability, no therapists, no counts. Nothing here takes a parameter, so nothing here can be made to answer a question about a particular person. CatalogueStore.anonymous distinguishes the three states so a visitor is never told 'no exclusions apply to your assessment' - a claim about a judgement that was never made.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spa contact details for the public site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SPA_PHONE, SPA_FACEBOOK, SPA_MAPS_URL, SPA_ADDRESS, SPA_HOURS in .env. The landing and contact pages hide any field left blank rather than showing an empty label.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Needs the real numbers from the spa. Contact is details-only by design - there is no mail path, and a form that silently files a message nobody reads is worse than no form because the client believes they have made contact and waits.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.43</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Therapist preference - a client may ask for a woman or a man</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sex enum on Therapist; Forms.therapistPreference (null = no preference); enforced in availability AND at assignment; refusal message distinguishes "no female therapist is free then" from "that time was just taken". Migration V4.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Built 2026-08-31 at Liodoq's request. Hilot is close, hands-on work and in this province this is a matter of dignity, not taste - a client who cannot say who they are comfortable with does not come back. Deliberately NO 'ANY' enum value: null means no preference, which keeps 'never asked' distinguishable from 'said it does not matter'. A therapist whose sex is not recorded matches NO preference - guessing is the one failure this feature exists to prevent. 2 tests, one of which compares two identical assessments differing only in preference and fails if availability is unchanged - i.e. it fails if the feature is decorative, which is exactly the state TherapistStatus was in an hour earlier. CAPACITY NOTE: Bulan seeds one woman and one man, so asking for a woman roughly halves availability. Honest, and worth seeing before the demo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.44</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Meet the team on the public site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PublicTherapist: first name and sex only. No surname, no photograph, no schedule, and no id - an id would let a stranger probe one named person's availability. Active staff only.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Built 2026-08-31. Shown so a client can see that both women and men are on the team BEFORE being asked to state a preference. Photos were considered and deliberately not built: a staff member's face on a public URL needs their written consent, which is a conversation the spa has to have, not a design decision.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Log the therapist-preference feature in paper-deltas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Scope mentions analysing "resources" but says nothing about therapist sex or client preference. An addition, not a contradiction - but it needs a paragraph before a panelist asks where it came from.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Also worth a sentence on WHY: it is a dignity and comfort requirement in a conservative province, and it demonstrably narrows availability rather than being cosmetic, which makes it defensible as a real constraint on the scheduling problem rather than a UI flourish.</t>
   </si>
   <si>
     <t xml:space="preserve">HilotSpa — Bug &amp; Finding Log</t>
@@ -3413,28 +3557,28 @@
         <v>9</v>
       </c>
       <c r="B5" s="6" t="n">
-        <f aca="false">COUNTIF(Tasks!$A$5:$A$110,$A5)</f>
-        <v>19</v>
+        <f aca="false">COUNTIF(Tasks!$A$5:$A$122,$A5)</f>
+        <v>24</v>
       </c>
       <c r="C5" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A5,Tasks!$E$5:$E$110,"Done")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$122,$A5,Tasks!$E$5:$E$122,"Done")</f>
         <v>17</v>
       </c>
       <c r="D5" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A5,Tasks!$E$5:$E$110,"In Progress")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$122,$A5,Tasks!$E$5:$E$122,"In Progress")</f>
         <v>0</v>
       </c>
       <c r="E5" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A5,Tasks!$E$5:$E$110,"Not Started")</f>
-        <v>2</v>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$122,$A5,Tasks!$E$5:$E$122,"Not Started")</f>
+        <v>7</v>
       </c>
       <c r="F5" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A5,Tasks!$E$5:$E$110,"Blocked")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$122,$A5,Tasks!$E$5:$E$122,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G5" s="7" t="n">
         <f aca="false">IFERROR($C5/$B5,0)</f>
-        <v>0.894736842105263</v>
+        <v>0.708333333333333</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3442,23 +3586,23 @@
         <v>10</v>
       </c>
       <c r="B6" s="6" t="n">
-        <f aca="false">COUNTIF(Tasks!$A$5:$A$110,$A6)</f>
+        <f aca="false">COUNTIF(Tasks!$A$5:$A$122,$A6)</f>
         <v>20</v>
       </c>
       <c r="C6" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A6,Tasks!$E$5:$E$110,"Done")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$122,$A6,Tasks!$E$5:$E$122,"Done")</f>
         <v>20</v>
       </c>
       <c r="D6" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A6,Tasks!$E$5:$E$110,"In Progress")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$122,$A6,Tasks!$E$5:$E$122,"In Progress")</f>
         <v>0</v>
       </c>
       <c r="E6" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A6,Tasks!$E$5:$E$110,"Not Started")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$122,$A6,Tasks!$E$5:$E$122,"Not Started")</f>
         <v>0</v>
       </c>
       <c r="F6" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A6,Tasks!$E$5:$E$110,"Blocked")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$122,$A6,Tasks!$E$5:$E$122,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G6" s="7" t="n">
@@ -3471,28 +3615,28 @@
         <v>11</v>
       </c>
       <c r="B7" s="6" t="n">
-        <f aca="false">COUNTIF(Tasks!$A$5:$A$110,$A7)</f>
-        <v>39</v>
+        <f aca="false">COUNTIF(Tasks!$A$5:$A$122,$A7)</f>
+        <v>44</v>
       </c>
       <c r="C7" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A7,Tasks!$E$5:$E$110,"Done")</f>
-        <v>34</v>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$122,$A7,Tasks!$E$5:$E$122,"Done")</f>
+        <v>40</v>
       </c>
       <c r="D7" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A7,Tasks!$E$5:$E$110,"In Progress")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$122,$A7,Tasks!$E$5:$E$122,"In Progress")</f>
         <v>3</v>
       </c>
       <c r="E7" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A7,Tasks!$E$5:$E$110,"Not Started")</f>
-        <v>2</v>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$122,$A7,Tasks!$E$5:$E$122,"Not Started")</f>
+        <v>1</v>
       </c>
       <c r="F7" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A7,Tasks!$E$5:$E$110,"Blocked")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$122,$A7,Tasks!$E$5:$E$122,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G7" s="7" t="n">
         <f aca="false">IFERROR($C7/$B7,0)</f>
-        <v>0.871794871794872</v>
+        <v>0.909090909090909</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3500,23 +3644,23 @@
         <v>12</v>
       </c>
       <c r="B8" s="6" t="n">
-        <f aca="false">COUNTIF(Tasks!$A$5:$A$110,$A8)</f>
+        <f aca="false">COUNTIF(Tasks!$A$5:$A$122,$A8)</f>
         <v>15</v>
       </c>
       <c r="C8" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A8,Tasks!$E$5:$E$110,"Done")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$122,$A8,Tasks!$E$5:$E$122,"Done")</f>
         <v>4</v>
       </c>
       <c r="D8" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A8,Tasks!$E$5:$E$110,"In Progress")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$122,$A8,Tasks!$E$5:$E$122,"In Progress")</f>
         <v>6</v>
       </c>
       <c r="E8" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A8,Tasks!$E$5:$E$110,"Not Started")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$122,$A8,Tasks!$E$5:$E$122,"Not Started")</f>
         <v>5</v>
       </c>
       <c r="F8" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A8,Tasks!$E$5:$E$110,"Blocked")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$122,$A8,Tasks!$E$5:$E$122,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G8" s="7" t="n">
@@ -3529,28 +3673,28 @@
         <v>13</v>
       </c>
       <c r="B9" s="6" t="n">
-        <f aca="false">COUNTIF(Tasks!$A$5:$A$110,$A9)</f>
+        <f aca="false">COUNTIF(Tasks!$A$5:$A$122,$A9)</f>
+        <v>15</v>
+      </c>
+      <c r="C9" s="6" t="n">
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$122,$A9,Tasks!$E$5:$E$122,"Done")</f>
+        <v>1</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$122,$A9,Tasks!$E$5:$E$122,"In Progress")</f>
+        <v>1</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$122,$A9,Tasks!$E$5:$E$122,"Not Started")</f>
         <v>13</v>
       </c>
-      <c r="C9" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A9,Tasks!$E$5:$E$110,"Done")</f>
-        <v>1</v>
-      </c>
-      <c r="D9" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A9,Tasks!$E$5:$E$110,"In Progress")</f>
-        <v>1</v>
-      </c>
-      <c r="E9" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A9,Tasks!$E$5:$E$110,"Not Started")</f>
-        <v>11</v>
-      </c>
       <c r="F9" s="6" t="n">
-        <f aca="false">COUNTIFS(Tasks!$A$5:$A$110,$A9,Tasks!$E$5:$E$110,"Blocked")</f>
+        <f aca="false">COUNTIFS(Tasks!$A$5:$A$122,$A9,Tasks!$E$5:$E$122,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="G9" s="7" t="n">
         <f aca="false">IFERROR($C9/$B9,0)</f>
-        <v>0.0769230769230769</v>
+        <v>0.0666666666666667</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3559,11 +3703,11 @@
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">SUM(B5:B9)</f>
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="C10" s="9" t="n">
         <f aca="false">SUM(C5:C9)</f>
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="D10" s="9" t="n">
         <f aca="false">SUM(D5:D9)</f>
@@ -3571,7 +3715,7 @@
       </c>
       <c r="E10" s="9" t="n">
         <f aca="false">SUM(E5:E9)</f>
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="F10" s="9" t="n">
         <f aca="false">SUM(F5:F9)</f>
@@ -3579,7 +3723,7 @@
       </c>
       <c r="G10" s="10" t="n">
         <f aca="false">IFERROR($C10/$B10,0)</f>
-        <v>0.716981132075472</v>
+        <v>0.694915254237288</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3616,7 +3760,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G110"/>
+  <dimension ref="A1:G122"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11"/>
@@ -5878,7 +6022,7 @@
         <v>421</v>
       </c>
       <c r="E104" s="20" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F104" s="20" t="s">
         <v>28</v>
@@ -6023,6 +6167,282 @@
       </c>
       <c r="G110" s="16" t="s">
         <v>444</v>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A111" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="B111" s="20" t="s">
+        <v>445</v>
+      </c>
+      <c r="C111" s="16" t="s">
+        <v>446</v>
+      </c>
+      <c r="D111" s="16" t="s">
+        <v>447</v>
+      </c>
+      <c r="E111" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="F111" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="G111" s="16" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="112" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A112" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="B112" s="20" t="s">
+        <v>449</v>
+      </c>
+      <c r="C112" s="16" t="s">
+        <v>450</v>
+      </c>
+      <c r="D112" s="16" t="s">
+        <v>451</v>
+      </c>
+      <c r="E112" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="F112" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="G112" s="16" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="113" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A113" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="B113" s="20" t="s">
+        <v>453</v>
+      </c>
+      <c r="C113" s="16" t="s">
+        <v>454</v>
+      </c>
+      <c r="D113" s="16" t="s">
+        <v>455</v>
+      </c>
+      <c r="E113" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="F113" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="G113" s="16" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="114" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A114" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="B114" s="20" t="s">
+        <v>457</v>
+      </c>
+      <c r="C114" s="16" t="s">
+        <v>458</v>
+      </c>
+      <c r="D114" s="16" t="s">
+        <v>459</v>
+      </c>
+      <c r="E114" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="F114" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="G114" s="16" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="115" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A115" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="B115" s="20" t="s">
+        <v>461</v>
+      </c>
+      <c r="C115" s="16" t="s">
+        <v>462</v>
+      </c>
+      <c r="D115" s="16" t="s">
+        <v>463</v>
+      </c>
+      <c r="E115" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="F115" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="G115" s="16" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="116" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A116" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="B116" s="20" t="s">
+        <v>465</v>
+      </c>
+      <c r="C116" s="16" t="s">
+        <v>466</v>
+      </c>
+      <c r="D116" s="16" t="s">
+        <v>467</v>
+      </c>
+      <c r="E116" s="20" t="s">
+        <v>4</v>
+      </c>
+      <c r="F116" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="G116" s="16" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="117" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A117" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="B117" s="20" t="s">
+        <v>469</v>
+      </c>
+      <c r="C117" s="16" t="s">
+        <v>470</v>
+      </c>
+      <c r="D117" s="16" t="s">
+        <v>471</v>
+      </c>
+      <c r="E117" s="20" t="s">
+        <v>4</v>
+      </c>
+      <c r="F117" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="G117" s="16" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="118" customFormat="false" ht="113.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A118" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="B118" s="20" t="s">
+        <v>473</v>
+      </c>
+      <c r="C118" s="16" t="s">
+        <v>474</v>
+      </c>
+      <c r="D118" s="16" t="s">
+        <v>475</v>
+      </c>
+      <c r="E118" s="20" t="s">
+        <v>4</v>
+      </c>
+      <c r="F118" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="G118" s="16" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="119" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A119" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="B119" s="20" t="s">
+        <v>477</v>
+      </c>
+      <c r="C119" s="16" t="s">
+        <v>478</v>
+      </c>
+      <c r="D119" s="16" t="s">
+        <v>479</v>
+      </c>
+      <c r="E119" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="F119" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="G119" s="16" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="120" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="B120" s="20" t="s">
+        <v>481</v>
+      </c>
+      <c r="C120" s="16" t="s">
+        <v>482</v>
+      </c>
+      <c r="D120" s="16" t="s">
+        <v>483</v>
+      </c>
+      <c r="E120" s="20" t="s">
+        <v>4</v>
+      </c>
+      <c r="F120" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="G120" s="16" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="121" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A121" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="B121" s="20" t="s">
+        <v>485</v>
+      </c>
+      <c r="C121" s="16" t="s">
+        <v>486</v>
+      </c>
+      <c r="D121" s="16" t="s">
+        <v>487</v>
+      </c>
+      <c r="E121" s="20" t="s">
+        <v>4</v>
+      </c>
+      <c r="F121" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="G121" s="16" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="122" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A122" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="B122" s="20" t="s">
+        <v>489</v>
+      </c>
+      <c r="C122" s="16" t="s">
+        <v>490</v>
+      </c>
+      <c r="D122" s="16" t="s">
+        <v>491</v>
+      </c>
+      <c r="E122" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="F122" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="G122" s="16" t="s">
+        <v>492</v>
       </c>
     </row>
   </sheetData>
@@ -6074,7 +6494,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>445</v>
+        <v>493</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6085,13 +6505,13 @@
         <v>20</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>446</v>
+        <v>494</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>447</v>
+        <v>495</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>448</v>
+        <v>496</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>22</v>
@@ -6102,2112 +6522,2112 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>449</v>
+        <v>497</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>25</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>450</v>
+        <v>498</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>451</v>
+        <v>499</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>452</v>
+        <v>500</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G4" s="16" t="s">
-        <v>454</v>
+        <v>502</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>455</v>
+        <v>503</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>25</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>456</v>
+        <v>504</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>457</v>
+        <v>505</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>452</v>
+        <v>500</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G5" s="16"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>458</v>
+        <v>506</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>25</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>459</v>
+        <v>507</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>460</v>
+        <v>508</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>461</v>
+        <v>509</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G6" s="16"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>462</v>
+        <v>510</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>25</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>459</v>
+        <v>507</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>463</v>
+        <v>511</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>465</v>
+        <v>513</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>466</v>
+        <v>514</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>25</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>467</v>
+        <v>515</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>468</v>
+        <v>516</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G8" s="16"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>469</v>
+        <v>517</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>30</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>470</v>
+        <v>518</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>471</v>
+        <v>519</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>452</v>
+        <v>500</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>472</v>
+        <v>520</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>473</v>
+        <v>521</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>30</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>474</v>
+        <v>522</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>475</v>
+        <v>523</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>452</v>
+        <v>500</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>476</v>
+        <v>524</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>477</v>
+        <v>525</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>30</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>450</v>
+        <v>498</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>478</v>
+        <v>526</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>452</v>
+        <v>500</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>479</v>
+        <v>527</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>480</v>
+        <v>528</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>30</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>481</v>
+        <v>529</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>482</v>
+        <v>530</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>483</v>
+        <v>531</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>484</v>
+        <v>532</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>30</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>485</v>
+        <v>533</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>486</v>
+        <v>534</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>487</v>
+        <v>535</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>488</v>
+        <v>536</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>30</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>489</v>
+        <v>537</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>490</v>
+        <v>538</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>491</v>
+        <v>539</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>492</v>
+        <v>540</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>493</v>
+        <v>541</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>494</v>
+        <v>542</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>495</v>
+        <v>543</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>496</v>
+        <v>544</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>497</v>
+        <v>545</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>34</v>
       </c>
       <c r="C16" s="16" t="s">
-        <v>498</v>
+        <v>546</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>499</v>
+        <v>547</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>452</v>
+        <v>500</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>500</v>
+        <v>548</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>501</v>
+        <v>549</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>47</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>502</v>
+        <v>550</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>503</v>
+        <v>551</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>452</v>
+        <v>500</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G17" s="16" t="s">
-        <v>504</v>
+        <v>552</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>505</v>
+        <v>553</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>52</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>506</v>
+        <v>554</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>507</v>
+        <v>555</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>461</v>
+        <v>509</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>508</v>
+        <v>556</v>
       </c>
       <c r="G18" s="16" t="s">
-        <v>509</v>
+        <v>557</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>510</v>
+        <v>558</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>493</v>
+        <v>541</v>
       </c>
       <c r="C19" s="16" t="s">
-        <v>511</v>
+        <v>559</v>
       </c>
       <c r="D19" s="16" t="s">
-        <v>512</v>
+        <v>560</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>461</v>
+        <v>509</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G19" s="16" t="s">
-        <v>513</v>
+        <v>561</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>514</v>
+        <v>562</v>
       </c>
       <c r="B20" s="6" t="s">
         <v>30</v>
       </c>
       <c r="C20" s="16" t="s">
-        <v>515</v>
+        <v>563</v>
       </c>
       <c r="D20" s="16" t="s">
-        <v>516</v>
+        <v>564</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>461</v>
+        <v>509</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G20" s="16" t="s">
-        <v>517</v>
+        <v>565</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>518</v>
+        <v>566</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>493</v>
+        <v>541</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>515</v>
+        <v>563</v>
       </c>
       <c r="D21" s="16" t="s">
-        <v>519</v>
+        <v>567</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G21" s="16" t="s">
-        <v>520</v>
+        <v>568</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>521</v>
+        <v>569</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>493</v>
+        <v>541</v>
       </c>
       <c r="C22" s="16" t="s">
-        <v>522</v>
+        <v>570</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>523</v>
+        <v>571</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G22" s="16" t="s">
-        <v>524</v>
+        <v>572</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>525</v>
+        <v>573</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>493</v>
+        <v>541</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>526</v>
+        <v>574</v>
       </c>
       <c r="D23" s="16" t="s">
-        <v>527</v>
+        <v>575</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>461</v>
+        <v>509</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G23" s="16" t="s">
-        <v>528</v>
+        <v>576</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>529</v>
+        <v>577</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>493</v>
+        <v>541</v>
       </c>
       <c r="C24" s="16" t="s">
-        <v>530</v>
+        <v>578</v>
       </c>
       <c r="D24" s="16" t="s">
-        <v>531</v>
+        <v>579</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>452</v>
+        <v>500</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G24" s="16" t="s">
-        <v>532</v>
+        <v>580</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>533</v>
+        <v>581</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>493</v>
+        <v>541</v>
       </c>
       <c r="C25" s="16" t="s">
-        <v>534</v>
+        <v>582</v>
       </c>
       <c r="D25" s="16" t="s">
-        <v>535</v>
+        <v>583</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G25" s="16" t="s">
-        <v>536</v>
+        <v>584</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>537</v>
+        <v>585</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>493</v>
+        <v>541</v>
       </c>
       <c r="C26" s="16" t="s">
-        <v>538</v>
+        <v>586</v>
       </c>
       <c r="D26" s="16" t="s">
-        <v>539</v>
+        <v>587</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>461</v>
+        <v>509</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G26" s="16" t="s">
-        <v>540</v>
+        <v>588</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
+        <v>589</v>
+      </c>
+      <c r="B27" s="6" t="s">
         <v>541</v>
       </c>
-      <c r="B27" s="6" t="s">
-        <v>493</v>
-      </c>
       <c r="C27" s="16" t="s">
-        <v>542</v>
+        <v>590</v>
       </c>
       <c r="D27" s="16" t="s">
-        <v>543</v>
+        <v>591</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>452</v>
+        <v>500</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G27" s="16" t="s">
-        <v>544</v>
+        <v>592</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>545</v>
+        <v>593</v>
       </c>
       <c r="B28" s="6" t="s">
         <v>39</v>
       </c>
       <c r="C28" s="16" t="s">
-        <v>456</v>
+        <v>504</v>
       </c>
       <c r="D28" s="16" t="s">
-        <v>546</v>
+        <v>594</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>452</v>
+        <v>500</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G28" s="16" t="s">
-        <v>547</v>
+        <v>595</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>548</v>
+        <v>596</v>
       </c>
       <c r="B29" s="6" t="s">
         <v>43</v>
       </c>
       <c r="C29" s="16" t="s">
-        <v>459</v>
+        <v>507</v>
       </c>
       <c r="D29" s="16" t="s">
-        <v>549</v>
+        <v>597</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G29" s="16" t="s">
-        <v>550</v>
+        <v>598</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>551</v>
+        <v>599</v>
       </c>
       <c r="B30" s="6" t="s">
         <v>43</v>
       </c>
       <c r="C30" s="16" t="s">
-        <v>470</v>
+        <v>518</v>
       </c>
       <c r="D30" s="16" t="s">
-        <v>552</v>
+        <v>600</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G30" s="16" t="s">
-        <v>553</v>
+        <v>601</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>554</v>
+        <v>602</v>
       </c>
       <c r="B31" s="6" t="s">
         <v>47</v>
       </c>
       <c r="C31" s="16" t="s">
-        <v>555</v>
+        <v>603</v>
       </c>
       <c r="D31" s="16" t="s">
-        <v>556</v>
+        <v>604</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>452</v>
+        <v>500</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G31" s="16" t="s">
-        <v>557</v>
+        <v>605</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>558</v>
+        <v>606</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>559</v>
+        <v>607</v>
       </c>
       <c r="C32" s="16" t="s">
-        <v>515</v>
+        <v>563</v>
       </c>
       <c r="D32" s="16" t="s">
-        <v>560</v>
+        <v>608</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>452</v>
+        <v>500</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G32" s="16" t="s">
-        <v>561</v>
+        <v>609</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="s">
-        <v>562</v>
+        <v>610</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>559</v>
+        <v>607</v>
       </c>
       <c r="C33" s="16" t="s">
-        <v>563</v>
+        <v>611</v>
       </c>
       <c r="D33" s="16" t="s">
-        <v>564</v>
+        <v>612</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>452</v>
+        <v>500</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G33" s="16" t="s">
-        <v>565</v>
+        <v>613</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="s">
-        <v>566</v>
+        <v>614</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>493</v>
+        <v>541</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>567</v>
+        <v>615</v>
       </c>
       <c r="D34" s="16" t="s">
-        <v>568</v>
+        <v>616</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>461</v>
+        <v>509</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>569</v>
+        <v>617</v>
       </c>
       <c r="G34" s="16" t="s">
-        <v>570</v>
+        <v>618</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="6" t="s">
-        <v>571</v>
+        <v>619</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>493</v>
+        <v>541</v>
       </c>
       <c r="C35" s="16" t="s">
-        <v>572</v>
+        <v>620</v>
       </c>
       <c r="D35" s="16" t="s">
-        <v>573</v>
+        <v>621</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>461</v>
+        <v>509</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>569</v>
+        <v>617</v>
       </c>
       <c r="G35" s="16" t="s">
-        <v>574</v>
+        <v>622</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="s">
-        <v>575</v>
+        <v>623</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>493</v>
+        <v>541</v>
       </c>
       <c r="C36" s="16" t="s">
-        <v>572</v>
+        <v>620</v>
       </c>
       <c r="D36" s="16" t="s">
-        <v>576</v>
+        <v>624</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>461</v>
+        <v>509</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G36" s="16" t="s">
-        <v>577</v>
+        <v>625</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="20" t="s">
-        <v>578</v>
+        <v>626</v>
       </c>
       <c r="B37" s="20" t="s">
         <v>56</v>
       </c>
       <c r="C37" s="20" t="s">
-        <v>579</v>
+        <v>627</v>
       </c>
       <c r="D37" s="16" t="s">
-        <v>580</v>
+        <v>628</v>
       </c>
       <c r="E37" s="20" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F37" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G37" s="16" t="s">
-        <v>581</v>
+        <v>629</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="20" t="s">
-        <v>582</v>
+        <v>630</v>
       </c>
       <c r="B38" s="20" t="s">
-        <v>583</v>
+        <v>631</v>
       </c>
       <c r="C38" s="20" t="s">
-        <v>584</v>
+        <v>632</v>
       </c>
       <c r="D38" s="16" t="s">
-        <v>585</v>
+        <v>633</v>
       </c>
       <c r="E38" s="20" t="s">
-        <v>461</v>
+        <v>509</v>
       </c>
       <c r="F38" s="20" t="s">
-        <v>569</v>
+        <v>617</v>
       </c>
       <c r="G38" s="16" t="s">
-        <v>586</v>
+        <v>634</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="20" t="s">
-        <v>587</v>
+        <v>635</v>
       </c>
       <c r="B39" s="20" t="s">
         <v>52</v>
       </c>
       <c r="C39" s="20" t="s">
-        <v>467</v>
+        <v>515</v>
       </c>
       <c r="D39" s="16" t="s">
-        <v>588</v>
+        <v>636</v>
       </c>
       <c r="E39" s="20" t="s">
-        <v>452</v>
+        <v>500</v>
       </c>
       <c r="F39" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G39" s="16" t="s">
-        <v>589</v>
+        <v>637</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="20" t="s">
-        <v>590</v>
+        <v>638</v>
       </c>
       <c r="B40" s="20" t="s">
-        <v>521</v>
+        <v>569</v>
       </c>
       <c r="C40" s="20" t="s">
-        <v>591</v>
+        <v>639</v>
       </c>
       <c r="D40" s="16" t="s">
-        <v>592</v>
+        <v>640</v>
       </c>
       <c r="E40" s="20" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F40" s="20" t="s">
-        <v>569</v>
+        <v>617</v>
       </c>
       <c r="G40" s="16" t="s">
-        <v>593</v>
+        <v>641</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="20" t="s">
-        <v>594</v>
+        <v>642</v>
       </c>
       <c r="B41" s="20" t="s">
         <v>76</v>
       </c>
       <c r="C41" s="20" t="s">
-        <v>595</v>
+        <v>643</v>
       </c>
       <c r="D41" s="16" t="s">
-        <v>596</v>
+        <v>644</v>
       </c>
       <c r="E41" s="20" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F41" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G41" s="16" t="s">
-        <v>597</v>
+        <v>645</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="20" t="s">
-        <v>598</v>
+        <v>646</v>
       </c>
       <c r="B42" s="20" t="s">
         <v>76</v>
       </c>
       <c r="C42" s="20" t="s">
-        <v>599</v>
+        <v>647</v>
       </c>
       <c r="D42" s="16" t="s">
-        <v>600</v>
+        <v>648</v>
       </c>
       <c r="E42" s="20" t="s">
-        <v>461</v>
+        <v>509</v>
       </c>
       <c r="F42" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G42" s="16" t="s">
-        <v>601</v>
+        <v>649</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="20" t="s">
-        <v>602</v>
+        <v>650</v>
       </c>
       <c r="B43" s="20" t="s">
         <v>84</v>
       </c>
       <c r="C43" s="20" t="s">
-        <v>603</v>
+        <v>651</v>
       </c>
       <c r="D43" s="16" t="s">
-        <v>604</v>
+        <v>652</v>
       </c>
       <c r="E43" s="20" t="s">
-        <v>461</v>
+        <v>509</v>
       </c>
       <c r="F43" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G43" s="16" t="s">
-        <v>605</v>
+        <v>653</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="20" t="s">
-        <v>606</v>
+        <v>654</v>
       </c>
       <c r="B44" s="20" t="s">
         <v>76</v>
       </c>
       <c r="C44" s="20" t="s">
-        <v>607</v>
+        <v>655</v>
       </c>
       <c r="D44" s="16" t="s">
-        <v>608</v>
+        <v>656</v>
       </c>
       <c r="E44" s="20" t="s">
-        <v>461</v>
+        <v>509</v>
       </c>
       <c r="F44" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G44" s="16" t="s">
-        <v>609</v>
+        <v>657</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="20" t="s">
-        <v>610</v>
+        <v>658</v>
       </c>
       <c r="B45" s="20" t="s">
         <v>183</v>
       </c>
       <c r="C45" s="20" t="s">
-        <v>611</v>
+        <v>659</v>
       </c>
       <c r="D45" s="16" t="s">
-        <v>612</v>
+        <v>660</v>
       </c>
       <c r="E45" s="20" t="s">
-        <v>452</v>
+        <v>500</v>
       </c>
       <c r="F45" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G45" s="16" t="s">
-        <v>613</v>
+        <v>661</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="20" t="s">
-        <v>614</v>
+        <v>662</v>
       </c>
       <c r="B46" s="20" t="s">
         <v>80</v>
       </c>
       <c r="C46" s="20" t="s">
-        <v>615</v>
+        <v>663</v>
       </c>
       <c r="D46" s="16" t="s">
-        <v>616</v>
+        <v>664</v>
       </c>
       <c r="E46" s="20" t="s">
-        <v>452</v>
+        <v>500</v>
       </c>
       <c r="F46" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G46" s="16" t="s">
-        <v>617</v>
+        <v>665</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="20" t="s">
-        <v>618</v>
+        <v>666</v>
       </c>
       <c r="B47" s="20" t="s">
         <v>183</v>
       </c>
       <c r="C47" s="20" t="s">
-        <v>619</v>
+        <v>667</v>
       </c>
       <c r="D47" s="16" t="s">
-        <v>620</v>
+        <v>668</v>
       </c>
       <c r="E47" s="20" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F47" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G47" s="16" t="s">
-        <v>621</v>
+        <v>669</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="20" t="s">
-        <v>622</v>
+        <v>670</v>
       </c>
       <c r="B48" s="20" t="s">
         <v>183</v>
       </c>
       <c r="C48" s="20" t="s">
-        <v>515</v>
+        <v>563</v>
       </c>
       <c r="D48" s="16" t="s">
-        <v>623</v>
+        <v>671</v>
       </c>
       <c r="E48" s="20" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F48" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G48" s="16" t="s">
-        <v>624</v>
+        <v>672</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="20" t="s">
-        <v>625</v>
+        <v>673</v>
       </c>
       <c r="B49" s="20" t="s">
         <v>207</v>
       </c>
       <c r="C49" s="20" t="s">
-        <v>626</v>
+        <v>674</v>
       </c>
       <c r="D49" s="16" t="s">
-        <v>627</v>
+        <v>675</v>
       </c>
       <c r="E49" s="20" t="s">
-        <v>461</v>
+        <v>509</v>
       </c>
       <c r="F49" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G49" s="16" t="s">
-        <v>628</v>
+        <v>676</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="20" t="s">
-        <v>629</v>
+        <v>677</v>
       </c>
       <c r="B50" s="20" t="s">
         <v>231</v>
       </c>
       <c r="C50" s="20" t="s">
-        <v>630</v>
+        <v>678</v>
       </c>
       <c r="D50" s="16" t="s">
-        <v>631</v>
+        <v>679</v>
       </c>
       <c r="E50" s="20" t="s">
-        <v>452</v>
+        <v>500</v>
       </c>
       <c r="F50" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G50" s="16" t="s">
-        <v>632</v>
+        <v>680</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="20" t="s">
-        <v>633</v>
+        <v>681</v>
       </c>
       <c r="B51" s="20" t="s">
         <v>231</v>
       </c>
       <c r="C51" s="20" t="s">
-        <v>634</v>
+        <v>682</v>
       </c>
       <c r="D51" s="16" t="s">
-        <v>635</v>
+        <v>683</v>
       </c>
       <c r="E51" s="20" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F51" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G51" s="16" t="s">
-        <v>636</v>
+        <v>684</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="20" t="s">
-        <v>637</v>
+        <v>685</v>
       </c>
       <c r="B52" s="20" t="s">
         <v>231</v>
       </c>
       <c r="C52" s="20" t="s">
-        <v>603</v>
+        <v>651</v>
       </c>
       <c r="D52" s="16" t="s">
-        <v>638</v>
+        <v>686</v>
       </c>
       <c r="E52" s="20" t="s">
-        <v>461</v>
+        <v>509</v>
       </c>
       <c r="F52" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G52" s="16" t="s">
-        <v>639</v>
+        <v>687</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="20" t="s">
-        <v>640</v>
+        <v>688</v>
       </c>
       <c r="B53" s="20" t="s">
         <v>231</v>
       </c>
       <c r="C53" s="20" t="s">
-        <v>641</v>
+        <v>689</v>
       </c>
       <c r="D53" s="16" t="s">
-        <v>642</v>
+        <v>690</v>
       </c>
       <c r="E53" s="20" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F53" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G53" s="16" t="s">
-        <v>643</v>
+        <v>691</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="20" t="s">
-        <v>644</v>
+        <v>692</v>
       </c>
       <c r="B54" s="20" t="s">
         <v>231</v>
       </c>
       <c r="C54" s="20" t="s">
-        <v>645</v>
+        <v>693</v>
       </c>
       <c r="D54" s="16" t="s">
-        <v>646</v>
+        <v>694</v>
       </c>
       <c r="E54" s="20" t="s">
-        <v>452</v>
+        <v>500</v>
       </c>
       <c r="F54" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G54" s="16" t="s">
-        <v>647</v>
+        <v>695</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="20" t="s">
-        <v>648</v>
+        <v>696</v>
       </c>
       <c r="B55" s="20" t="s">
         <v>231</v>
       </c>
       <c r="C55" s="20" t="s">
-        <v>649</v>
+        <v>697</v>
       </c>
       <c r="D55" s="16" t="s">
-        <v>650</v>
+        <v>698</v>
       </c>
       <c r="E55" s="20" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F55" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G55" s="16" t="s">
-        <v>651</v>
+        <v>699</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="20" t="s">
-        <v>652</v>
+        <v>700</v>
       </c>
       <c r="B56" s="20" t="s">
         <v>231</v>
       </c>
       <c r="C56" s="20" t="s">
-        <v>641</v>
+        <v>689</v>
       </c>
       <c r="D56" s="16" t="s">
-        <v>653</v>
+        <v>701</v>
       </c>
       <c r="E56" s="20" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F56" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G56" s="16" t="s">
-        <v>654</v>
+        <v>702</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="20" t="s">
-        <v>655</v>
+        <v>703</v>
       </c>
       <c r="B57" s="20" t="s">
         <v>231</v>
       </c>
       <c r="C57" s="20" t="s">
-        <v>656</v>
+        <v>704</v>
       </c>
       <c r="D57" s="16" t="s">
-        <v>657</v>
+        <v>705</v>
       </c>
       <c r="E57" s="20" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F57" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G57" s="16" t="s">
-        <v>658</v>
+        <v>706</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="20" t="s">
-        <v>659</v>
+        <v>707</v>
       </c>
       <c r="B58" s="20" t="s">
         <v>231</v>
       </c>
       <c r="C58" s="20" t="s">
-        <v>660</v>
+        <v>708</v>
       </c>
       <c r="D58" s="16" t="s">
-        <v>661</v>
+        <v>709</v>
       </c>
       <c r="E58" s="20" t="s">
-        <v>452</v>
+        <v>500</v>
       </c>
       <c r="F58" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G58" s="16" t="s">
-        <v>662</v>
+        <v>710</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="20" t="s">
-        <v>663</v>
+        <v>711</v>
       </c>
       <c r="B59" s="20" t="s">
         <v>231</v>
       </c>
       <c r="C59" s="20" t="s">
-        <v>664</v>
+        <v>712</v>
       </c>
       <c r="D59" s="16" t="s">
-        <v>665</v>
+        <v>713</v>
       </c>
       <c r="E59" s="20" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F59" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G59" s="16" t="s">
-        <v>666</v>
+        <v>714</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="20" t="s">
-        <v>667</v>
+        <v>715</v>
       </c>
       <c r="B60" s="20" t="s">
         <v>231</v>
       </c>
       <c r="C60" s="20" t="s">
-        <v>668</v>
+        <v>716</v>
       </c>
       <c r="D60" s="16" t="s">
-        <v>669</v>
+        <v>717</v>
       </c>
       <c r="E60" s="20" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F60" s="20" t="s">
-        <v>508</v>
+        <v>556</v>
       </c>
       <c r="G60" s="16" t="s">
-        <v>670</v>
+        <v>718</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="20" t="s">
-        <v>671</v>
+        <v>719</v>
       </c>
       <c r="B61" s="20" t="s">
         <v>231</v>
       </c>
       <c r="C61" s="20" t="s">
-        <v>672</v>
+        <v>720</v>
       </c>
       <c r="D61" s="16" t="s">
-        <v>673</v>
+        <v>721</v>
       </c>
       <c r="E61" s="20" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F61" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G61" s="16" t="s">
-        <v>674</v>
+        <v>722</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="20" t="s">
-        <v>675</v>
+        <v>723</v>
       </c>
       <c r="B62" s="20" t="s">
         <v>255</v>
       </c>
       <c r="C62" s="20" t="s">
-        <v>676</v>
+        <v>724</v>
       </c>
       <c r="D62" s="16" t="s">
-        <v>677</v>
+        <v>725</v>
       </c>
       <c r="E62" s="20" t="s">
-        <v>452</v>
+        <v>500</v>
       </c>
       <c r="F62" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G62" s="16" t="s">
-        <v>678</v>
+        <v>726</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="20" t="s">
-        <v>679</v>
+        <v>727</v>
       </c>
       <c r="B63" s="20" t="s">
         <v>267</v>
       </c>
       <c r="C63" s="20" t="s">
-        <v>680</v>
+        <v>728</v>
       </c>
       <c r="D63" s="16" t="s">
-        <v>681</v>
+        <v>729</v>
       </c>
       <c r="E63" s="20" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F63" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G63" s="16" t="s">
-        <v>682</v>
+        <v>730</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="20" t="s">
-        <v>683</v>
+        <v>731</v>
       </c>
       <c r="B64" s="20" t="s">
         <v>275</v>
       </c>
       <c r="C64" s="20" t="s">
-        <v>684</v>
+        <v>732</v>
       </c>
       <c r="D64" s="16" t="s">
-        <v>685</v>
+        <v>733</v>
       </c>
       <c r="E64" s="20" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F64" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G64" s="16" t="s">
-        <v>686</v>
+        <v>734</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="20" t="s">
-        <v>687</v>
+        <v>735</v>
       </c>
       <c r="B65" s="20" t="s">
         <v>263</v>
       </c>
       <c r="C65" s="20" t="s">
-        <v>555</v>
+        <v>603</v>
       </c>
       <c r="D65" s="16" t="s">
-        <v>688</v>
+        <v>736</v>
       </c>
       <c r="E65" s="20" t="s">
-        <v>461</v>
+        <v>509</v>
       </c>
       <c r="F65" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G65" s="16" t="s">
-        <v>689</v>
+        <v>737</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="20" t="s">
-        <v>690</v>
+        <v>738</v>
       </c>
       <c r="B66" s="20" t="s">
         <v>275</v>
       </c>
       <c r="C66" s="20" t="s">
-        <v>691</v>
+        <v>739</v>
       </c>
       <c r="D66" s="16" t="s">
-        <v>692</v>
+        <v>740</v>
       </c>
       <c r="E66" s="20" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F66" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G66" s="16" t="s">
-        <v>693</v>
+        <v>741</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="20" t="s">
-        <v>694</v>
+        <v>742</v>
       </c>
       <c r="B67" s="20" t="s">
         <v>271</v>
       </c>
       <c r="C67" s="20" t="s">
-        <v>695</v>
+        <v>743</v>
       </c>
       <c r="D67" s="16" t="s">
-        <v>696</v>
+        <v>744</v>
       </c>
       <c r="E67" s="20" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F67" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G67" s="16" t="s">
-        <v>697</v>
+        <v>745</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="20" t="s">
-        <v>698</v>
+        <v>746</v>
       </c>
       <c r="B68" s="20" t="s">
         <v>307</v>
       </c>
       <c r="C68" s="20" t="s">
-        <v>699</v>
+        <v>747</v>
       </c>
       <c r="D68" s="16" t="s">
-        <v>700</v>
+        <v>748</v>
       </c>
       <c r="E68" s="20" t="s">
-        <v>452</v>
+        <v>500</v>
       </c>
       <c r="F68" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G68" s="16" t="s">
-        <v>701</v>
+        <v>749</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="20" t="s">
-        <v>702</v>
+        <v>750</v>
       </c>
       <c r="B69" s="20" t="s">
         <v>307</v>
       </c>
       <c r="C69" s="20" t="s">
-        <v>703</v>
+        <v>751</v>
       </c>
       <c r="D69" s="16" t="s">
-        <v>704</v>
+        <v>752</v>
       </c>
       <c r="E69" s="20" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F69" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G69" s="16" t="s">
-        <v>705</v>
+        <v>753</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="20" t="s">
-        <v>706</v>
+        <v>754</v>
       </c>
       <c r="B70" s="20" t="s">
         <v>307</v>
       </c>
       <c r="C70" s="20" t="s">
-        <v>707</v>
+        <v>755</v>
       </c>
       <c r="D70" s="16" t="s">
-        <v>708</v>
+        <v>756</v>
       </c>
       <c r="E70" s="20" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F70" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G70" s="16" t="s">
-        <v>709</v>
+        <v>757</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="20" t="s">
-        <v>710</v>
+        <v>758</v>
       </c>
       <c r="B71" s="20" t="s">
         <v>263</v>
       </c>
       <c r="C71" s="20" t="s">
-        <v>711</v>
+        <v>759</v>
       </c>
       <c r="D71" s="16" t="s">
-        <v>712</v>
+        <v>760</v>
       </c>
       <c r="E71" s="20" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F71" s="20" t="s">
-        <v>508</v>
+        <v>556</v>
       </c>
       <c r="G71" s="16" t="s">
-        <v>713</v>
+        <v>761</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="20" t="s">
-        <v>714</v>
+        <v>762</v>
       </c>
       <c r="B72" s="20" t="s">
-        <v>715</v>
+        <v>763</v>
       </c>
       <c r="C72" s="20" t="s">
-        <v>716</v>
+        <v>764</v>
       </c>
       <c r="D72" s="16" t="s">
-        <v>717</v>
+        <v>765</v>
       </c>
       <c r="E72" s="20" t="s">
-        <v>452</v>
+        <v>500</v>
       </c>
       <c r="F72" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G72" s="16" t="s">
-        <v>718</v>
+        <v>766</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="20" t="s">
-        <v>719</v>
+        <v>767</v>
       </c>
       <c r="B73" s="20" t="s">
-        <v>715</v>
+        <v>763</v>
       </c>
       <c r="C73" s="20" t="s">
-        <v>720</v>
+        <v>768</v>
       </c>
       <c r="D73" s="16" t="s">
-        <v>721</v>
+        <v>769</v>
       </c>
       <c r="E73" s="20" t="s">
-        <v>452</v>
+        <v>500</v>
       </c>
       <c r="F73" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G73" s="16" t="s">
-        <v>722</v>
+        <v>770</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="20" t="s">
-        <v>723</v>
+        <v>771</v>
       </c>
       <c r="B74" s="20" t="s">
-        <v>715</v>
+        <v>763</v>
       </c>
       <c r="C74" s="20" t="s">
-        <v>660</v>
+        <v>708</v>
       </c>
       <c r="D74" s="16" t="s">
-        <v>724</v>
+        <v>772</v>
       </c>
       <c r="E74" s="20" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F74" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G74" s="16" t="s">
-        <v>725</v>
+        <v>773</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="20" t="s">
-        <v>726</v>
+        <v>774</v>
       </c>
       <c r="B75" s="20" t="s">
         <v>351</v>
       </c>
       <c r="C75" s="20" t="s">
-        <v>727</v>
+        <v>775</v>
       </c>
       <c r="D75" s="16" t="s">
-        <v>728</v>
+        <v>776</v>
       </c>
       <c r="E75" s="20" t="s">
-        <v>452</v>
+        <v>500</v>
       </c>
       <c r="F75" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G75" s="16" t="s">
-        <v>729</v>
+        <v>777</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="20" t="s">
-        <v>730</v>
+        <v>778</v>
       </c>
       <c r="B76" s="20" t="s">
         <v>351</v>
       </c>
       <c r="C76" s="20" t="s">
-        <v>731</v>
+        <v>779</v>
       </c>
       <c r="D76" s="16" t="s">
-        <v>732</v>
+        <v>780</v>
       </c>
       <c r="E76" s="20" t="s">
-        <v>452</v>
+        <v>500</v>
       </c>
       <c r="F76" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G76" s="16" t="s">
-        <v>733</v>
+        <v>781</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="20" t="s">
-        <v>734</v>
+        <v>782</v>
       </c>
       <c r="B77" s="20" t="s">
         <v>351</v>
       </c>
       <c r="C77" s="20" t="s">
-        <v>735</v>
+        <v>783</v>
       </c>
       <c r="D77" s="16" t="s">
-        <v>736</v>
+        <v>784</v>
       </c>
       <c r="E77" s="20" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F77" s="20" t="s">
-        <v>569</v>
+        <v>617</v>
       </c>
       <c r="G77" s="16" t="s">
-        <v>737</v>
+        <v>785</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="20" t="s">
-        <v>738</v>
+        <v>786</v>
       </c>
       <c r="B78" s="20" t="s">
-        <v>739</v>
+        <v>787</v>
       </c>
       <c r="C78" s="20" t="s">
-        <v>740</v>
+        <v>788</v>
       </c>
       <c r="D78" s="16" t="s">
-        <v>741</v>
+        <v>789</v>
       </c>
       <c r="E78" s="20" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F78" s="20" t="s">
-        <v>569</v>
+        <v>617</v>
       </c>
       <c r="G78" s="16" t="s">
-        <v>742</v>
+        <v>790</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="20" t="s">
-        <v>743</v>
+        <v>791</v>
       </c>
       <c r="B79" s="20" t="s">
-        <v>739</v>
+        <v>787</v>
       </c>
       <c r="C79" s="20" t="s">
-        <v>744</v>
+        <v>792</v>
       </c>
       <c r="D79" s="16" t="s">
-        <v>745</v>
+        <v>793</v>
       </c>
       <c r="E79" s="20" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F79" s="20" t="s">
-        <v>569</v>
+        <v>617</v>
       </c>
       <c r="G79" s="16" t="s">
-        <v>746</v>
+        <v>794</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="20" t="s">
-        <v>747</v>
+        <v>795</v>
       </c>
       <c r="B80" s="20" t="s">
         <v>379</v>
       </c>
       <c r="C80" s="20" t="s">
-        <v>748</v>
+        <v>796</v>
       </c>
       <c r="D80" s="16" t="s">
-        <v>749</v>
+        <v>797</v>
       </c>
       <c r="E80" s="20" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F80" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G80" s="16" t="s">
-        <v>750</v>
+        <v>798</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="20" t="s">
-        <v>751</v>
+        <v>799</v>
       </c>
       <c r="B81" s="20" t="s">
         <v>371</v>
       </c>
       <c r="C81" s="20" t="s">
-        <v>752</v>
+        <v>800</v>
       </c>
       <c r="D81" s="16" t="s">
-        <v>753</v>
+        <v>801</v>
       </c>
       <c r="E81" s="20" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F81" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G81" s="16" t="s">
-        <v>754</v>
+        <v>802</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="20" t="s">
-        <v>755</v>
+        <v>803</v>
       </c>
       <c r="B82" s="20" t="s">
         <v>367</v>
       </c>
       <c r="C82" s="20" t="s">
-        <v>756</v>
+        <v>804</v>
       </c>
       <c r="D82" s="16" t="s">
-        <v>757</v>
+        <v>805</v>
       </c>
       <c r="E82" s="20" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F82" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G82" s="16" t="s">
-        <v>758</v>
+        <v>806</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="20" t="s">
-        <v>759</v>
+        <v>807</v>
       </c>
       <c r="B83" s="20" t="s">
         <v>367</v>
       </c>
       <c r="C83" s="20" t="s">
-        <v>760</v>
+        <v>808</v>
       </c>
       <c r="D83" s="16" t="s">
-        <v>761</v>
+        <v>809</v>
       </c>
       <c r="E83" s="20" t="s">
-        <v>461</v>
+        <v>509</v>
       </c>
       <c r="F83" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G83" s="16" t="s">
-        <v>762</v>
+        <v>810</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="20" t="s">
-        <v>763</v>
+        <v>811</v>
       </c>
       <c r="B84" s="20" t="s">
         <v>351</v>
       </c>
       <c r="C84" s="20" t="s">
-        <v>764</v>
+        <v>812</v>
       </c>
       <c r="D84" s="16" t="s">
-        <v>765</v>
+        <v>813</v>
       </c>
       <c r="E84" s="20" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F84" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G84" s="16" t="s">
-        <v>766</v>
+        <v>814</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="20" t="s">
-        <v>767</v>
+        <v>815</v>
       </c>
       <c r="B85" s="20" t="s">
         <v>323</v>
       </c>
       <c r="C85" s="20" t="s">
-        <v>768</v>
+        <v>816</v>
       </c>
       <c r="D85" s="16" t="s">
-        <v>769</v>
+        <v>817</v>
       </c>
       <c r="E85" s="20" t="s">
-        <v>452</v>
+        <v>500</v>
       </c>
       <c r="F85" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G85" s="16" t="s">
-        <v>770</v>
+        <v>818</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="20" t="s">
-        <v>771</v>
+        <v>819</v>
       </c>
       <c r="B86" s="20" t="s">
         <v>323</v>
       </c>
       <c r="C86" s="20" t="s">
-        <v>772</v>
+        <v>820</v>
       </c>
       <c r="D86" s="16" t="s">
-        <v>773</v>
+        <v>821</v>
       </c>
       <c r="E86" s="20" t="s">
-        <v>461</v>
+        <v>509</v>
       </c>
       <c r="F86" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G86" s="16" t="s">
-        <v>774</v>
+        <v>822</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="20" t="s">
-        <v>775</v>
+        <v>823</v>
       </c>
       <c r="B87" s="20" t="s">
         <v>375</v>
       </c>
       <c r="C87" s="20" t="s">
-        <v>776</v>
+        <v>824</v>
       </c>
       <c r="D87" s="16" t="s">
-        <v>777</v>
+        <v>825</v>
       </c>
       <c r="E87" s="20" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F87" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G87" s="16" t="s">
-        <v>778</v>
+        <v>826</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="20" t="s">
-        <v>779</v>
+        <v>827</v>
       </c>
       <c r="B88" s="20" t="s">
         <v>379</v>
       </c>
       <c r="C88" s="20" t="s">
-        <v>780</v>
+        <v>828</v>
       </c>
       <c r="D88" s="16" t="s">
-        <v>781</v>
+        <v>829</v>
       </c>
       <c r="E88" s="20" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F88" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G88" s="16" t="s">
-        <v>782</v>
+        <v>830</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="20" t="s">
-        <v>783</v>
+        <v>831</v>
       </c>
       <c r="B89" s="20" t="s">
         <v>331</v>
       </c>
       <c r="C89" s="20" t="s">
-        <v>784</v>
+        <v>832</v>
       </c>
       <c r="D89" s="16" t="s">
-        <v>785</v>
+        <v>833</v>
       </c>
       <c r="E89" s="20" t="s">
-        <v>461</v>
+        <v>509</v>
       </c>
       <c r="F89" s="20" t="s">
-        <v>569</v>
+        <v>617</v>
       </c>
       <c r="G89" s="16" t="s">
-        <v>786</v>
+        <v>834</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="20" t="s">
-        <v>787</v>
+        <v>835</v>
       </c>
       <c r="B90" s="20" t="s">
         <v>279</v>
       </c>
       <c r="C90" s="20" t="s">
-        <v>788</v>
+        <v>836</v>
       </c>
       <c r="D90" s="16" t="s">
-        <v>789</v>
+        <v>837</v>
       </c>
       <c r="E90" s="20" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F90" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G90" s="16" t="s">
-        <v>790</v>
+        <v>838</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="20" t="s">
-        <v>791</v>
+        <v>839</v>
       </c>
       <c r="B91" s="20" t="s">
         <v>279</v>
       </c>
       <c r="C91" s="20" t="s">
-        <v>788</v>
+        <v>836</v>
       </c>
       <c r="D91" s="16" t="s">
-        <v>792</v>
+        <v>840</v>
       </c>
       <c r="E91" s="20" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F91" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G91" s="16" t="s">
-        <v>793</v>
+        <v>841</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="20" t="s">
-        <v>794</v>
+        <v>842</v>
       </c>
       <c r="B92" s="20" t="s">
         <v>291</v>
       </c>
       <c r="C92" s="20" t="s">
-        <v>795</v>
+        <v>843</v>
       </c>
       <c r="D92" s="16" t="s">
-        <v>796</v>
+        <v>844</v>
       </c>
       <c r="E92" s="20" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F92" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G92" s="16" t="s">
-        <v>797</v>
+        <v>845</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="20" t="s">
-        <v>798</v>
+        <v>846</v>
       </c>
       <c r="B93" s="20" t="s">
         <v>299</v>
       </c>
       <c r="C93" s="20" t="s">
-        <v>799</v>
+        <v>847</v>
       </c>
       <c r="D93" s="16" t="s">
-        <v>800</v>
+        <v>848</v>
       </c>
       <c r="E93" s="20" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F93" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G93" s="16" t="s">
-        <v>801</v>
+        <v>849</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="157.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="20" t="s">
-        <v>802</v>
+        <v>850</v>
       </c>
       <c r="B94" s="20" t="s">
         <v>291</v>
       </c>
       <c r="C94" s="20" t="s">
-        <v>803</v>
+        <v>851</v>
       </c>
       <c r="D94" s="16" t="s">
-        <v>804</v>
+        <v>852</v>
       </c>
       <c r="E94" s="20" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F94" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G94" s="16" t="s">
-        <v>805</v>
+        <v>853</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A95" s="20" t="s">
-        <v>806</v>
+        <v>854</v>
       </c>
       <c r="B95" s="20" t="s">
         <v>371</v>
       </c>
       <c r="C95" s="20" t="s">
-        <v>807</v>
+        <v>855</v>
       </c>
       <c r="D95" s="16" t="s">
-        <v>808</v>
+        <v>856</v>
       </c>
       <c r="E95" s="20" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="F95" s="20" t="s">
-        <v>453</v>
+        <v>501</v>
       </c>
       <c r="G95" s="16" t="s">
-        <v>809</v>
+        <v>857</v>
       </c>
     </row>
   </sheetData>
@@ -8260,12 +8680,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>810</v>
+        <v>858</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>811</v>
+        <v>859</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8273,16 +8693,16 @@
         <v>19</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>812</v>
+        <v>860</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>813</v>
+        <v>861</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>814</v>
+        <v>862</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>815</v>
+        <v>863</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>22</v>
@@ -8290,382 +8710,382 @@
     </row>
     <row r="5" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>816</v>
+        <v>864</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>817</v>
+        <v>865</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>818</v>
+        <v>866</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>819</v>
+        <v>867</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>820</v>
+        <v>868</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>569</v>
+        <v>617</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>821</v>
+        <v>869</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>822</v>
+        <v>870</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>823</v>
+        <v>871</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>824</v>
+        <v>872</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>825</v>
+        <v>873</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>826</v>
+        <v>874</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>827</v>
+        <v>875</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>828</v>
+        <v>876</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>829</v>
+        <v>877</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>830</v>
+        <v>878</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>831</v>
+        <v>879</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>508</v>
+        <v>556</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>832</v>
+        <v>880</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>833</v>
+        <v>881</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>834</v>
+        <v>882</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>835</v>
+        <v>883</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>836</v>
+        <v>884</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>508</v>
+        <v>556</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>837</v>
+        <v>885</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>838</v>
+        <v>886</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>839</v>
+        <v>887</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>840</v>
+        <v>888</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>841</v>
+        <v>889</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>569</v>
+        <v>617</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>842</v>
+        <v>890</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>838</v>
+        <v>886</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>843</v>
+        <v>891</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>844</v>
+        <v>892</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>845</v>
+        <v>893</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>569</v>
+        <v>617</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>846</v>
+        <v>894</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>847</v>
+        <v>895</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>848</v>
+        <v>896</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>849</v>
+        <v>897</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>850</v>
+        <v>898</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>826</v>
+        <v>874</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>851</v>
+        <v>899</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>852</v>
+        <v>900</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>853</v>
+        <v>901</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>854</v>
+        <v>902</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>855</v>
+        <v>903</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>569</v>
+        <v>617</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="s">
-        <v>856</v>
+        <v>904</v>
       </c>
       <c r="B13" s="20" t="s">
-        <v>847</v>
+        <v>895</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>857</v>
+        <v>905</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>858</v>
+        <v>906</v>
       </c>
       <c r="E13" s="20" t="s">
-        <v>859</v>
+        <v>907</v>
       </c>
       <c r="F13" s="20" t="s">
-        <v>569</v>
+        <v>617</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
-        <v>860</v>
+        <v>908</v>
       </c>
       <c r="B14" s="20" t="s">
-        <v>852</v>
+        <v>900</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>861</v>
+        <v>909</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>862</v>
+        <v>910</v>
       </c>
       <c r="E14" s="20" t="s">
-        <v>863</v>
+        <v>911</v>
       </c>
       <c r="F14" s="20" t="s">
-        <v>569</v>
+        <v>617</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="20" t="s">
-        <v>864</v>
+        <v>912</v>
       </c>
       <c r="B15" s="20" t="s">
-        <v>865</v>
+        <v>913</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>866</v>
+        <v>914</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>867</v>
+        <v>915</v>
       </c>
       <c r="E15" s="20" t="s">
-        <v>868</v>
+        <v>916</v>
       </c>
       <c r="F15" s="20" t="s">
-        <v>569</v>
+        <v>617</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="20" t="s">
-        <v>869</v>
+        <v>917</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>817</v>
+        <v>865</v>
       </c>
       <c r="C16" s="16" t="s">
-        <v>870</v>
+        <v>918</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>871</v>
+        <v>919</v>
       </c>
       <c r="E16" s="20" t="s">
-        <v>872</v>
+        <v>920</v>
       </c>
       <c r="F16" s="20" t="s">
-        <v>569</v>
+        <v>617</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="20" t="s">
-        <v>873</v>
+        <v>921</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>838</v>
+        <v>886</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>874</v>
+        <v>922</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>875</v>
+        <v>923</v>
       </c>
       <c r="E17" s="20" t="s">
-        <v>876</v>
+        <v>924</v>
       </c>
       <c r="F17" s="20" t="s">
-        <v>569</v>
+        <v>617</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="20" t="s">
-        <v>877</v>
+        <v>925</v>
       </c>
       <c r="B18" s="20" t="s">
-        <v>847</v>
+        <v>895</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>878</v>
+        <v>926</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>879</v>
+        <v>927</v>
       </c>
       <c r="E18" s="20" t="s">
-        <v>880</v>
+        <v>928</v>
       </c>
       <c r="F18" s="20" t="s">
-        <v>569</v>
+        <v>617</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="20" t="s">
-        <v>881</v>
+        <v>929</v>
       </c>
       <c r="B19" s="20" t="s">
-        <v>882</v>
+        <v>930</v>
       </c>
       <c r="C19" s="16" t="s">
-        <v>883</v>
+        <v>931</v>
       </c>
       <c r="D19" s="16" t="s">
-        <v>884</v>
+        <v>932</v>
       </c>
       <c r="E19" s="20" t="s">
-        <v>885</v>
+        <v>933</v>
       </c>
       <c r="F19" s="20" t="s">
-        <v>569</v>
+        <v>617</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="20" t="s">
-        <v>886</v>
+        <v>934</v>
       </c>
       <c r="B20" s="20" t="s">
-        <v>887</v>
+        <v>935</v>
       </c>
       <c r="C20" s="16" t="s">
-        <v>888</v>
+        <v>936</v>
       </c>
       <c r="D20" s="16" t="s">
-        <v>889</v>
+        <v>937</v>
       </c>
       <c r="E20" s="20" t="s">
-        <v>890</v>
+        <v>938</v>
       </c>
       <c r="F20" s="20" t="s">
-        <v>826</v>
+        <v>874</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="20" t="s">
-        <v>891</v>
+        <v>939</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>892</v>
+        <v>940</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>893</v>
+        <v>941</v>
       </c>
       <c r="D21" s="16" t="s">
-        <v>894</v>
+        <v>942</v>
       </c>
       <c r="E21" s="20" t="s">
-        <v>895</v>
+        <v>943</v>
       </c>
       <c r="F21" s="20" t="s">
-        <v>508</v>
+        <v>556</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="20" t="s">
-        <v>896</v>
+        <v>944</v>
       </c>
       <c r="B22" s="20" t="s">
-        <v>897</v>
+        <v>945</v>
       </c>
       <c r="C22" s="16" t="s">
-        <v>898</v>
+        <v>946</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>899</v>
+        <v>947</v>
       </c>
       <c r="E22" s="20" t="s">
-        <v>900</v>
+        <v>948</v>
       </c>
       <c r="F22" s="20" t="s">
-        <v>569</v>
+        <v>617</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="20" t="s">
-        <v>901</v>
+        <v>949</v>
       </c>
       <c r="B23" s="20" t="s">
-        <v>902</v>
+        <v>950</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>903</v>
+        <v>951</v>
       </c>
       <c r="D23" s="16" t="s">
-        <v>904</v>
+        <v>952</v>
       </c>
       <c r="E23" s="20" t="s">
-        <v>905</v>
+        <v>953</v>
       </c>
       <c r="F23" s="20" t="s">
-        <v>569</v>
+        <v>617</v>
       </c>
     </row>
   </sheetData>

</xml_diff>